<commit_message>
Bind V3.1.1 artifacts to release source
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R8608aeade3ac429f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R7e58dc54edc44d53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Ra67eb87f2dcf4fc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R69783272255348c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="Re77d3fdaeb234cda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Rd88a8734ee5a4c18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R4ee08f05ec404b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R25cde8a934384465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rc0a91b9b177f4e29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R8cdf3854b2ec452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R8e5b0b0e79ac48ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Reae36a8cd6144619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rd9f49ea763014f13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R11caee2a4d2c4ad0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R173c6b8851a54166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R81d0782ae1194435"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Rc658f84655974244"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R780ab728fc5741f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,88 +18,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={4E1AE514-D801-4652-03C7-9C017258FA7F}</x:author>
-    <x:author>tc={7AF82130-B0E4-209A-4618-1E50825A54D3}</x:author>
-    <x:author>tc={BD247F29-1779-BD7B-3A76-2F9CA2B1AEA9}</x:author>
-    <x:author>tc={8590D4C8-7BB2-B37F-ACBC-5CA173521159}</x:author>
-    <x:author>tc={6A216E8E-92DF-AFFE-18E5-1ADFA3F82056}</x:author>
-    <x:author>tc={9E1F9529-F6B7-697E-B0FD-B1D4C6227B7A}</x:author>
-    <x:author>tc={F089E3CB-60B3-03AC-8E7F-93C9E42FD894}</x:author>
-    <x:author>tc={12B1A270-E94D-50AD-DA4E-7A1FDAC30DCB}</x:author>
-    <x:author>tc={F82771A3-A99A-0510-B8AC-7E29E6FBE5B1}</x:author>
-    <x:author>tc={DECC8597-377C-34CD-E2B3-03E4CDE64DFF}</x:author>
-    <x:author>tc={A3F9A96A-539F-D063-AEBF-141AFA0AEA2C}</x:author>
-    <x:author>tc={F77443F4-B61F-3FED-1AC7-E110785A7261}</x:author>
-    <x:author>tc={1C6A08E6-783A-C52C-B877-668C4C7E5003}</x:author>
-    <x:author>tc={0F981EA1-CC3D-603E-597F-65F2467C1919}</x:author>
-    <x:author>tc={ABDACCC2-BC8D-D7BC-E624-89AFBED9A48A}</x:author>
-    <x:author>tc={77511AD6-56CE-9400-F619-68EA4585C300}</x:author>
-    <x:author>tc={AE25BDD5-A88A-96AE-1536-194D620DACC9}</x:author>
-    <x:author>tc={7E91EDEA-AE21-2A10-7796-101B5EB303ED}</x:author>
-    <x:author>tc={AB37BBD1-EAC2-1806-05D1-3E40151E0FB3}</x:author>
-    <x:author>tc={2033EF05-7942-CEF2-D58F-D6A916653FF1}</x:author>
-    <x:author>tc={12C0A1BD-809D-FC6E-3D30-5FCDE04C97C5}</x:author>
-    <x:author>tc={70578AA2-42B1-6F34-4F79-10A8377EC411}</x:author>
-    <x:author>tc={930D6326-AE26-A3E2-41D4-DB2F1315FE3F}</x:author>
-    <x:author>tc={77C52D62-9ABD-CEEC-8BEC-6DED4F1AD77E}</x:author>
-    <x:author>tc={42A245CA-6701-571C-656F-ED22619AE455}</x:author>
-    <x:author>tc={09D2F53C-2FB5-DF17-E66B-64A20096B902}</x:author>
-    <x:author>tc={0B4B9E10-CD50-7AE8-9351-443FC7976775}</x:author>
-    <x:author>tc={EF0AABF9-7514-8518-3F4D-89EBB487598C}</x:author>
-    <x:author>tc={BAB5CD16-8499-7562-748B-81FED2199AD3}</x:author>
-    <x:author>tc={A0FE3388-188D-CDE5-F93F-B9C0A24C4B8A}</x:author>
-    <x:author>tc={F0A4E1AD-BA57-0436-18A2-DC817E7CF4B0}</x:author>
-    <x:author>tc={A018C91F-E498-493B-7893-3D0D4A4140CB}</x:author>
-    <x:author>tc={88E48B16-E609-1658-B572-C8C7649727B7}</x:author>
-    <x:author>tc={BC0DB942-644A-E26D-1052-6EE3E6387EBE}</x:author>
-    <x:author>tc={7C04529D-D62F-DE14-50C7-42103ED0CF71}</x:author>
-    <x:author>tc={FFF220B9-C2F5-88A5-2D98-BDC2655B4F6C}</x:author>
-    <x:author>tc={256B1B8E-6075-057C-D0E8-D8074868B2CE}</x:author>
-    <x:author>tc={177C9E8F-A7F5-67B6-0E7B-9A56137E74E7}</x:author>
-    <x:author>tc={5BD3FACD-18BC-5907-BF86-DC29E80F69AD}</x:author>
-    <x:author>tc={A937D63B-EECD-4806-A5A4-B6BA4D87459D}</x:author>
-    <x:author>tc={01DC81F7-B232-E08C-2E3A-2B0A088D3DCB}</x:author>
-    <x:author>tc={F7DC8988-FE5D-D931-343B-E7DFF94ADC6D}</x:author>
-    <x:author>tc={9F99EA2B-8A6B-9D13-B687-5A5DCFD90EBA}</x:author>
-    <x:author>tc={B4D8B064-2F4B-C72D-486F-85A729D78211}</x:author>
-    <x:author>tc={2F1C4DC6-216A-45E8-4A6A-FA97A15D4209}</x:author>
-    <x:author>tc={8A18C50E-DC3C-5532-B5A0-D7D3206EE588}</x:author>
-    <x:author>tc={E1436310-3D0A-5ED3-B7FD-B71C6EEA744D}</x:author>
-    <x:author>tc={AEBA1112-D7A2-7717-56A7-55183A0B4F02}</x:author>
-    <x:author>tc={FFC501B4-2A76-5FFF-FEE3-DAB31E1BDF6B}</x:author>
-    <x:author>tc={F8735732-5181-02E5-6876-FC558AC48877}</x:author>
-    <x:author>tc={68661F0E-1601-8C19-9F72-7D34300F621A}</x:author>
-    <x:author>tc={45555C8B-D3E4-89DC-EA2E-36F835CCD69A}</x:author>
-    <x:author>tc={A1E0D2CA-9465-1500-C09F-4F7F8F228816}</x:author>
-    <x:author>tc={378234E5-9A13-E7B2-22B6-26FC3D1A3EAB}</x:author>
-    <x:author>tc={62A4D9DF-4950-0BF6-1F7F-88EB0C5BA434}</x:author>
-    <x:author>tc={CE4B8C1A-B7B4-76C7-DF0F-399A81A6457D}</x:author>
-    <x:author>tc={B6437DAD-9558-F897-75A1-647BB4BCF355}</x:author>
-    <x:author>tc={45038E8A-BBA7-AC80-70AF-84A160231648}</x:author>
-    <x:author>tc={08A775BA-068E-89DB-8707-C0CF68DC6ACE}</x:author>
-    <x:author>tc={69D9BA54-EA91-B23E-3CE9-CE75E4E2CBE5}</x:author>
-    <x:author>tc={2F4EFF2A-6F9A-D919-A3C7-181F749AB2D9}</x:author>
-    <x:author>tc={34940E54-7873-D99C-3270-5FD1306E91D2}</x:author>
-    <x:author>tc={45CC6F17-DD16-810C-C9F4-CF68C28FF2F0}</x:author>
-    <x:author>tc={2A5316C3-E913-21D0-A456-7037D496237C}</x:author>
-    <x:author>tc={F1A61732-1316-7EC7-1342-68EF4BDB990A}</x:author>
-    <x:author>tc={C71237D2-00AD-8BDD-11BA-B2BC6B1EF5A4}</x:author>
-    <x:author>tc={DD145447-1B37-50EF-AD97-B0B7D9706660}</x:author>
-    <x:author>tc={9AB79405-3889-D910-89FF-04A657405ACF}</x:author>
-    <x:author>tc={75A0A0AF-5DF2-8170-0772-7DF4E8B37829}</x:author>
-    <x:author>tc={82B78876-7388-0695-52D1-4E4432F6E93D}</x:author>
-    <x:author>tc={68D67B86-D278-871C-44A8-846D953CEFB9}</x:author>
-    <x:author>tc={F5F688FF-BCB0-A284-DEB9-9D0BB1057AE9}</x:author>
-    <x:author>tc={0E492FED-F462-8D12-38CB-22CA7E3F9193}</x:author>
-    <x:author>tc={266B374E-62C8-E8E0-3DA1-497290CB09E5}</x:author>
-    <x:author>tc={A3575B29-6FB7-B0C7-39C7-2334956167F0}</x:author>
-    <x:author>tc={F59D604D-70C1-1F32-D0B5-95664CAD0CE1}</x:author>
-    <x:author>tc={0D3A7C23-7E4C-ACC7-E1E3-864F55C876EA}</x:author>
-    <x:author>tc={8081BED2-29B8-83FE-B585-D5ACB424124F}</x:author>
-    <x:author>tc={115C4C2E-AF99-B4D5-AE18-1EBF6DFE5F1C}</x:author>
-    <x:author>tc={F28617DD-7C10-92B5-2F6D-718086383385}</x:author>
-    <x:author>tc={398B97E6-1155-3F6C-AEDA-B66764E4EEB6}</x:author>
-    <x:author>tc={71A0D50F-D1A8-87A5-E39B-C454EBC526C3}</x:author>
+    <x:author>tc={75551666-5AE4-C06F-F275-345195AD9824}</x:author>
+    <x:author>tc={564C1C2A-9CE5-EA61-5DCD-F4FE8503953B}</x:author>
+    <x:author>tc={6B84FBAC-76BC-060D-35F0-ACDFC46FEED9}</x:author>
+    <x:author>tc={E272EB50-439D-B2DD-2DF1-EA75847E6ED8}</x:author>
+    <x:author>tc={2BDBC44B-72B0-BE02-1CD3-59028DB471DB}</x:author>
+    <x:author>tc={77D96203-6107-53E4-2A0C-3E2E98D4FAD4}</x:author>
+    <x:author>tc={78A9ED23-6B0D-B401-C5DC-831E23F15C31}</x:author>
+    <x:author>tc={ACA3EDE8-684B-1099-8486-C7FF1B13DB7E}</x:author>
+    <x:author>tc={055DB408-E0EA-A2F3-06F1-2255F199A597}</x:author>
+    <x:author>tc={9DD9D7DF-B5C6-4A72-5620-8D579DC7A395}</x:author>
+    <x:author>tc={38743DC3-BEC9-B6B3-EE19-C2A7150C7E5F}</x:author>
+    <x:author>tc={1681E5A1-644C-4F49-E9F5-473EDC3106DD}</x:author>
+    <x:author>tc={08A165E7-1078-8440-2818-F2ED3F3298F4}</x:author>
+    <x:author>tc={67841105-8DD3-58EA-6E86-0E1D75050B48}</x:author>
+    <x:author>tc={6838EBFF-AD44-1E4D-1CE6-64B69E9D00B6}</x:author>
+    <x:author>tc={423C179F-5F8C-3495-39C3-5A3C8A6AF2BE}</x:author>
+    <x:author>tc={3615ABDC-CE76-6317-52F6-295F96996482}</x:author>
+    <x:author>tc={03A863CC-C443-36F1-88DD-197230A3C218}</x:author>
+    <x:author>tc={BA1F7F5A-69CF-2A50-4D76-136DBEEF91A0}</x:author>
+    <x:author>tc={3856393E-6F1E-8E64-E73F-53BEE2CFD334}</x:author>
+    <x:author>tc={C4E32F58-B171-DA72-C52B-E695171754C0}</x:author>
+    <x:author>tc={3F621C88-4B70-7F61-0136-EB359AA5D0DF}</x:author>
+    <x:author>tc={672D185B-9D4C-9FC6-A4BA-36C418B71A99}</x:author>
+    <x:author>tc={49E31FAE-AC0B-6B9E-42FF-4DF348CB71CA}</x:author>
+    <x:author>tc={B499671D-EDC5-571C-F4EA-699941D0AC08}</x:author>
+    <x:author>tc={7BF3F0D5-2C28-AC82-3B38-3C4997446926}</x:author>
+    <x:author>tc={8067B179-C218-DDEE-402A-47BBD893AAD9}</x:author>
+    <x:author>tc={5DFD983F-0230-623B-F299-D70185218300}</x:author>
+    <x:author>tc={E407B8C4-8D66-09E4-5388-A6BED433D14F}</x:author>
+    <x:author>tc={68AD1868-B5AA-7CB0-0686-6B067C5C217E}</x:author>
+    <x:author>tc={D4BD99D9-46A9-3F6B-37CD-620F0123098E}</x:author>
+    <x:author>tc={4832AFE5-5336-0617-B446-43C1D1044874}</x:author>
+    <x:author>tc={1175AC3C-7D1F-23C8-74BB-CDA1B793F3A7}</x:author>
+    <x:author>tc={2D6229C6-77F1-0DB7-E1EC-418843C35F53}</x:author>
+    <x:author>tc={A2565DB1-37B7-3FE6-F0EE-6FA12E6A25D3}</x:author>
+    <x:author>tc={D3EF764D-2D5E-904F-9AB1-3A38E612BA26}</x:author>
+    <x:author>tc={8D7B5EDF-4CFB-DBBB-FA2D-C9B68C40C153}</x:author>
+    <x:author>tc={D587F045-A020-A06B-AB17-12DBCABBD168}</x:author>
+    <x:author>tc={D7DE69B5-A8B1-11B2-C950-F41D8CBD9F15}</x:author>
+    <x:author>tc={BEE2D092-C2E2-3467-8307-A5C89B8B68AE}</x:author>
+    <x:author>tc={44719A85-CEF6-270A-B1DF-36205A4BD2DF}</x:author>
+    <x:author>tc={D220E222-EBCE-94A7-D472-3CDFB73FEC99}</x:author>
+    <x:author>tc={CF3183DE-4FFD-CC85-557B-92B5C2FBBDA4}</x:author>
+    <x:author>tc={7BD1BCA9-983D-4F81-F09B-5256770BD208}</x:author>
+    <x:author>tc={2A1DD6A3-F325-89A6-3642-16C0B71CF7E7}</x:author>
+    <x:author>tc={1B0F2425-537F-8832-6F2B-C5E1367F17F5}</x:author>
+    <x:author>tc={51E6CFE9-07B2-BFE8-8A2D-97D2F6E2D86D}</x:author>
+    <x:author>tc={13064D26-4B82-ABAE-7912-BCB10B5229FC}</x:author>
+    <x:author>tc={2D5ECB66-708D-32B9-396B-2E302301F13A}</x:author>
+    <x:author>tc={AE338A8D-E206-E06B-F8A1-90D3D7F3C769}</x:author>
+    <x:author>tc={30C6CC82-6FCC-FA84-891A-A29620402234}</x:author>
+    <x:author>tc={BBD5CB37-08D4-D4AA-3F59-A8FBDB944903}</x:author>
+    <x:author>tc={668F0A05-5026-1B02-ED6E-D9C966D3E4EC}</x:author>
+    <x:author>tc={B4147D19-C24D-6C5E-BFE9-9844FBEA64A4}</x:author>
+    <x:author>tc={B540F690-35AF-9C2C-E6EF-AB99A19D3CB4}</x:author>
+    <x:author>tc={7CE0EECF-5DF4-B1E6-228F-4CDBAA7E88DF}</x:author>
+    <x:author>tc={4A35FCBF-8F2C-BA1D-568D-1D8DD20B97D3}</x:author>
+    <x:author>tc={A882E23F-032E-FA6E-B4A2-12C63FF54E0C}</x:author>
+    <x:author>tc={4142D1C2-7A4B-B9FA-2C32-810525F47331}</x:author>
+    <x:author>tc={E13BB1CE-65C2-66DC-EE1F-C6C3D55667C6}</x:author>
+    <x:author>tc={A91352D0-D317-15A4-7D71-C2A6585D0F68}</x:author>
+    <x:author>tc={72227493-2DF3-671B-9FA1-275E12824727}</x:author>
+    <x:author>tc={12FCF11E-4671-2735-753D-4D2C8E642B4C}</x:author>
+    <x:author>tc={E3A0655B-7B8D-2B4E-C29C-1690F7526BA5}</x:author>
+    <x:author>tc={95BEE8B6-7DEB-63DC-740F-662516460A29}</x:author>
+    <x:author>tc={C064FFA2-40E3-8C1B-4948-37B03A027824}</x:author>
+    <x:author>tc={65F77BF5-7F3D-8006-4E53-04C8F692A7BC}</x:author>
+    <x:author>tc={13B8E3E6-9F10-4C37-F266-33CBF672A835}</x:author>
+    <x:author>tc={723E4FE8-3707-41C4-4952-BD4B93DA8F34}</x:author>
+    <x:author>tc={94512158-8255-618B-61A4-46E5CB9BF4C3}</x:author>
+    <x:author>tc={57A2F342-59EC-EACD-8B0F-5A6C592ABFF8}</x:author>
+    <x:author>tc={AD130745-00D7-E1FF-EA07-3CC642EA0F28}</x:author>
+    <x:author>tc={EDFB07F6-6133-A276-AF5F-C8288FD3F3EB}</x:author>
+    <x:author>tc={A77E6851-727A-030B-1988-B0388B67B634}</x:author>
+    <x:author>tc={A1D96AFA-2F56-9EA9-D5BE-E6AF517B18E0}</x:author>
+    <x:author>tc={20B59283-4381-3AB4-7593-513964766437}</x:author>
+    <x:author>tc={907378BD-9DAE-40DB-115C-B4F40FAB09FA}</x:author>
+    <x:author>tc={BCB38F7A-3E13-06F4-0C9E-D41451B2A27D}</x:author>
+    <x:author>tc={6F30520B-6B11-7059-994F-29C43B5F8C2B}</x:author>
+    <x:author>tc={3424E448-7943-8047-3807-09928D5E0FC4}</x:author>
+    <x:author>tc={25606D75-0F2B-3440-6C4C-6AEC6AD95783}</x:author>
+    <x:author>tc={CC3668EB-71D5-4F1F-12DE-1FE2F18B5AE3}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1175,26 +1175,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={83E72AB5-7925-FA85-BF71-FAF3D1500196}</x:author>
-    <x:author>tc={E85ACA00-079E-9490-9352-94DF9C7EB52C}</x:author>
-    <x:author>tc={356420CE-D09C-94A4-089E-683B9D741A9B}</x:author>
-    <x:author>tc={6F71C9F1-54AC-76C9-935D-39C484542808}</x:author>
-    <x:author>tc={688CE58B-116A-F83D-8DDA-C91032C8C2CA}</x:author>
-    <x:author>tc={5DB0A32E-BDE8-05FE-90D4-A3A24860714D}</x:author>
-    <x:author>tc={1825B652-FFC8-B945-12E4-BBCAB0818413}</x:author>
-    <x:author>tc={38F94339-320A-B8BF-AB55-688CDFC2BA66}</x:author>
-    <x:author>tc={456A94A7-3147-6099-3E13-E5C7514DC723}</x:author>
-    <x:author>tc={1DEEE897-D256-1700-BF79-EA37E2A44AE3}</x:author>
-    <x:author>tc={C084081A-6A1E-6BAB-52F4-183CE4D7AC04}</x:author>
-    <x:author>tc={47FA69B3-CE50-5399-2C0A-79C51708A827}</x:author>
-    <x:author>tc={F42EE526-63CA-59B8-5B33-1134D8F293E9}</x:author>
-    <x:author>tc={E7BD4014-E12C-C218-CAFB-4355043AF7A1}</x:author>
-    <x:author>tc={ADA962AD-95A0-36BC-24AE-A66D17648317}</x:author>
-    <x:author>tc={CE67D18A-66B1-25B0-1B67-EB6772BC02A8}</x:author>
-    <x:author>tc={5BFF82FC-2EEE-42D1-4BB0-918F503D1992}</x:author>
-    <x:author>tc={57B1331D-63B5-A3A3-CA70-9C7FA11D1CDB}</x:author>
-    <x:author>tc={221AB76F-6B18-5E53-1B73-2B780E4264A9}</x:author>
-    <x:author>tc={D3B471EB-3120-DC1F-E970-8D271E59F6A9}</x:author>
+    <x:author>tc={1838D36A-0B6F-90ED-EEF7-EC269097E000}</x:author>
+    <x:author>tc={25664E63-F7D0-2ED2-1E36-B86F6453DBCB}</x:author>
+    <x:author>tc={80412385-F135-D38A-004D-6F5F6C63C5F6}</x:author>
+    <x:author>tc={9E6EFBC5-ABE1-615A-AF44-25D10AE6E7F4}</x:author>
+    <x:author>tc={C8EDEBC0-9E31-AD81-3E27-7A04D720EE10}</x:author>
+    <x:author>tc={C55543F7-83A1-C507-C151-19B020556FC2}</x:author>
+    <x:author>tc={6B4C6DC8-5E02-8BB5-27C6-E437E820E45B}</x:author>
+    <x:author>tc={7EE12C14-0C36-7979-3EB2-B9DBCADAC67F}</x:author>
+    <x:author>tc={F4CF8361-796D-E1ED-658C-37FD5BE42402}</x:author>
+    <x:author>tc={61E96BB7-8123-81EC-BA03-94C430C99D86}</x:author>
+    <x:author>tc={0BB437E8-B12C-B8A8-B0B0-460BF96CBBE0}</x:author>
+    <x:author>tc={1482B62C-D7DA-F789-CE45-A7B2609F1141}</x:author>
+    <x:author>tc={F7CC6DE2-EB78-E65C-2B11-8FEC33112CF1}</x:author>
+    <x:author>tc={5B619671-60EC-DDB3-6328-C666564CA16E}</x:author>
+    <x:author>tc={E2519075-1BEC-D13A-A7BA-0882E4D90356}</x:author>
+    <x:author>tc={A309184C-D446-A9CA-6A98-DE97B2886C79}</x:author>
+    <x:author>tc={D8DEC458-CF8E-683F-BC94-01B941CFE541}</x:author>
+    <x:author>tc={AD84876E-767D-A96E-6751-D4DFAE7D1131}</x:author>
+    <x:author>tc={1F015695-0961-7C20-4F5D-A510B3E38413}</x:author>
+    <x:author>tc={BF7AB4AB-5D80-B11C-F9A6-264AE0D86812}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2037,7 +2037,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a297fdda8a34c1c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6a7a0c8792ea46ba"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2048,7 +2048,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}"/>
 </xltc:personList>
 </file>
 
@@ -2245,493 +2245,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-12T19:56:47.915" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{4E1AE514-D801-4652-03C7-9C017258FA7F}">
+  <xltc:threadedComment ref="P5" dT="2026-08-12T20:09:22.914" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{75551666-5AE4-C06F-F275-345195AD9824}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-12T19:56:47.92" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{7AF82130-B0E4-209A-4618-1E50825A54D3}">
+  <xltc:threadedComment ref="P6" dT="2026-08-12T20:09:22.916" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{564C1C2A-9CE5-EA61-5DCD-F4FE8503953B}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-12T19:56:47.92" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{BD247F29-1779-BD7B-3A76-2F9CA2B1AEA9}">
+  <xltc:threadedComment ref="P7" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{6B84FBAC-76BC-060D-35F0-ACDFC46FEED9}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-12T19:56:47.92" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{8590D4C8-7BB2-B37F-ACBC-5CA173521159}">
+  <xltc:threadedComment ref="P8" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E272EB50-439D-B2DD-2DF1-EA75847E6ED8}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-12T19:56:47.921" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{6A216E8E-92DF-AFFE-18E5-1ADFA3F82056}">
+  <xltc:threadedComment ref="P9" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{2BDBC44B-72B0-BE02-1CD3-59028DB471DB}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-12T19:56:47.921" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{9E1F9529-F6B7-697E-B0FD-B1D4C6227B7A}">
+  <xltc:threadedComment ref="P10" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{77D96203-6107-53E4-2A0C-3E2E98D4FAD4}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-12T19:56:47.921" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F089E3CB-60B3-03AC-8E7F-93C9E42FD894}">
+  <xltc:threadedComment ref="P11" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{78A9ED23-6B0D-B401-C5DC-831E23F15C31}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-12T19:56:47.921" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{12B1A270-E94D-50AD-DA4E-7A1FDAC30DCB}">
+  <xltc:threadedComment ref="P12" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{ACA3EDE8-684B-1099-8486-C7FF1B13DB7E}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-12T19:56:47.921" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F82771A3-A99A-0510-B8AC-7E29E6FBE5B1}">
+  <xltc:threadedComment ref="P13" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{055DB408-E0EA-A2F3-06F1-2255F199A597}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{DECC8597-377C-34CD-E2B3-03E4CDE64DFF}">
+  <xltc:threadedComment ref="P14" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{9DD9D7DF-B5C6-4A72-5620-8D579DC7A395}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{A3F9A96A-539F-D063-AEBF-141AFA0AEA2C}">
+  <xltc:threadedComment ref="P15" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{38743DC3-BEC9-B6B3-EE19-C2A7150C7E5F}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F77443F4-B61F-3FED-1AC7-E110785A7261}">
+  <xltc:threadedComment ref="P16" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1681E5A1-644C-4F49-E9F5-473EDC3106DD}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{1C6A08E6-783A-C52C-B877-668C4C7E5003}">
+  <xltc:threadedComment ref="P17" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{08A165E7-1078-8440-2818-F2ED3F3298F4}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{0F981EA1-CC3D-603E-597F-65F2467C1919}">
+  <xltc:threadedComment ref="P18" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{67841105-8DD3-58EA-6E86-0E1D75050B48}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{ABDACCC2-BC8D-D7BC-E624-89AFBED9A48A}">
+  <xltc:threadedComment ref="P19" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{6838EBFF-AD44-1E4D-1CE6-64B69E9D00B6}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{77511AD6-56CE-9400-F619-68EA4585C300}">
+  <xltc:threadedComment ref="P20" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{423C179F-5F8C-3495-39C3-5A3C8A6AF2BE}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{AE25BDD5-A88A-96AE-1536-194D620DACC9}">
+  <xltc:threadedComment ref="P21" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{3615ABDC-CE76-6317-52F6-295F96996482}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{7E91EDEA-AE21-2A10-7796-101B5EB303ED}">
+  <xltc:threadedComment ref="P22" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{03A863CC-C443-36F1-88DD-197230A3C218}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{AB37BBD1-EAC2-1806-05D1-3E40151E0FB3}">
+  <xltc:threadedComment ref="P23" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BA1F7F5A-69CF-2A50-4D76-136DBEEF91A0}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{2033EF05-7942-CEF2-D58F-D6A916653FF1}">
+  <xltc:threadedComment ref="P24" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{3856393E-6F1E-8E64-E73F-53BEE2CFD334}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{12C0A1BD-809D-FC6E-3D30-5FCDE04C97C5}">
+  <xltc:threadedComment ref="P25" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{C4E32F58-B171-DA72-C52B-E695171754C0}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{70578AA2-42B1-6F34-4F79-10A8377EC411}">
+  <xltc:threadedComment ref="P26" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{3F621C88-4B70-7F61-0136-EB359AA5D0DF}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{930D6326-AE26-A3E2-41D4-DB2F1315FE3F}">
+  <xltc:threadedComment ref="P27" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{672D185B-9D4C-9FC6-A4BA-36C418B71A99}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{77C52D62-9ABD-CEEC-8BEC-6DED4F1AD77E}">
+  <xltc:threadedComment ref="P28" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{49E31FAE-AC0B-6B9E-42FF-4DF348CB71CA}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{42A245CA-6701-571C-656F-ED22619AE455}">
+  <xltc:threadedComment ref="P29" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{B499671D-EDC5-571C-F4EA-699941D0AC08}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{09D2F53C-2FB5-DF17-E66B-64A20096B902}">
+  <xltc:threadedComment ref="P30" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{7BF3F0D5-2C28-AC82-3B38-3C4997446926}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{0B4B9E10-CD50-7AE8-9351-443FC7976775}">
+  <xltc:threadedComment ref="P31" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{8067B179-C218-DDEE-402A-47BBD893AAD9}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{EF0AABF9-7514-8518-3F4D-89EBB487598C}">
+  <xltc:threadedComment ref="P32" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{5DFD983F-0230-623B-F299-D70185218300}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{BAB5CD16-8499-7562-748B-81FED2199AD3}">
+  <xltc:threadedComment ref="P33" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E407B8C4-8D66-09E4-5388-A6BED433D14F}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{A0FE3388-188D-CDE5-F93F-B9C0A24C4B8A}">
+  <xltc:threadedComment ref="P34" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{68AD1868-B5AA-7CB0-0686-6B067C5C217E}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F0A4E1AD-BA57-0436-18A2-DC817E7CF4B0}">
+  <xltc:threadedComment ref="P35" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D4BD99D9-46A9-3F6B-37CD-620F0123098E}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-12T19:56:47.922" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{A018C91F-E498-493B-7893-3D0D4A4140CB}">
+  <xltc:threadedComment ref="P36" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{4832AFE5-5336-0617-B446-43C1D1044874}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{88E48B16-E609-1658-B572-C8C7649727B7}">
+  <xltc:threadedComment ref="P37" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1175AC3C-7D1F-23C8-74BB-CDA1B793F3A7}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{BC0DB942-644A-E26D-1052-6EE3E6387EBE}">
+  <xltc:threadedComment ref="P38" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{2D6229C6-77F1-0DB7-E1EC-418843C35F53}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{7C04529D-D62F-DE14-50C7-42103ED0CF71}">
+  <xltc:threadedComment ref="P39" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A2565DB1-37B7-3FE6-F0EE-6FA12E6A25D3}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{FFF220B9-C2F5-88A5-2D98-BDC2655B4F6C}">
+  <xltc:threadedComment ref="P40" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D3EF764D-2D5E-904F-9AB1-3A38E612BA26}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{256B1B8E-6075-057C-D0E8-D8074868B2CE}">
+  <xltc:threadedComment ref="P41" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{8D7B5EDF-4CFB-DBBB-FA2D-C9B68C40C153}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{177C9E8F-A7F5-67B6-0E7B-9A56137E74E7}">
+  <xltc:threadedComment ref="P42" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D587F045-A020-A06B-AB17-12DBCABBD168}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{5BD3FACD-18BC-5907-BF86-DC29E80F69AD}">
+  <xltc:threadedComment ref="P43" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D7DE69B5-A8B1-11B2-C950-F41D8CBD9F15}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{A937D63B-EECD-4806-A5A4-B6BA4D87459D}">
+  <xltc:threadedComment ref="P44" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BEE2D092-C2E2-3467-8307-A5C89B8B68AE}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{01DC81F7-B232-E08C-2E3A-2B0A088D3DCB}">
+  <xltc:threadedComment ref="P45" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{44719A85-CEF6-270A-B1DF-36205A4BD2DF}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F7DC8988-FE5D-D931-343B-E7DFF94ADC6D}">
+  <xltc:threadedComment ref="P46" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D220E222-EBCE-94A7-D472-3CDFB73FEC99}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{9F99EA2B-8A6B-9D13-B687-5A5DCFD90EBA}">
+  <xltc:threadedComment ref="P47" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{CF3183DE-4FFD-CC85-557B-92B5C2FBBDA4}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{B4D8B064-2F4B-C72D-486F-85A729D78211}">
+  <xltc:threadedComment ref="P48" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{7BD1BCA9-983D-4F81-F09B-5256770BD208}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{2F1C4DC6-216A-45E8-4A6A-FA97A15D4209}">
+  <xltc:threadedComment ref="P49" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{2A1DD6A3-F325-89A6-3642-16C0B71CF7E7}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{8A18C50E-DC3C-5532-B5A0-D7D3206EE588}">
+  <xltc:threadedComment ref="P50" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1B0F2425-537F-8832-6F2B-C5E1367F17F5}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{E1436310-3D0A-5ED3-B7FD-B71C6EEA744D}">
+  <xltc:threadedComment ref="P51" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{51E6CFE9-07B2-BFE8-8A2D-97D2F6E2D86D}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{AEBA1112-D7A2-7717-56A7-55183A0B4F02}">
+  <xltc:threadedComment ref="P52" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{13064D26-4B82-ABAE-7912-BCB10B5229FC}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{FFC501B4-2A76-5FFF-FEE3-DAB31E1BDF6B}">
+  <xltc:threadedComment ref="P53" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{2D5ECB66-708D-32B9-396B-2E302301F13A}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F8735732-5181-02E5-6876-FC558AC48877}">
+  <xltc:threadedComment ref="P54" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{AE338A8D-E206-E06B-F8A1-90D3D7F3C769}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{68661F0E-1601-8C19-9F72-7D34300F621A}">
+  <xltc:threadedComment ref="P55" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{30C6CC82-6FCC-FA84-891A-A29620402234}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{45555C8B-D3E4-89DC-EA2E-36F835CCD69A}">
+  <xltc:threadedComment ref="P56" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BBD5CB37-08D4-D4AA-3F59-A8FBDB944903}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{A1E0D2CA-9465-1500-C09F-4F7F8F228816}">
+  <xltc:threadedComment ref="P57" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{668F0A05-5026-1B02-ED6E-D9C966D3E4EC}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{378234E5-9A13-E7B2-22B6-26FC3D1A3EAB}">
+  <xltc:threadedComment ref="P58" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{B4147D19-C24D-6C5E-BFE9-9844FBEA64A4}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{62A4D9DF-4950-0BF6-1F7F-88EB0C5BA434}">
+  <xltc:threadedComment ref="P59" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{B540F690-35AF-9C2C-E6EF-AB99A19D3CB4}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{CE4B8C1A-B7B4-76C7-DF0F-399A81A6457D}">
+  <xltc:threadedComment ref="P60" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{7CE0EECF-5DF4-B1E6-228F-4CDBAA7E88DF}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{B6437DAD-9558-F897-75A1-647BB4BCF355}">
+  <xltc:threadedComment ref="P61" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{4A35FCBF-8F2C-BA1D-568D-1D8DD20B97D3}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{45038E8A-BBA7-AC80-70AF-84A160231648}">
+  <xltc:threadedComment ref="P62" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A882E23F-032E-FA6E-B4A2-12C63FF54E0C}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{08A775BA-068E-89DB-8707-C0CF68DC6ACE}">
+  <xltc:threadedComment ref="P63" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{4142D1C2-7A4B-B9FA-2C32-810525F47331}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{69D9BA54-EA91-B23E-3CE9-CE75E4E2CBE5}">
+  <xltc:threadedComment ref="P64" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E13BB1CE-65C2-66DC-EE1F-C6C3D55667C6}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{2F4EFF2A-6F9A-D919-A3C7-181F749AB2D9}">
+  <xltc:threadedComment ref="P65" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A91352D0-D317-15A4-7D71-C2A6585D0F68}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{34940E54-7873-D99C-3270-5FD1306E91D2}">
+  <xltc:threadedComment ref="P66" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{72227493-2DF3-671B-9FA1-275E12824727}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{45CC6F17-DD16-810C-C9F4-CF68C28FF2F0}">
+  <xltc:threadedComment ref="P67" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{12FCF11E-4671-2735-753D-4D2C8E642B4C}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{2A5316C3-E913-21D0-A456-7037D496237C}">
+  <xltc:threadedComment ref="P68" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E3A0655B-7B8D-2B4E-C29C-1690F7526BA5}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-12T19:56:47.923" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F1A61732-1316-7EC7-1342-68EF4BDB990A}">
+  <xltc:threadedComment ref="P69" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{95BEE8B6-7DEB-63DC-740F-662516460A29}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{C71237D2-00AD-8BDD-11BA-B2BC6B1EF5A4}">
+  <xltc:threadedComment ref="P70" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{C064FFA2-40E3-8C1B-4948-37B03A027824}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{DD145447-1B37-50EF-AD97-B0B7D9706660}">
+  <xltc:threadedComment ref="P71" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{65F77BF5-7F3D-8006-4E53-04C8F692A7BC}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{9AB79405-3889-D910-89FF-04A657405ACF}">
+  <xltc:threadedComment ref="P72" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{13B8E3E6-9F10-4C37-F266-33CBF672A835}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{75A0A0AF-5DF2-8170-0772-7DF4E8B37829}">
+  <xltc:threadedComment ref="P73" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{723E4FE8-3707-41C4-4952-BD4B93DA8F34}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{82B78876-7388-0695-52D1-4E4432F6E93D}">
+  <xltc:threadedComment ref="P74" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{94512158-8255-618B-61A4-46E5CB9BF4C3}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{68D67B86-D278-871C-44A8-846D953CEFB9}">
+  <xltc:threadedComment ref="P75" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{57A2F342-59EC-EACD-8B0F-5A6C592ABFF8}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F5F688FF-BCB0-A284-DEB9-9D0BB1057AE9}">
+  <xltc:threadedComment ref="P76" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{AD130745-00D7-E1FF-EA07-3CC642EA0F28}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{0E492FED-F462-8D12-38CB-22CA7E3F9193}">
+  <xltc:threadedComment ref="P77" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{EDFB07F6-6133-A276-AF5F-C8288FD3F3EB}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{266B374E-62C8-E8E0-3DA1-497290CB09E5}">
+  <xltc:threadedComment ref="P78" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A77E6851-727A-030B-1988-B0388B67B634}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{A3575B29-6FB7-B0C7-39C7-2334956167F0}">
+  <xltc:threadedComment ref="P79" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A1D96AFA-2F56-9EA9-D5BE-E6AF517B18E0}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F59D604D-70C1-1F32-D0B5-95664CAD0CE1}">
+  <xltc:threadedComment ref="P80" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{20B59283-4381-3AB4-7593-513964766437}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{0D3A7C23-7E4C-ACC7-E1E3-864F55C876EA}">
+  <xltc:threadedComment ref="P81" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{907378BD-9DAE-40DB-115C-B4F40FAB09FA}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{8081BED2-29B8-83FE-B585-D5ACB424124F}">
+  <xltc:threadedComment ref="P82" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BCB38F7A-3E13-06F4-0C9E-D41451B2A27D}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{115C4C2E-AF99-B4D5-AE18-1EBF6DFE5F1C}">
+  <xltc:threadedComment ref="P83" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{6F30520B-6B11-7059-994F-29C43B5F8C2B}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F28617DD-7C10-92B5-2F6D-718086383385}">
+  <xltc:threadedComment ref="P84" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{3424E448-7943-8047-3807-09928D5E0FC4}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{398B97E6-1155-3F6C-AEDA-B66764E4EEB6}">
+  <xltc:threadedComment ref="P85" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{25606D75-0F2B-3440-6C4C-6AEC6AD95783}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-12T19:56:47.924" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{71A0D50F-D1A8-87A5-E39B-C454EBC526C3}">
+  <xltc:threadedComment ref="P86" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{CC3668EB-71D5-4F1F-12DE-1FE2F18B5AE3}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2742,64 +2742,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-12T19:56:48.316" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{83E72AB5-7925-FA85-BF71-FAF3D1500196}">
+  <xltc:threadedComment ref="J5" dT="2026-08-12T20:09:23.291" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1838D36A-0B6F-90ED-EEF7-EC269097E000}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-12T19:56:48.319" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{E85ACA00-079E-9490-9352-94DF9C7EB52C}">
+  <xltc:threadedComment ref="J6" dT="2026-08-12T20:09:23.294" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{25664E63-F7D0-2ED2-1E36-B86F6453DBCB}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-12T19:56:48.322" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{356420CE-D09C-94A4-089E-683B9D741A9B}">
+  <xltc:threadedComment ref="J7" dT="2026-08-12T20:09:23.296" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{80412385-F135-D38A-004D-6F5F6C63C5F6}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-12T19:56:48.325" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{6F71C9F1-54AC-76C9-935D-39C484542808}">
+  <xltc:threadedComment ref="J8" dT="2026-08-12T20:09:23.299" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{9E6EFBC5-ABE1-615A-AF44-25D10AE6E7F4}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-12T19:56:48.327" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{688CE58B-116A-F83D-8DDA-C91032C8C2CA}">
+  <xltc:threadedComment ref="J9" dT="2026-08-12T20:09:23.302" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{C8EDEBC0-9E31-AD81-3E27-7A04D720EE10}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-12T19:56:48.33" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{5DB0A32E-BDE8-05FE-90D4-A3A24860714D}">
+  <xltc:threadedComment ref="J10" dT="2026-08-12T20:09:23.304" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{C55543F7-83A1-C507-C151-19B020556FC2}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-12T19:56:48.334" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{1825B652-FFC8-B945-12E4-BBCAB0818413}">
+  <xltc:threadedComment ref="J11" dT="2026-08-12T20:09:23.307" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{6B4C6DC8-5E02-8BB5-27C6-E437E820E45B}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-12T19:56:48.336" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{38F94339-320A-B8BF-AB55-688CDFC2BA66}">
+  <xltc:threadedComment ref="J12" dT="2026-08-12T20:09:23.31" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{7EE12C14-0C36-7979-3EB2-B9DBCADAC67F}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-12T19:56:48.338" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{456A94A7-3147-6099-3E13-E5C7514DC723}">
+  <xltc:threadedComment ref="J13" dT="2026-08-12T20:09:23.313" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{F4CF8361-796D-E1ED-658C-37FD5BE42402}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-12T19:56:48.34" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{1DEEE897-D256-1700-BF79-EA37E2A44AE3}">
+  <xltc:threadedComment ref="J14" dT="2026-08-12T20:09:23.316" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{61E96BB7-8123-81EC-BA03-94C430C99D86}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-12T19:56:48.343" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{C084081A-6A1E-6BAB-52F4-183CE4D7AC04}">
+  <xltc:threadedComment ref="J15" dT="2026-08-12T20:09:23.318" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{0BB437E8-B12C-B8A8-B0B0-460BF96CBBE0}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-12T19:56:48.346" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{47FA69B3-CE50-5399-2C0A-79C51708A827}">
+  <xltc:threadedComment ref="J16" dT="2026-08-12T20:09:23.322" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1482B62C-D7DA-F789-CE45-A7B2609F1141}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-12T19:56:48.348" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{F42EE526-63CA-59B8-5B33-1134D8F293E9}">
+  <xltc:threadedComment ref="J17" dT="2026-08-12T20:09:23.324" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{F7CC6DE2-EB78-E65C-2B11-8FEC33112CF1}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-12T19:56:48.35" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{E7BD4014-E12C-C218-CAFB-4355043AF7A1}">
+  <xltc:threadedComment ref="J18" dT="2026-08-12T20:09:23.327" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{5B619671-60EC-DDB3-6328-C666564CA16E}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-12T19:56:48.352" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{ADA962AD-95A0-36BC-24AE-A66D17648317}">
+  <xltc:threadedComment ref="J19" dT="2026-08-12T20:09:23.329" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E2519075-1BEC-D13A-A7BA-0882E4D90356}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-12T19:56:48.354" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{CE67D18A-66B1-25B0-1B67-EB6772BC02A8}">
+  <xltc:threadedComment ref="J20" dT="2026-08-12T20:09:23.331" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A309184C-D446-A9CA-6A98-DE97B2886C79}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-12T19:56:48.359" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{5BFF82FC-2EEE-42D1-4BB0-918F503D1992}">
+  <xltc:threadedComment ref="J21" dT="2026-08-12T20:09:23.333" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D8DEC458-CF8E-683F-BC94-01B941CFE541}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-12T19:56:48.362" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{57B1331D-63B5-A3A3-CA70-9C7FA11D1CDB}">
+  <xltc:threadedComment ref="J22" dT="2026-08-12T20:09:23.337" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{AD84876E-767D-A96E-6751-D4DFAE7D1131}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-12T19:56:48.364" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{221AB76F-6B18-5E53-1B73-2B780E4264A9}">
+  <xltc:threadedComment ref="J23" dT="2026-08-12T20:09:23.34" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1F015695-0961-7C20-4F5D-A510B3E38413}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-12T19:56:48.367" personId="{3D0FDF34-4C91-4852-BC31-8BADFDAD15D7}" id="{D3B471EB-3120-DC1F-E970-8D271E59F6A9}">
+  <xltc:threadedComment ref="J24" dT="2026-08-12T20:09:23.344" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BF7AB4AB-5D80-B11C-F9A6-264AE0D86812}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -7802,7 +7802,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R630e6b069d9945d3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f1a10d85f848f1"/>
 </x:worksheet>
 </file>
 
@@ -8862,7 +8862,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80ae79f344804096"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R813bdb3960b54ec4"/>
 </x:worksheet>
 </file>
 
@@ -20015,6 +20015,6 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0e8b9b3b1e74704"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcead52240fa44262"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Bind canonical V3.1.1 submission release
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R8cdf3854b2ec452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R8e5b0b0e79ac48ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Reae36a8cd6144619"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rd9f49ea763014f13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R11caee2a4d2c4ad0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R173c6b8851a54166"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R81d0782ae1194435"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Rc658f84655974244"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R780ab728fc5741f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rd1ffe793c0054f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R3f65de9dedce4afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rf6fd4f58afdb43af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rd5f0909783b14bfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="Rbcfe6e4453ef4e4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R28243a9317964192"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R5033da0595304c36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R5318b55946a541cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R74b838b5d8c24721"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,88 +18,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={75551666-5AE4-C06F-F275-345195AD9824}</x:author>
-    <x:author>tc={564C1C2A-9CE5-EA61-5DCD-F4FE8503953B}</x:author>
-    <x:author>tc={6B84FBAC-76BC-060D-35F0-ACDFC46FEED9}</x:author>
-    <x:author>tc={E272EB50-439D-B2DD-2DF1-EA75847E6ED8}</x:author>
-    <x:author>tc={2BDBC44B-72B0-BE02-1CD3-59028DB471DB}</x:author>
-    <x:author>tc={77D96203-6107-53E4-2A0C-3E2E98D4FAD4}</x:author>
-    <x:author>tc={78A9ED23-6B0D-B401-C5DC-831E23F15C31}</x:author>
-    <x:author>tc={ACA3EDE8-684B-1099-8486-C7FF1B13DB7E}</x:author>
-    <x:author>tc={055DB408-E0EA-A2F3-06F1-2255F199A597}</x:author>
-    <x:author>tc={9DD9D7DF-B5C6-4A72-5620-8D579DC7A395}</x:author>
-    <x:author>tc={38743DC3-BEC9-B6B3-EE19-C2A7150C7E5F}</x:author>
-    <x:author>tc={1681E5A1-644C-4F49-E9F5-473EDC3106DD}</x:author>
-    <x:author>tc={08A165E7-1078-8440-2818-F2ED3F3298F4}</x:author>
-    <x:author>tc={67841105-8DD3-58EA-6E86-0E1D75050B48}</x:author>
-    <x:author>tc={6838EBFF-AD44-1E4D-1CE6-64B69E9D00B6}</x:author>
-    <x:author>tc={423C179F-5F8C-3495-39C3-5A3C8A6AF2BE}</x:author>
-    <x:author>tc={3615ABDC-CE76-6317-52F6-295F96996482}</x:author>
-    <x:author>tc={03A863CC-C443-36F1-88DD-197230A3C218}</x:author>
-    <x:author>tc={BA1F7F5A-69CF-2A50-4D76-136DBEEF91A0}</x:author>
-    <x:author>tc={3856393E-6F1E-8E64-E73F-53BEE2CFD334}</x:author>
-    <x:author>tc={C4E32F58-B171-DA72-C52B-E695171754C0}</x:author>
-    <x:author>tc={3F621C88-4B70-7F61-0136-EB359AA5D0DF}</x:author>
-    <x:author>tc={672D185B-9D4C-9FC6-A4BA-36C418B71A99}</x:author>
-    <x:author>tc={49E31FAE-AC0B-6B9E-42FF-4DF348CB71CA}</x:author>
-    <x:author>tc={B499671D-EDC5-571C-F4EA-699941D0AC08}</x:author>
-    <x:author>tc={7BF3F0D5-2C28-AC82-3B38-3C4997446926}</x:author>
-    <x:author>tc={8067B179-C218-DDEE-402A-47BBD893AAD9}</x:author>
-    <x:author>tc={5DFD983F-0230-623B-F299-D70185218300}</x:author>
-    <x:author>tc={E407B8C4-8D66-09E4-5388-A6BED433D14F}</x:author>
-    <x:author>tc={68AD1868-B5AA-7CB0-0686-6B067C5C217E}</x:author>
-    <x:author>tc={D4BD99D9-46A9-3F6B-37CD-620F0123098E}</x:author>
-    <x:author>tc={4832AFE5-5336-0617-B446-43C1D1044874}</x:author>
-    <x:author>tc={1175AC3C-7D1F-23C8-74BB-CDA1B793F3A7}</x:author>
-    <x:author>tc={2D6229C6-77F1-0DB7-E1EC-418843C35F53}</x:author>
-    <x:author>tc={A2565DB1-37B7-3FE6-F0EE-6FA12E6A25D3}</x:author>
-    <x:author>tc={D3EF764D-2D5E-904F-9AB1-3A38E612BA26}</x:author>
-    <x:author>tc={8D7B5EDF-4CFB-DBBB-FA2D-C9B68C40C153}</x:author>
-    <x:author>tc={D587F045-A020-A06B-AB17-12DBCABBD168}</x:author>
-    <x:author>tc={D7DE69B5-A8B1-11B2-C950-F41D8CBD9F15}</x:author>
-    <x:author>tc={BEE2D092-C2E2-3467-8307-A5C89B8B68AE}</x:author>
-    <x:author>tc={44719A85-CEF6-270A-B1DF-36205A4BD2DF}</x:author>
-    <x:author>tc={D220E222-EBCE-94A7-D472-3CDFB73FEC99}</x:author>
-    <x:author>tc={CF3183DE-4FFD-CC85-557B-92B5C2FBBDA4}</x:author>
-    <x:author>tc={7BD1BCA9-983D-4F81-F09B-5256770BD208}</x:author>
-    <x:author>tc={2A1DD6A3-F325-89A6-3642-16C0B71CF7E7}</x:author>
-    <x:author>tc={1B0F2425-537F-8832-6F2B-C5E1367F17F5}</x:author>
-    <x:author>tc={51E6CFE9-07B2-BFE8-8A2D-97D2F6E2D86D}</x:author>
-    <x:author>tc={13064D26-4B82-ABAE-7912-BCB10B5229FC}</x:author>
-    <x:author>tc={2D5ECB66-708D-32B9-396B-2E302301F13A}</x:author>
-    <x:author>tc={AE338A8D-E206-E06B-F8A1-90D3D7F3C769}</x:author>
-    <x:author>tc={30C6CC82-6FCC-FA84-891A-A29620402234}</x:author>
-    <x:author>tc={BBD5CB37-08D4-D4AA-3F59-A8FBDB944903}</x:author>
-    <x:author>tc={668F0A05-5026-1B02-ED6E-D9C966D3E4EC}</x:author>
-    <x:author>tc={B4147D19-C24D-6C5E-BFE9-9844FBEA64A4}</x:author>
-    <x:author>tc={B540F690-35AF-9C2C-E6EF-AB99A19D3CB4}</x:author>
-    <x:author>tc={7CE0EECF-5DF4-B1E6-228F-4CDBAA7E88DF}</x:author>
-    <x:author>tc={4A35FCBF-8F2C-BA1D-568D-1D8DD20B97D3}</x:author>
-    <x:author>tc={A882E23F-032E-FA6E-B4A2-12C63FF54E0C}</x:author>
-    <x:author>tc={4142D1C2-7A4B-B9FA-2C32-810525F47331}</x:author>
-    <x:author>tc={E13BB1CE-65C2-66DC-EE1F-C6C3D55667C6}</x:author>
-    <x:author>tc={A91352D0-D317-15A4-7D71-C2A6585D0F68}</x:author>
-    <x:author>tc={72227493-2DF3-671B-9FA1-275E12824727}</x:author>
-    <x:author>tc={12FCF11E-4671-2735-753D-4D2C8E642B4C}</x:author>
-    <x:author>tc={E3A0655B-7B8D-2B4E-C29C-1690F7526BA5}</x:author>
-    <x:author>tc={95BEE8B6-7DEB-63DC-740F-662516460A29}</x:author>
-    <x:author>tc={C064FFA2-40E3-8C1B-4948-37B03A027824}</x:author>
-    <x:author>tc={65F77BF5-7F3D-8006-4E53-04C8F692A7BC}</x:author>
-    <x:author>tc={13B8E3E6-9F10-4C37-F266-33CBF672A835}</x:author>
-    <x:author>tc={723E4FE8-3707-41C4-4952-BD4B93DA8F34}</x:author>
-    <x:author>tc={94512158-8255-618B-61A4-46E5CB9BF4C3}</x:author>
-    <x:author>tc={57A2F342-59EC-EACD-8B0F-5A6C592ABFF8}</x:author>
-    <x:author>tc={AD130745-00D7-E1FF-EA07-3CC642EA0F28}</x:author>
-    <x:author>tc={EDFB07F6-6133-A276-AF5F-C8288FD3F3EB}</x:author>
-    <x:author>tc={A77E6851-727A-030B-1988-B0388B67B634}</x:author>
-    <x:author>tc={A1D96AFA-2F56-9EA9-D5BE-E6AF517B18E0}</x:author>
-    <x:author>tc={20B59283-4381-3AB4-7593-513964766437}</x:author>
-    <x:author>tc={907378BD-9DAE-40DB-115C-B4F40FAB09FA}</x:author>
-    <x:author>tc={BCB38F7A-3E13-06F4-0C9E-D41451B2A27D}</x:author>
-    <x:author>tc={6F30520B-6B11-7059-994F-29C43B5F8C2B}</x:author>
-    <x:author>tc={3424E448-7943-8047-3807-09928D5E0FC4}</x:author>
-    <x:author>tc={25606D75-0F2B-3440-6C4C-6AEC6AD95783}</x:author>
-    <x:author>tc={CC3668EB-71D5-4F1F-12DE-1FE2F18B5AE3}</x:author>
+    <x:author>tc={2E92C6EB-E2D8-BFDA-3FFB-FFE8C919781C}</x:author>
+    <x:author>tc={9996CDE2-D7F4-241B-DFFA-F4D42D8806B1}</x:author>
+    <x:author>tc={69DC4563-C2A0-EF5E-09E6-5E87691F837D}</x:author>
+    <x:author>tc={FF1A8A11-134D-C38D-8DB5-E9C4D1C91AD5}</x:author>
+    <x:author>tc={EA8BE9CD-E745-69B6-0CDE-1DBF7788ACA3}</x:author>
+    <x:author>tc={9112B102-4421-CD24-704F-50C3393D092E}</x:author>
+    <x:author>tc={7386AD46-E177-EAF6-158B-6EB952819DA5}</x:author>
+    <x:author>tc={03678F6D-9AE2-D0F2-43D1-F62224D8F251}</x:author>
+    <x:author>tc={3028E4BF-4DB9-7B67-D957-2AD9FF0DB62C}</x:author>
+    <x:author>tc={FD880EAB-91D0-0E6E-801C-B75442FA218C}</x:author>
+    <x:author>tc={638261E2-D0D3-145A-FCDE-93F77D04A644}</x:author>
+    <x:author>tc={881DE873-A154-A8D5-B621-A50E6FD4CEAD}</x:author>
+    <x:author>tc={9CB972C8-2825-D061-D42D-EB50B2E674C2}</x:author>
+    <x:author>tc={DB8F07C9-F7F7-FE73-9AA9-4C295B9B23EB}</x:author>
+    <x:author>tc={7B44EA3A-3423-C44B-17E3-6D0080C46F05}</x:author>
+    <x:author>tc={4954549F-3C47-FC30-5755-EE5CE0B1AB51}</x:author>
+    <x:author>tc={8404FF8A-6FCC-C393-80A0-6D6067BC4469}</x:author>
+    <x:author>tc={C87DDDBD-70BD-3F5F-3775-4FB9E051071A}</x:author>
+    <x:author>tc={43AC33EC-4AC1-7B72-3678-E9AF3E6C0947}</x:author>
+    <x:author>tc={D056F8AD-8D62-71DB-77C6-7D348E118036}</x:author>
+    <x:author>tc={D9B69C3A-2770-73F9-D4CF-BF9B35B56E67}</x:author>
+    <x:author>tc={7266B7B5-E168-4A57-FF19-4DFFCA6F6429}</x:author>
+    <x:author>tc={BC835D1B-78AB-F8B6-7665-58CF307B8CBD}</x:author>
+    <x:author>tc={B3C562D9-57EF-1A70-F0B0-C9ED2533183A}</x:author>
+    <x:author>tc={15E9E26E-BDFC-A1A7-B42D-11B46DC791D9}</x:author>
+    <x:author>tc={F41AD288-E4D5-652C-F9ED-09E5CBA414F4}</x:author>
+    <x:author>tc={54ACF17B-CCA7-F56F-1606-F13A0C880FB9}</x:author>
+    <x:author>tc={106CDE0D-0847-8774-3A88-7967F6FEFBF5}</x:author>
+    <x:author>tc={E4A9B24A-2E53-E635-0FD1-86B1E7B4D4FC}</x:author>
+    <x:author>tc={6744C604-48FA-71F0-0984-3B0C76DF0FCF}</x:author>
+    <x:author>tc={5D9FC781-90BA-3859-6F84-328CAEB64272}</x:author>
+    <x:author>tc={B7538A62-EED4-E0E2-C67B-592CD2DA0EAC}</x:author>
+    <x:author>tc={734EE82A-EC02-AC53-6229-5EB357680EF6}</x:author>
+    <x:author>tc={2449F982-692F-3693-49FB-AC235D7CF5FF}</x:author>
+    <x:author>tc={02F9064B-60A6-572B-3507-D60BCDE6CE0D}</x:author>
+    <x:author>tc={BE555562-4937-00C3-67AF-22CB735AE30A}</x:author>
+    <x:author>tc={2D48255E-57E9-A21E-E862-5B16DA725673}</x:author>
+    <x:author>tc={BF4A3063-2BA5-12E8-4DE1-94E638E86565}</x:author>
+    <x:author>tc={339D2B45-F391-AD3F-9928-68F2417BA655}</x:author>
+    <x:author>tc={FE419763-CFB1-9E71-B022-6BFB85067D47}</x:author>
+    <x:author>tc={33C5D95A-DFC4-9AEF-3518-07183671F73B}</x:author>
+    <x:author>tc={23880101-D8FB-6F6B-00C1-B84E43313AE5}</x:author>
+    <x:author>tc={BB5FAFEA-EF75-8EFF-94A2-FAB3033B9471}</x:author>
+    <x:author>tc={0038C068-A2EF-FD32-47D0-82185638F797}</x:author>
+    <x:author>tc={A0397957-B818-A5A2-6206-70C445C43FD0}</x:author>
+    <x:author>tc={A396B3E0-3A78-1A9C-4BB6-1C7265D008EC}</x:author>
+    <x:author>tc={92EB273B-9878-A3EF-23CB-31CA5D97583F}</x:author>
+    <x:author>tc={9B29E06A-F146-42D1-9431-2F1B83073011}</x:author>
+    <x:author>tc={A6A30EF1-3BD8-AE42-4ADC-3E139B8D75CB}</x:author>
+    <x:author>tc={C779C7F9-D99C-2006-AC15-975B5210F958}</x:author>
+    <x:author>tc={A25459FF-4404-A5D9-9C6A-981C855D41B4}</x:author>
+    <x:author>tc={CD5CFED8-5444-8040-5FE5-40D1BFCFCDEA}</x:author>
+    <x:author>tc={011BE363-BC65-1234-80BD-35C095BA9EA8}</x:author>
+    <x:author>tc={489756A7-607C-E95E-93FA-958ECFD99B77}</x:author>
+    <x:author>tc={3110FEFE-CFCC-6E61-2F84-E3010F2A2E56}</x:author>
+    <x:author>tc={11AEAC18-8255-69B8-C307-F3A8EC597CBB}</x:author>
+    <x:author>tc={7E257C73-E64C-C310-0726-0CC995D04D73}</x:author>
+    <x:author>tc={A26BBA99-261D-A8C1-1C19-3B6C23781518}</x:author>
+    <x:author>tc={42C4F2D4-D997-8E25-DBF5-E416D13982E9}</x:author>
+    <x:author>tc={0200DEEE-8DDD-F98D-D75B-354DA4F82D96}</x:author>
+    <x:author>tc={C8BD88E9-9304-50E3-8E16-D6C55A85D82F}</x:author>
+    <x:author>tc={6D8D1C81-76D3-7096-11BA-5A5EC67B2A6A}</x:author>
+    <x:author>tc={31BD5FE4-E91C-E52C-7DE9-DC8E66E74B66}</x:author>
+    <x:author>tc={B8746BCC-7A92-5A75-D95A-97D8AFB392FD}</x:author>
+    <x:author>tc={AE775D8D-A6BF-AD24-E330-D32376FC9EFF}</x:author>
+    <x:author>tc={097E4B9D-D491-0EE3-2052-ACEAFB247869}</x:author>
+    <x:author>tc={BAB54389-08BB-FCB3-FA4E-D008BD27EF98}</x:author>
+    <x:author>tc={B6EB26F3-1F85-E7B1-0864-D3DE48E3B21F}</x:author>
+    <x:author>tc={019F2DF5-928D-1D4C-DE17-4E340A98EF86}</x:author>
+    <x:author>tc={99DC1528-B916-6FB8-3288-9715AE9DD2B9}</x:author>
+    <x:author>tc={1DE7D797-4DF6-30EA-56A0-7F11E54456D2}</x:author>
+    <x:author>tc={3111A50E-EAEE-E93F-39D6-3C3749F5171B}</x:author>
+    <x:author>tc={BAEBA302-ADD3-AE44-452C-C97146616383}</x:author>
+    <x:author>tc={5C0FBD2A-5940-3C5D-2C6B-542E0F6BB157}</x:author>
+    <x:author>tc={79C20CC6-A9AC-211C-F83E-1635C7DAC3E4}</x:author>
+    <x:author>tc={64B0F472-67A6-40C1-30B0-8CE7DFC47D2A}</x:author>
+    <x:author>tc={1D13A87F-E7F0-347E-6024-33FE60195697}</x:author>
+    <x:author>tc={3147F0B5-2D94-55A9-492D-95CBAA3E40C1}</x:author>
+    <x:author>tc={FF7CAD37-5E80-7B10-8138-128DF1E42913}</x:author>
+    <x:author>tc={E5B395E6-BE93-46DB-6176-E9240DBE5FA7}</x:author>
+    <x:author>tc={7A281728-42ED-41E8-0344-E95F40D4E6E1}</x:author>
+    <x:author>tc={E92CF26C-E2E0-4E74-967C-976222B2ED8D}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1175,26 +1175,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={1838D36A-0B6F-90ED-EEF7-EC269097E000}</x:author>
-    <x:author>tc={25664E63-F7D0-2ED2-1E36-B86F6453DBCB}</x:author>
-    <x:author>tc={80412385-F135-D38A-004D-6F5F6C63C5F6}</x:author>
-    <x:author>tc={9E6EFBC5-ABE1-615A-AF44-25D10AE6E7F4}</x:author>
-    <x:author>tc={C8EDEBC0-9E31-AD81-3E27-7A04D720EE10}</x:author>
-    <x:author>tc={C55543F7-83A1-C507-C151-19B020556FC2}</x:author>
-    <x:author>tc={6B4C6DC8-5E02-8BB5-27C6-E437E820E45B}</x:author>
-    <x:author>tc={7EE12C14-0C36-7979-3EB2-B9DBCADAC67F}</x:author>
-    <x:author>tc={F4CF8361-796D-E1ED-658C-37FD5BE42402}</x:author>
-    <x:author>tc={61E96BB7-8123-81EC-BA03-94C430C99D86}</x:author>
-    <x:author>tc={0BB437E8-B12C-B8A8-B0B0-460BF96CBBE0}</x:author>
-    <x:author>tc={1482B62C-D7DA-F789-CE45-A7B2609F1141}</x:author>
-    <x:author>tc={F7CC6DE2-EB78-E65C-2B11-8FEC33112CF1}</x:author>
-    <x:author>tc={5B619671-60EC-DDB3-6328-C666564CA16E}</x:author>
-    <x:author>tc={E2519075-1BEC-D13A-A7BA-0882E4D90356}</x:author>
-    <x:author>tc={A309184C-D446-A9CA-6A98-DE97B2886C79}</x:author>
-    <x:author>tc={D8DEC458-CF8E-683F-BC94-01B941CFE541}</x:author>
-    <x:author>tc={AD84876E-767D-A96E-6751-D4DFAE7D1131}</x:author>
-    <x:author>tc={1F015695-0961-7C20-4F5D-A510B3E38413}</x:author>
-    <x:author>tc={BF7AB4AB-5D80-B11C-F9A6-264AE0D86812}</x:author>
+    <x:author>tc={8812A0C8-AE12-CDC4-6559-5ED2998582C7}</x:author>
+    <x:author>tc={FF227541-2EBA-6C23-20BF-5B28E39E9681}</x:author>
+    <x:author>tc={6DE872F6-CA39-0FC9-7DE8-CCF9546B71E5}</x:author>
+    <x:author>tc={CA7CA3B9-387D-9A7E-E5BD-07FB06E11781}</x:author>
+    <x:author>tc={CB8B831A-CE11-2600-48F0-6351067797E4}</x:author>
+    <x:author>tc={C9E6A202-F5C7-C993-DCDC-007DFBA7BEA6}</x:author>
+    <x:author>tc={CDF35263-C850-DFCD-98B8-586343840BE3}</x:author>
+    <x:author>tc={44D94C18-83CB-3B9B-2D29-05BBC1FBF62B}</x:author>
+    <x:author>tc={0B3D40B5-E2AC-994F-57E0-3315321ACDDB}</x:author>
+    <x:author>tc={B2711685-4E1D-9BB8-5657-87F356D886BB}</x:author>
+    <x:author>tc={4E54290C-D4A3-B396-1C0F-2BE4BFF8B4FC}</x:author>
+    <x:author>tc={DA55FDFC-FFC0-B937-406F-09F9817E6A38}</x:author>
+    <x:author>tc={583B0DDD-9F98-5FA2-37E3-5C63FE21466A}</x:author>
+    <x:author>tc={DCC83C46-E129-758A-352E-069886DF1D30}</x:author>
+    <x:author>tc={E41433D0-30E7-C9AD-5360-E0480823C874}</x:author>
+    <x:author>tc={74CC3BFD-C520-7302-3AA5-63E435AA8BF1}</x:author>
+    <x:author>tc={22072459-F97F-B746-085E-C1638D4655EB}</x:author>
+    <x:author>tc={C4E12AE5-C49C-C348-687A-9FF2BF406408}</x:author>
+    <x:author>tc={29DD92EC-6D8D-4931-C0AC-C83AA74C94FE}</x:author>
+    <x:author>tc={37F22D93-CFD6-BE05-6212-E8097B58D230}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2037,7 +2037,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6a7a0c8792ea46ba"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R23e26fa3f9f945d1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2048,7 +2048,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}"/>
 </xltc:personList>
 </file>
 
@@ -2245,493 +2245,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-12T20:09:22.914" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{75551666-5AE4-C06F-F275-345195AD9824}">
+  <xltc:threadedComment ref="P5" dT="2026-08-12T20:51:37.472" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{2E92C6EB-E2D8-BFDA-3FFB-FFE8C919781C}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-12T20:09:22.916" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{564C1C2A-9CE5-EA61-5DCD-F4FE8503953B}">
+  <xltc:threadedComment ref="P6" dT="2026-08-12T20:51:37.484" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{9996CDE2-D7F4-241B-DFFA-F4D42D8806B1}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{6B84FBAC-76BC-060D-35F0-ACDFC46FEED9}">
+  <xltc:threadedComment ref="P7" dT="2026-08-12T20:51:37.484" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{69DC4563-C2A0-EF5E-09E6-5E87691F837D}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E272EB50-439D-B2DD-2DF1-EA75847E6ED8}">
+  <xltc:threadedComment ref="P8" dT="2026-08-12T20:51:37.484" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FF1A8A11-134D-C38D-8DB5-E9C4D1C91AD5}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{2BDBC44B-72B0-BE02-1CD3-59028DB471DB}">
+  <xltc:threadedComment ref="P9" dT="2026-08-12T20:51:37.484" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{EA8BE9CD-E745-69B6-0CDE-1DBF7788ACA3}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{77D96203-6107-53E4-2A0C-3E2E98D4FAD4}">
+  <xltc:threadedComment ref="P10" dT="2026-08-12T20:51:37.485" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{9112B102-4421-CD24-704F-50C3393D092E}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{78A9ED23-6B0D-B401-C5DC-831E23F15C31}">
+  <xltc:threadedComment ref="P11" dT="2026-08-12T20:51:37.485" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7386AD46-E177-EAF6-158B-6EB952819DA5}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{ACA3EDE8-684B-1099-8486-C7FF1B13DB7E}">
+  <xltc:threadedComment ref="P12" dT="2026-08-12T20:51:37.485" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{03678F6D-9AE2-D0F2-43D1-F62224D8F251}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-12T20:09:22.917" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{055DB408-E0EA-A2F3-06F1-2255F199A597}">
+  <xltc:threadedComment ref="P13" dT="2026-08-12T20:51:37.485" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{3028E4BF-4DB9-7B67-D957-2AD9FF0DB62C}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{9DD9D7DF-B5C6-4A72-5620-8D579DC7A395}">
+  <xltc:threadedComment ref="P14" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FD880EAB-91D0-0E6E-801C-B75442FA218C}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{38743DC3-BEC9-B6B3-EE19-C2A7150C7E5F}">
+  <xltc:threadedComment ref="P15" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{638261E2-D0D3-145A-FCDE-93F77D04A644}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1681E5A1-644C-4F49-E9F5-473EDC3106DD}">
+  <xltc:threadedComment ref="P16" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{881DE873-A154-A8D5-B621-A50E6FD4CEAD}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{08A165E7-1078-8440-2818-F2ED3F3298F4}">
+  <xltc:threadedComment ref="P17" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{9CB972C8-2825-D061-D42D-EB50B2E674C2}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{67841105-8DD3-58EA-6E86-0E1D75050B48}">
+  <xltc:threadedComment ref="P18" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{DB8F07C9-F7F7-FE73-9AA9-4C295B9B23EB}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{6838EBFF-AD44-1E4D-1CE6-64B69E9D00B6}">
+  <xltc:threadedComment ref="P19" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7B44EA3A-3423-C44B-17E3-6D0080C46F05}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{423C179F-5F8C-3495-39C3-5A3C8A6AF2BE}">
+  <xltc:threadedComment ref="P20" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{4954549F-3C47-FC30-5755-EE5CE0B1AB51}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{3615ABDC-CE76-6317-52F6-295F96996482}">
+  <xltc:threadedComment ref="P21" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{8404FF8A-6FCC-C393-80A0-6D6067BC4469}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{03A863CC-C443-36F1-88DD-197230A3C218}">
+  <xltc:threadedComment ref="P22" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C87DDDBD-70BD-3F5F-3775-4FB9E051071A}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BA1F7F5A-69CF-2A50-4D76-136DBEEF91A0}">
+  <xltc:threadedComment ref="P23" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{43AC33EC-4AC1-7B72-3678-E9AF3E6C0947}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{3856393E-6F1E-8E64-E73F-53BEE2CFD334}">
+  <xltc:threadedComment ref="P24" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{D056F8AD-8D62-71DB-77C6-7D348E118036}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{C4E32F58-B171-DA72-C52B-E695171754C0}">
+  <xltc:threadedComment ref="P25" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{D9B69C3A-2770-73F9-D4CF-BF9B35B56E67}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{3F621C88-4B70-7F61-0136-EB359AA5D0DF}">
+  <xltc:threadedComment ref="P26" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7266B7B5-E168-4A57-FF19-4DFFCA6F6429}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{672D185B-9D4C-9FC6-A4BA-36C418B71A99}">
+  <xltc:threadedComment ref="P27" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BC835D1B-78AB-F8B6-7665-58CF307B8CBD}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{49E31FAE-AC0B-6B9E-42FF-4DF348CB71CA}">
+  <xltc:threadedComment ref="P28" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B3C562D9-57EF-1A70-F0B0-C9ED2533183A}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{B499671D-EDC5-571C-F4EA-699941D0AC08}">
+  <xltc:threadedComment ref="P29" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{15E9E26E-BDFC-A1A7-B42D-11B46DC791D9}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{7BF3F0D5-2C28-AC82-3B38-3C4997446926}">
+  <xltc:threadedComment ref="P30" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{F41AD288-E4D5-652C-F9ED-09E5CBA414F4}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{8067B179-C218-DDEE-402A-47BBD893AAD9}">
+  <xltc:threadedComment ref="P31" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{54ACF17B-CCA7-F56F-1606-F13A0C880FB9}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{5DFD983F-0230-623B-F299-D70185218300}">
+  <xltc:threadedComment ref="P32" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{106CDE0D-0847-8774-3A88-7967F6FEFBF5}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E407B8C4-8D66-09E4-5388-A6BED433D14F}">
+  <xltc:threadedComment ref="P33" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{E4A9B24A-2E53-E635-0FD1-86B1E7B4D4FC}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{68AD1868-B5AA-7CB0-0686-6B067C5C217E}">
+  <xltc:threadedComment ref="P34" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{6744C604-48FA-71F0-0984-3B0C76DF0FCF}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D4BD99D9-46A9-3F6B-37CD-620F0123098E}">
+  <xltc:threadedComment ref="P35" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{5D9FC781-90BA-3859-6F84-328CAEB64272}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{4832AFE5-5336-0617-B446-43C1D1044874}">
+  <xltc:threadedComment ref="P36" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B7538A62-EED4-E0E2-C67B-592CD2DA0EAC}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-12T20:09:22.918" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1175AC3C-7D1F-23C8-74BB-CDA1B793F3A7}">
+  <xltc:threadedComment ref="P37" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{734EE82A-EC02-AC53-6229-5EB357680EF6}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{2D6229C6-77F1-0DB7-E1EC-418843C35F53}">
+  <xltc:threadedComment ref="P38" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{2449F982-692F-3693-49FB-AC235D7CF5FF}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A2565DB1-37B7-3FE6-F0EE-6FA12E6A25D3}">
+  <xltc:threadedComment ref="P39" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{02F9064B-60A6-572B-3507-D60BCDE6CE0D}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D3EF764D-2D5E-904F-9AB1-3A38E612BA26}">
+  <xltc:threadedComment ref="P40" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BE555562-4937-00C3-67AF-22CB735AE30A}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{8D7B5EDF-4CFB-DBBB-FA2D-C9B68C40C153}">
+  <xltc:threadedComment ref="P41" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{2D48255E-57E9-A21E-E862-5B16DA725673}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D587F045-A020-A06B-AB17-12DBCABBD168}">
+  <xltc:threadedComment ref="P42" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BF4A3063-2BA5-12E8-4DE1-94E638E86565}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D7DE69B5-A8B1-11B2-C950-F41D8CBD9F15}">
+  <xltc:threadedComment ref="P43" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{339D2B45-F391-AD3F-9928-68F2417BA655}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BEE2D092-C2E2-3467-8307-A5C89B8B68AE}">
+  <xltc:threadedComment ref="P44" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FE419763-CFB1-9E71-B022-6BFB85067D47}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{44719A85-CEF6-270A-B1DF-36205A4BD2DF}">
+  <xltc:threadedComment ref="P45" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{33C5D95A-DFC4-9AEF-3518-07183671F73B}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D220E222-EBCE-94A7-D472-3CDFB73FEC99}">
+  <xltc:threadedComment ref="P46" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{23880101-D8FB-6F6B-00C1-B84E43313AE5}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{CF3183DE-4FFD-CC85-557B-92B5C2FBBDA4}">
+  <xltc:threadedComment ref="P47" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BB5FAFEA-EF75-8EFF-94A2-FAB3033B9471}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{7BD1BCA9-983D-4F81-F09B-5256770BD208}">
+  <xltc:threadedComment ref="P48" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{0038C068-A2EF-FD32-47D0-82185638F797}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{2A1DD6A3-F325-89A6-3642-16C0B71CF7E7}">
+  <xltc:threadedComment ref="P49" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A0397957-B818-A5A2-6206-70C445C43FD0}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1B0F2425-537F-8832-6F2B-C5E1367F17F5}">
+  <xltc:threadedComment ref="P50" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A396B3E0-3A78-1A9C-4BB6-1C7265D008EC}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{51E6CFE9-07B2-BFE8-8A2D-97D2F6E2D86D}">
+  <xltc:threadedComment ref="P51" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{92EB273B-9878-A3EF-23CB-31CA5D97583F}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{13064D26-4B82-ABAE-7912-BCB10B5229FC}">
+  <xltc:threadedComment ref="P52" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{9B29E06A-F146-42D1-9431-2F1B83073011}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{2D5ECB66-708D-32B9-396B-2E302301F13A}">
+  <xltc:threadedComment ref="P53" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A6A30EF1-3BD8-AE42-4ADC-3E139B8D75CB}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{AE338A8D-E206-E06B-F8A1-90D3D7F3C769}">
+  <xltc:threadedComment ref="P54" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C779C7F9-D99C-2006-AC15-975B5210F958}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{30C6CC82-6FCC-FA84-891A-A29620402234}">
+  <xltc:threadedComment ref="P55" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A25459FF-4404-A5D9-9C6A-981C855D41B4}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BBD5CB37-08D4-D4AA-3F59-A8FBDB944903}">
+  <xltc:threadedComment ref="P56" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{CD5CFED8-5444-8040-5FE5-40D1BFCFCDEA}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{668F0A05-5026-1B02-ED6E-D9C966D3E4EC}">
+  <xltc:threadedComment ref="P57" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{011BE363-BC65-1234-80BD-35C095BA9EA8}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{B4147D19-C24D-6C5E-BFE9-9844FBEA64A4}">
+  <xltc:threadedComment ref="P58" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{489756A7-607C-E95E-93FA-958ECFD99B77}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{B540F690-35AF-9C2C-E6EF-AB99A19D3CB4}">
+  <xltc:threadedComment ref="P59" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{3110FEFE-CFCC-6E61-2F84-E3010F2A2E56}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{7CE0EECF-5DF4-B1E6-228F-4CDBAA7E88DF}">
+  <xltc:threadedComment ref="P60" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{11AEAC18-8255-69B8-C307-F3A8EC597CBB}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{4A35FCBF-8F2C-BA1D-568D-1D8DD20B97D3}">
+  <xltc:threadedComment ref="P61" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7E257C73-E64C-C310-0726-0CC995D04D73}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-12T20:09:22.919" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A882E23F-032E-FA6E-B4A2-12C63FF54E0C}">
+  <xltc:threadedComment ref="P62" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A26BBA99-261D-A8C1-1C19-3B6C23781518}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{4142D1C2-7A4B-B9FA-2C32-810525F47331}">
+  <xltc:threadedComment ref="P63" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{42C4F2D4-D997-8E25-DBF5-E416D13982E9}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E13BB1CE-65C2-66DC-EE1F-C6C3D55667C6}">
+  <xltc:threadedComment ref="P64" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{0200DEEE-8DDD-F98D-D75B-354DA4F82D96}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A91352D0-D317-15A4-7D71-C2A6585D0F68}">
+  <xltc:threadedComment ref="P65" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C8BD88E9-9304-50E3-8E16-D6C55A85D82F}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{72227493-2DF3-671B-9FA1-275E12824727}">
+  <xltc:threadedComment ref="P66" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{6D8D1C81-76D3-7096-11BA-5A5EC67B2A6A}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{12FCF11E-4671-2735-753D-4D2C8E642B4C}">
+  <xltc:threadedComment ref="P67" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{31BD5FE4-E91C-E52C-7DE9-DC8E66E74B66}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E3A0655B-7B8D-2B4E-C29C-1690F7526BA5}">
+  <xltc:threadedComment ref="P68" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B8746BCC-7A92-5A75-D95A-97D8AFB392FD}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{95BEE8B6-7DEB-63DC-740F-662516460A29}">
+  <xltc:threadedComment ref="P69" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{AE775D8D-A6BF-AD24-E330-D32376FC9EFF}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{C064FFA2-40E3-8C1B-4948-37B03A027824}">
+  <xltc:threadedComment ref="P70" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{097E4B9D-D491-0EE3-2052-ACEAFB247869}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{65F77BF5-7F3D-8006-4E53-04C8F692A7BC}">
+  <xltc:threadedComment ref="P71" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BAB54389-08BB-FCB3-FA4E-D008BD27EF98}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{13B8E3E6-9F10-4C37-F266-33CBF672A835}">
+  <xltc:threadedComment ref="P72" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B6EB26F3-1F85-E7B1-0864-D3DE48E3B21F}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{723E4FE8-3707-41C4-4952-BD4B93DA8F34}">
+  <xltc:threadedComment ref="P73" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{019F2DF5-928D-1D4C-DE17-4E340A98EF86}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{94512158-8255-618B-61A4-46E5CB9BF4C3}">
+  <xltc:threadedComment ref="P74" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{99DC1528-B916-6FB8-3288-9715AE9DD2B9}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{57A2F342-59EC-EACD-8B0F-5A6C592ABFF8}">
+  <xltc:threadedComment ref="P75" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{1DE7D797-4DF6-30EA-56A0-7F11E54456D2}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{AD130745-00D7-E1FF-EA07-3CC642EA0F28}">
+  <xltc:threadedComment ref="P76" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{3111A50E-EAEE-E93F-39D6-3C3749F5171B}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{EDFB07F6-6133-A276-AF5F-C8288FD3F3EB}">
+  <xltc:threadedComment ref="P77" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BAEBA302-ADD3-AE44-452C-C97146616383}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A77E6851-727A-030B-1988-B0388B67B634}">
+  <xltc:threadedComment ref="P78" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{5C0FBD2A-5940-3C5D-2C6B-542E0F6BB157}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A1D96AFA-2F56-9EA9-D5BE-E6AF517B18E0}">
+  <xltc:threadedComment ref="P79" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{79C20CC6-A9AC-211C-F83E-1635C7DAC3E4}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{20B59283-4381-3AB4-7593-513964766437}">
+  <xltc:threadedComment ref="P80" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{64B0F472-67A6-40C1-30B0-8CE7DFC47D2A}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{907378BD-9DAE-40DB-115C-B4F40FAB09FA}">
+  <xltc:threadedComment ref="P81" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{1D13A87F-E7F0-347E-6024-33FE60195697}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BCB38F7A-3E13-06F4-0C9E-D41451B2A27D}">
+  <xltc:threadedComment ref="P82" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{3147F0B5-2D94-55A9-492D-95CBAA3E40C1}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{6F30520B-6B11-7059-994F-29C43B5F8C2B}">
+  <xltc:threadedComment ref="P83" dT="2026-08-12T20:51:37.49" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FF7CAD37-5E80-7B10-8138-128DF1E42913}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{3424E448-7943-8047-3807-09928D5E0FC4}">
+  <xltc:threadedComment ref="P84" dT="2026-08-12T20:51:37.49" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{E5B395E6-BE93-46DB-6176-E9240DBE5FA7}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{25606D75-0F2B-3440-6C4C-6AEC6AD95783}">
+  <xltc:threadedComment ref="P85" dT="2026-08-12T20:51:37.49" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7A281728-42ED-41E8-0344-E95F40D4E6E1}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-12T20:09:22.92" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{CC3668EB-71D5-4F1F-12DE-1FE2F18B5AE3}">
+  <xltc:threadedComment ref="P86" dT="2026-08-12T20:51:37.49" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{E92CF26C-E2E0-4E74-967C-976222B2ED8D}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2742,64 +2742,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-12T20:09:23.291" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1838D36A-0B6F-90ED-EEF7-EC269097E000}">
+  <xltc:threadedComment ref="J5" dT="2026-08-12T20:51:38.167" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{8812A0C8-AE12-CDC4-6559-5ED2998582C7}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-12T20:09:23.294" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{25664E63-F7D0-2ED2-1E36-B86F6453DBCB}">
+  <xltc:threadedComment ref="J6" dT="2026-08-12T20:51:38.172" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FF227541-2EBA-6C23-20BF-5B28E39E9681}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-12T20:09:23.296" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{80412385-F135-D38A-004D-6F5F6C63C5F6}">
+  <xltc:threadedComment ref="J7" dT="2026-08-12T20:51:38.176" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{6DE872F6-CA39-0FC9-7DE8-CCF9546B71E5}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-12T20:09:23.299" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{9E6EFBC5-ABE1-615A-AF44-25D10AE6E7F4}">
+  <xltc:threadedComment ref="J8" dT="2026-08-12T20:51:38.181" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{CA7CA3B9-387D-9A7E-E5BD-07FB06E11781}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-12T20:09:23.302" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{C8EDEBC0-9E31-AD81-3E27-7A04D720EE10}">
+  <xltc:threadedComment ref="J9" dT="2026-08-12T20:51:38.185" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{CB8B831A-CE11-2600-48F0-6351067797E4}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-12T20:09:23.304" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{C55543F7-83A1-C507-C151-19B020556FC2}">
+  <xltc:threadedComment ref="J10" dT="2026-08-12T20:51:38.189" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C9E6A202-F5C7-C993-DCDC-007DFBA7BEA6}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-12T20:09:23.307" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{6B4C6DC8-5E02-8BB5-27C6-E437E820E45B}">
+  <xltc:threadedComment ref="J11" dT="2026-08-12T20:51:38.194" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{CDF35263-C850-DFCD-98B8-586343840BE3}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-12T20:09:23.31" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{7EE12C14-0C36-7979-3EB2-B9DBCADAC67F}">
+  <xltc:threadedComment ref="J12" dT="2026-08-12T20:51:38.199" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{44D94C18-83CB-3B9B-2D29-05BBC1FBF62B}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-12T20:09:23.313" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{F4CF8361-796D-E1ED-658C-37FD5BE42402}">
+  <xltc:threadedComment ref="J13" dT="2026-08-12T20:51:38.204" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{0B3D40B5-E2AC-994F-57E0-3315321ACDDB}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-12T20:09:23.316" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{61E96BB7-8123-81EC-BA03-94C430C99D86}">
+  <xltc:threadedComment ref="J14" dT="2026-08-12T20:51:38.209" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B2711685-4E1D-9BB8-5657-87F356D886BB}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-12T20:09:23.318" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{0BB437E8-B12C-B8A8-B0B0-460BF96CBBE0}">
+  <xltc:threadedComment ref="J15" dT="2026-08-12T20:51:38.213" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{4E54290C-D4A3-B396-1C0F-2BE4BFF8B4FC}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-12T20:09:23.322" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1482B62C-D7DA-F789-CE45-A7B2609F1141}">
+  <xltc:threadedComment ref="J16" dT="2026-08-12T20:51:38.217" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{DA55FDFC-FFC0-B937-406F-09F9817E6A38}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-12T20:09:23.324" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{F7CC6DE2-EB78-E65C-2B11-8FEC33112CF1}">
+  <xltc:threadedComment ref="J17" dT="2026-08-12T20:51:38.22" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{583B0DDD-9F98-5FA2-37E3-5C63FE21466A}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-12T20:09:23.327" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{5B619671-60EC-DDB3-6328-C666564CA16E}">
+  <xltc:threadedComment ref="J18" dT="2026-08-12T20:51:38.224" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{DCC83C46-E129-758A-352E-069886DF1D30}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-12T20:09:23.329" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{E2519075-1BEC-D13A-A7BA-0882E4D90356}">
+  <xltc:threadedComment ref="J19" dT="2026-08-12T20:51:38.227" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{E41433D0-30E7-C9AD-5360-E0480823C874}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-12T20:09:23.331" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{A309184C-D446-A9CA-6A98-DE97B2886C79}">
+  <xltc:threadedComment ref="J20" dT="2026-08-12T20:51:38.231" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{74CC3BFD-C520-7302-3AA5-63E435AA8BF1}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-12T20:09:23.333" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{D8DEC458-CF8E-683F-BC94-01B941CFE541}">
+  <xltc:threadedComment ref="J21" dT="2026-08-12T20:51:38.233" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{22072459-F97F-B746-085E-C1638D4655EB}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-12T20:09:23.337" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{AD84876E-767D-A96E-6751-D4DFAE7D1131}">
+  <xltc:threadedComment ref="J22" dT="2026-08-12T20:51:38.238" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C4E12AE5-C49C-C348-687A-9FF2BF406408}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-12T20:09:23.34" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{1F015695-0961-7C20-4F5D-A510B3E38413}">
+  <xltc:threadedComment ref="J23" dT="2026-08-12T20:51:38.242" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{29DD92EC-6D8D-4931-C0AC-C83AA74C94FE}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-12T20:09:23.344" personId="{0C3580B4-ED2E-45B0-8EA6-D9E897799064}" id="{BF7AB4AB-5D80-B11C-F9A6-264AE0D86812}">
+  <xltc:threadedComment ref="J24" dT="2026-08-12T20:51:38.246" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{37F22D93-CFD6-BE05-6212-E8097B58D230}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -7802,7 +7802,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f1a10d85f848f1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ddb199f43394c37"/>
 </x:worksheet>
 </file>
 
@@ -8862,7 +8862,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R813bdb3960b54ec4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16f89965a1d645a4"/>
 </x:worksheet>
 </file>
 
@@ -20015,6 +20015,6 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcead52240fa44262"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9209b29ba07c40d5"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Bind final canonical V3.1.1 judging artifacts
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rd1ffe793c0054f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R3f65de9dedce4afe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rf6fd4f58afdb43af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rd5f0909783b14bfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="Rbcfe6e4453ef4e4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R28243a9317964192"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R5033da0595304c36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R5318b55946a541cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R74b838b5d8c24721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R5479d667b91a41da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R1cf8fe4b73d94fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rc86845b7ef8d470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R9ebf82b829c64679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R2583efb584614649"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R119b6ab68baf40ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R5bb9062add75423a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Rd0ca1092916b426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R1a340cffa65d454b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,88 +18,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={2E92C6EB-E2D8-BFDA-3FFB-FFE8C919781C}</x:author>
-    <x:author>tc={9996CDE2-D7F4-241B-DFFA-F4D42D8806B1}</x:author>
-    <x:author>tc={69DC4563-C2A0-EF5E-09E6-5E87691F837D}</x:author>
-    <x:author>tc={FF1A8A11-134D-C38D-8DB5-E9C4D1C91AD5}</x:author>
-    <x:author>tc={EA8BE9CD-E745-69B6-0CDE-1DBF7788ACA3}</x:author>
-    <x:author>tc={9112B102-4421-CD24-704F-50C3393D092E}</x:author>
-    <x:author>tc={7386AD46-E177-EAF6-158B-6EB952819DA5}</x:author>
-    <x:author>tc={03678F6D-9AE2-D0F2-43D1-F62224D8F251}</x:author>
-    <x:author>tc={3028E4BF-4DB9-7B67-D957-2AD9FF0DB62C}</x:author>
-    <x:author>tc={FD880EAB-91D0-0E6E-801C-B75442FA218C}</x:author>
-    <x:author>tc={638261E2-D0D3-145A-FCDE-93F77D04A644}</x:author>
-    <x:author>tc={881DE873-A154-A8D5-B621-A50E6FD4CEAD}</x:author>
-    <x:author>tc={9CB972C8-2825-D061-D42D-EB50B2E674C2}</x:author>
-    <x:author>tc={DB8F07C9-F7F7-FE73-9AA9-4C295B9B23EB}</x:author>
-    <x:author>tc={7B44EA3A-3423-C44B-17E3-6D0080C46F05}</x:author>
-    <x:author>tc={4954549F-3C47-FC30-5755-EE5CE0B1AB51}</x:author>
-    <x:author>tc={8404FF8A-6FCC-C393-80A0-6D6067BC4469}</x:author>
-    <x:author>tc={C87DDDBD-70BD-3F5F-3775-4FB9E051071A}</x:author>
-    <x:author>tc={43AC33EC-4AC1-7B72-3678-E9AF3E6C0947}</x:author>
-    <x:author>tc={D056F8AD-8D62-71DB-77C6-7D348E118036}</x:author>
-    <x:author>tc={D9B69C3A-2770-73F9-D4CF-BF9B35B56E67}</x:author>
-    <x:author>tc={7266B7B5-E168-4A57-FF19-4DFFCA6F6429}</x:author>
-    <x:author>tc={BC835D1B-78AB-F8B6-7665-58CF307B8CBD}</x:author>
-    <x:author>tc={B3C562D9-57EF-1A70-F0B0-C9ED2533183A}</x:author>
-    <x:author>tc={15E9E26E-BDFC-A1A7-B42D-11B46DC791D9}</x:author>
-    <x:author>tc={F41AD288-E4D5-652C-F9ED-09E5CBA414F4}</x:author>
-    <x:author>tc={54ACF17B-CCA7-F56F-1606-F13A0C880FB9}</x:author>
-    <x:author>tc={106CDE0D-0847-8774-3A88-7967F6FEFBF5}</x:author>
-    <x:author>tc={E4A9B24A-2E53-E635-0FD1-86B1E7B4D4FC}</x:author>
-    <x:author>tc={6744C604-48FA-71F0-0984-3B0C76DF0FCF}</x:author>
-    <x:author>tc={5D9FC781-90BA-3859-6F84-328CAEB64272}</x:author>
-    <x:author>tc={B7538A62-EED4-E0E2-C67B-592CD2DA0EAC}</x:author>
-    <x:author>tc={734EE82A-EC02-AC53-6229-5EB357680EF6}</x:author>
-    <x:author>tc={2449F982-692F-3693-49FB-AC235D7CF5FF}</x:author>
-    <x:author>tc={02F9064B-60A6-572B-3507-D60BCDE6CE0D}</x:author>
-    <x:author>tc={BE555562-4937-00C3-67AF-22CB735AE30A}</x:author>
-    <x:author>tc={2D48255E-57E9-A21E-E862-5B16DA725673}</x:author>
-    <x:author>tc={BF4A3063-2BA5-12E8-4DE1-94E638E86565}</x:author>
-    <x:author>tc={339D2B45-F391-AD3F-9928-68F2417BA655}</x:author>
-    <x:author>tc={FE419763-CFB1-9E71-B022-6BFB85067D47}</x:author>
-    <x:author>tc={33C5D95A-DFC4-9AEF-3518-07183671F73B}</x:author>
-    <x:author>tc={23880101-D8FB-6F6B-00C1-B84E43313AE5}</x:author>
-    <x:author>tc={BB5FAFEA-EF75-8EFF-94A2-FAB3033B9471}</x:author>
-    <x:author>tc={0038C068-A2EF-FD32-47D0-82185638F797}</x:author>
-    <x:author>tc={A0397957-B818-A5A2-6206-70C445C43FD0}</x:author>
-    <x:author>tc={A396B3E0-3A78-1A9C-4BB6-1C7265D008EC}</x:author>
-    <x:author>tc={92EB273B-9878-A3EF-23CB-31CA5D97583F}</x:author>
-    <x:author>tc={9B29E06A-F146-42D1-9431-2F1B83073011}</x:author>
-    <x:author>tc={A6A30EF1-3BD8-AE42-4ADC-3E139B8D75CB}</x:author>
-    <x:author>tc={C779C7F9-D99C-2006-AC15-975B5210F958}</x:author>
-    <x:author>tc={A25459FF-4404-A5D9-9C6A-981C855D41B4}</x:author>
-    <x:author>tc={CD5CFED8-5444-8040-5FE5-40D1BFCFCDEA}</x:author>
-    <x:author>tc={011BE363-BC65-1234-80BD-35C095BA9EA8}</x:author>
-    <x:author>tc={489756A7-607C-E95E-93FA-958ECFD99B77}</x:author>
-    <x:author>tc={3110FEFE-CFCC-6E61-2F84-E3010F2A2E56}</x:author>
-    <x:author>tc={11AEAC18-8255-69B8-C307-F3A8EC597CBB}</x:author>
-    <x:author>tc={7E257C73-E64C-C310-0726-0CC995D04D73}</x:author>
-    <x:author>tc={A26BBA99-261D-A8C1-1C19-3B6C23781518}</x:author>
-    <x:author>tc={42C4F2D4-D997-8E25-DBF5-E416D13982E9}</x:author>
-    <x:author>tc={0200DEEE-8DDD-F98D-D75B-354DA4F82D96}</x:author>
-    <x:author>tc={C8BD88E9-9304-50E3-8E16-D6C55A85D82F}</x:author>
-    <x:author>tc={6D8D1C81-76D3-7096-11BA-5A5EC67B2A6A}</x:author>
-    <x:author>tc={31BD5FE4-E91C-E52C-7DE9-DC8E66E74B66}</x:author>
-    <x:author>tc={B8746BCC-7A92-5A75-D95A-97D8AFB392FD}</x:author>
-    <x:author>tc={AE775D8D-A6BF-AD24-E330-D32376FC9EFF}</x:author>
-    <x:author>tc={097E4B9D-D491-0EE3-2052-ACEAFB247869}</x:author>
-    <x:author>tc={BAB54389-08BB-FCB3-FA4E-D008BD27EF98}</x:author>
-    <x:author>tc={B6EB26F3-1F85-E7B1-0864-D3DE48E3B21F}</x:author>
-    <x:author>tc={019F2DF5-928D-1D4C-DE17-4E340A98EF86}</x:author>
-    <x:author>tc={99DC1528-B916-6FB8-3288-9715AE9DD2B9}</x:author>
-    <x:author>tc={1DE7D797-4DF6-30EA-56A0-7F11E54456D2}</x:author>
-    <x:author>tc={3111A50E-EAEE-E93F-39D6-3C3749F5171B}</x:author>
-    <x:author>tc={BAEBA302-ADD3-AE44-452C-C97146616383}</x:author>
-    <x:author>tc={5C0FBD2A-5940-3C5D-2C6B-542E0F6BB157}</x:author>
-    <x:author>tc={79C20CC6-A9AC-211C-F83E-1635C7DAC3E4}</x:author>
-    <x:author>tc={64B0F472-67A6-40C1-30B0-8CE7DFC47D2A}</x:author>
-    <x:author>tc={1D13A87F-E7F0-347E-6024-33FE60195697}</x:author>
-    <x:author>tc={3147F0B5-2D94-55A9-492D-95CBAA3E40C1}</x:author>
-    <x:author>tc={FF7CAD37-5E80-7B10-8138-128DF1E42913}</x:author>
-    <x:author>tc={E5B395E6-BE93-46DB-6176-E9240DBE5FA7}</x:author>
-    <x:author>tc={7A281728-42ED-41E8-0344-E95F40D4E6E1}</x:author>
-    <x:author>tc={E92CF26C-E2E0-4E74-967C-976222B2ED8D}</x:author>
+    <x:author>tc={EE808468-1A8F-6BF2-A061-4A7638F69B4F}</x:author>
+    <x:author>tc={6E34D41F-1133-57CD-4563-EF7A95211AD1}</x:author>
+    <x:author>tc={9FB4D332-049B-3B73-FC58-DC11CBCB6572}</x:author>
+    <x:author>tc={9D3501BC-A500-CE84-B5E6-E155A39BAB9B}</x:author>
+    <x:author>tc={783D909C-6D29-04BA-2094-3992826C3E41}</x:author>
+    <x:author>tc={AEAB2683-F521-B2EE-C37F-42C87EF94DF3}</x:author>
+    <x:author>tc={52CB55C7-B411-4BEC-7139-D2CD26A500B9}</x:author>
+    <x:author>tc={BFD9E4FB-2E78-F919-6C44-91F1DEA04EAD}</x:author>
+    <x:author>tc={4B0F141B-CB22-4CDB-7485-A13E53E72F8D}</x:author>
+    <x:author>tc={BFE9149C-9576-3BEB-27C2-B3903F2C4F9B}</x:author>
+    <x:author>tc={273D5C2B-4CDD-9FA6-3398-A13DB683C94D}</x:author>
+    <x:author>tc={9784883F-9DF5-7690-A035-85FF5ECED254}</x:author>
+    <x:author>tc={E7286862-FFFD-0B76-4375-E1B8A27D14B7}</x:author>
+    <x:author>tc={04E7811F-A3E7-1812-18AC-7B9233EFED0E}</x:author>
+    <x:author>tc={C8B8C70C-0F71-84B5-6B91-75569FA36493}</x:author>
+    <x:author>tc={053A9B83-8DAB-2260-BF5A-31521075D3AF}</x:author>
+    <x:author>tc={38859312-CD6C-159F-43B0-CD57BCD2F9B8}</x:author>
+    <x:author>tc={56612900-921E-DBCB-4BD7-54BBF74ABF52}</x:author>
+    <x:author>tc={FDF97378-F548-D44C-9439-682243FFD703}</x:author>
+    <x:author>tc={526B1780-94D7-5E9B-3D2A-4631AFB48172}</x:author>
+    <x:author>tc={3DC5ECEF-306C-2BAE-7FB9-63D1A4F9A7C3}</x:author>
+    <x:author>tc={EDC9DB79-09E3-1A57-8367-29F618EE1C00}</x:author>
+    <x:author>tc={63CC1148-0375-81E0-784E-A6C2A93C801C}</x:author>
+    <x:author>tc={35D67AD4-96E3-A164-85EC-4113D7220D7C}</x:author>
+    <x:author>tc={7C5D98EB-F28B-2F48-E724-33FF59A76A1C}</x:author>
+    <x:author>tc={EDEBAD77-9DD8-C6CC-1DAC-1078DBA43048}</x:author>
+    <x:author>tc={FAAA3689-5021-D3F6-C1D3-F9E3A3FBD8A4}</x:author>
+    <x:author>tc={F8AD885E-FEB0-BDD4-247B-B4C5B4E0D0D9}</x:author>
+    <x:author>tc={513488CD-DA7A-0663-2201-2084B17D22C6}</x:author>
+    <x:author>tc={115E7CF2-DF60-273C-0932-CE8171DA8D79}</x:author>
+    <x:author>tc={64AADA98-73EA-F1F7-55B9-2ABF6E3E0F52}</x:author>
+    <x:author>tc={C93AE36A-4D69-1794-5687-2D1FD1FDA31B}</x:author>
+    <x:author>tc={4D7AD839-4DE1-AB06-946D-2F348A3B1DAA}</x:author>
+    <x:author>tc={1031016E-EC69-58F2-3F88-CE85DA157D24}</x:author>
+    <x:author>tc={5849F2AC-0A3B-9F2E-A1E7-5992A49DE4B0}</x:author>
+    <x:author>tc={9127DDB2-4E9F-3B47-D25E-FFE4FAF7F457}</x:author>
+    <x:author>tc={F50EBB24-CA8D-6B51-0A65-774249D47C9E}</x:author>
+    <x:author>tc={D0F541E5-408C-CE81-2EB1-3BEEB8A77847}</x:author>
+    <x:author>tc={E37EFC61-5447-9F9C-7B5E-FEA801F1E211}</x:author>
+    <x:author>tc={48FB6D04-A282-3ABC-20AC-10356AD05BBF}</x:author>
+    <x:author>tc={E226DFA5-0E1C-B8A4-F90C-EABDC1D94ED0}</x:author>
+    <x:author>tc={4B0F2B90-0E46-E722-6CC0-0CE8F6D6CFAF}</x:author>
+    <x:author>tc={19919615-1524-1EC2-4674-E7FF34A68A5A}</x:author>
+    <x:author>tc={AA2DE2F5-D0A2-1725-8BA6-7B4952AF281E}</x:author>
+    <x:author>tc={CA711E05-CDE3-41A6-5A6E-ECAF7A97BAE6}</x:author>
+    <x:author>tc={2963596C-2203-2274-A670-205C6579640E}</x:author>
+    <x:author>tc={F40671F1-F455-6791-FE77-304A0C5E1CC7}</x:author>
+    <x:author>tc={6C590A8A-E99D-75EC-05E2-09DBC3A22200}</x:author>
+    <x:author>tc={D73A24F7-B13A-95CD-0C82-0D67008E1A99}</x:author>
+    <x:author>tc={10BFFEC8-5BDE-B9DD-5B54-7553FB8B90F9}</x:author>
+    <x:author>tc={FA73CF8A-A1AF-B949-D042-1BD8564EA5BA}</x:author>
+    <x:author>tc={626C096F-1A95-4AD0-B5B2-531E101A1D26}</x:author>
+    <x:author>tc={8530A33E-F10F-F115-9A0B-86AE6357F680}</x:author>
+    <x:author>tc={54DDD8BD-37ED-08F8-B317-1FDD96DE29DF}</x:author>
+    <x:author>tc={EDDD8B0C-FADF-F92E-9EC5-8BB3373989A5}</x:author>
+    <x:author>tc={DDB422DA-0EE9-489D-AB13-2E7AC64CA5AA}</x:author>
+    <x:author>tc={6C730BAF-6D04-ABDC-E564-82DECC058B99}</x:author>
+    <x:author>tc={12483A20-F933-9EF7-0180-2190AE789983}</x:author>
+    <x:author>tc={892AC851-0CD4-4741-AFE1-65C9C015CFE1}</x:author>
+    <x:author>tc={4544D647-7CB2-143E-ABC8-0A8B8DBAEC6B}</x:author>
+    <x:author>tc={97A23423-4C9E-6127-30CE-D02ABD0EEE46}</x:author>
+    <x:author>tc={41BB1A98-21A6-0AB9-4F6B-9666F98FDC13}</x:author>
+    <x:author>tc={2DB3DE93-BA2B-1FF8-7606-5E5888241207}</x:author>
+    <x:author>tc={7DD61FDF-6800-155E-7AD7-F4D8FDF44584}</x:author>
+    <x:author>tc={B612BDA3-2957-C11B-1864-83B81372AE5E}</x:author>
+    <x:author>tc={BD68943E-8A6F-FE6A-C0AF-D6A988CF26C9}</x:author>
+    <x:author>tc={3E8211A8-00BD-BD96-075F-2D7E7B35A5E7}</x:author>
+    <x:author>tc={9E8B48B0-45C8-8EB6-3188-B97F2019D711}</x:author>
+    <x:author>tc={91725D02-5D33-3D8A-4BF5-87F90B04DB1C}</x:author>
+    <x:author>tc={43B6808D-EF83-40EA-0766-527F606A7061}</x:author>
+    <x:author>tc={0F374BE8-0F57-F04A-5392-F3B4F67B103D}</x:author>
+    <x:author>tc={7D90E353-4ACE-7E2F-4231-401D01F4599B}</x:author>
+    <x:author>tc={48AB9CC7-2F02-AC73-AE13-2014F18E0B8D}</x:author>
+    <x:author>tc={4F12B842-9FCD-F1E0-1AF4-EEF2E8D2A478}</x:author>
+    <x:author>tc={DE1C148B-43F4-0B5E-6AD1-EA1F5928146F}</x:author>
+    <x:author>tc={AE559F99-B4F9-1A12-086C-1D93807DFDD2}</x:author>
+    <x:author>tc={786A0985-07AF-7396-059E-5426D4D26280}</x:author>
+    <x:author>tc={C71D34D4-97A3-8C9F-CD72-6FAF6F232460}</x:author>
+    <x:author>tc={1F753C0F-C99C-069A-3154-9F653B82545F}</x:author>
+    <x:author>tc={73247C21-669F-ED28-2428-0B10BBDEF920}</x:author>
+    <x:author>tc={4842873A-57B6-5A39-FB1C-088F4EB5E885}</x:author>
+    <x:author>tc={52D9658A-6AD5-097E-974C-90373148BCE1}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1175,26 +1175,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={8812A0C8-AE12-CDC4-6559-5ED2998582C7}</x:author>
-    <x:author>tc={FF227541-2EBA-6C23-20BF-5B28E39E9681}</x:author>
-    <x:author>tc={6DE872F6-CA39-0FC9-7DE8-CCF9546B71E5}</x:author>
-    <x:author>tc={CA7CA3B9-387D-9A7E-E5BD-07FB06E11781}</x:author>
-    <x:author>tc={CB8B831A-CE11-2600-48F0-6351067797E4}</x:author>
-    <x:author>tc={C9E6A202-F5C7-C993-DCDC-007DFBA7BEA6}</x:author>
-    <x:author>tc={CDF35263-C850-DFCD-98B8-586343840BE3}</x:author>
-    <x:author>tc={44D94C18-83CB-3B9B-2D29-05BBC1FBF62B}</x:author>
-    <x:author>tc={0B3D40B5-E2AC-994F-57E0-3315321ACDDB}</x:author>
-    <x:author>tc={B2711685-4E1D-9BB8-5657-87F356D886BB}</x:author>
-    <x:author>tc={4E54290C-D4A3-B396-1C0F-2BE4BFF8B4FC}</x:author>
-    <x:author>tc={DA55FDFC-FFC0-B937-406F-09F9817E6A38}</x:author>
-    <x:author>tc={583B0DDD-9F98-5FA2-37E3-5C63FE21466A}</x:author>
-    <x:author>tc={DCC83C46-E129-758A-352E-069886DF1D30}</x:author>
-    <x:author>tc={E41433D0-30E7-C9AD-5360-E0480823C874}</x:author>
-    <x:author>tc={74CC3BFD-C520-7302-3AA5-63E435AA8BF1}</x:author>
-    <x:author>tc={22072459-F97F-B746-085E-C1638D4655EB}</x:author>
-    <x:author>tc={C4E12AE5-C49C-C348-687A-9FF2BF406408}</x:author>
-    <x:author>tc={29DD92EC-6D8D-4931-C0AC-C83AA74C94FE}</x:author>
-    <x:author>tc={37F22D93-CFD6-BE05-6212-E8097B58D230}</x:author>
+    <x:author>tc={FDECAD22-EABF-9950-F3B0-568ED895D606}</x:author>
+    <x:author>tc={52DEF696-296C-56C3-EBF4-D60CBF9065E1}</x:author>
+    <x:author>tc={06517651-F593-169E-103E-FE9EFCFD8C65}</x:author>
+    <x:author>tc={D78C5F5C-6C3A-3C38-2490-7150707B82A5}</x:author>
+    <x:author>tc={69922CBA-FF6F-D1B8-C13E-A808E3819AE4}</x:author>
+    <x:author>tc={F186F349-7A2D-81AF-79BC-9B687D906C29}</x:author>
+    <x:author>tc={BFCDE376-E9B0-1F1E-6478-8B5616DBF0B2}</x:author>
+    <x:author>tc={A234F373-E1F2-D524-D490-355FF332813B}</x:author>
+    <x:author>tc={EC8D2654-0413-5627-5C86-20C98A8B96B9}</x:author>
+    <x:author>tc={FBF17285-3D1D-1A05-3EA3-15EEEDA91D84}</x:author>
+    <x:author>tc={7755BE64-3FAD-A0C9-8423-BC69B057B0AD}</x:author>
+    <x:author>tc={989F5CBD-3C93-4F19-5827-DA026A80655A}</x:author>
+    <x:author>tc={1B746040-AD86-C505-EBEF-908BAFE29A8B}</x:author>
+    <x:author>tc={9A0D7E97-6B1A-82B0-3D4E-805A4B7275CF}</x:author>
+    <x:author>tc={6D5BEAAC-D760-FF23-0D33-4EDDDA1AF04E}</x:author>
+    <x:author>tc={E4073DD0-238C-4811-FF2E-C69DD5E485B8}</x:author>
+    <x:author>tc={CB642E2C-5B8F-F05C-B68F-B944BA6BD445}</x:author>
+    <x:author>tc={F2DC5096-2FB2-2BCB-A6D5-D5EE178CD1D9}</x:author>
+    <x:author>tc={1676377A-CBA1-47E4-0084-0969CA1E87C0}</x:author>
+    <x:author>tc={2F20AB08-3138-AE31-6FB1-28B40662FC41}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2037,7 +2037,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R23e26fa3f9f945d1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2126ecb792d2492b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2048,7 +2048,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}"/>
 </xltc:personList>
 </file>
 
@@ -2245,493 +2245,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-12T20:51:37.472" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{2E92C6EB-E2D8-BFDA-3FFB-FFE8C919781C}">
+  <xltc:threadedComment ref="P5" dT="2026-08-13T06:21:04.91" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{EE808468-1A8F-6BF2-A061-4A7638F69B4F}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-12T20:51:37.484" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{9996CDE2-D7F4-241B-DFFA-F4D42D8806B1}">
+  <xltc:threadedComment ref="P6" dT="2026-08-13T06:21:04.918" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{6E34D41F-1133-57CD-4563-EF7A95211AD1}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-12T20:51:37.484" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{69DC4563-C2A0-EF5E-09E6-5E87691F837D}">
+  <xltc:threadedComment ref="P7" dT="2026-08-13T06:21:04.918" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{9FB4D332-049B-3B73-FC58-DC11CBCB6572}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-12T20:51:37.484" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FF1A8A11-134D-C38D-8DB5-E9C4D1C91AD5}">
+  <xltc:threadedComment ref="P8" dT="2026-08-13T06:21:04.919" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{9D3501BC-A500-CE84-B5E6-E155A39BAB9B}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-12T20:51:37.484" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{EA8BE9CD-E745-69B6-0CDE-1DBF7788ACA3}">
+  <xltc:threadedComment ref="P9" dT="2026-08-13T06:21:04.919" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{783D909C-6D29-04BA-2094-3992826C3E41}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-12T20:51:37.485" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{9112B102-4421-CD24-704F-50C3393D092E}">
+  <xltc:threadedComment ref="P10" dT="2026-08-13T06:21:04.919" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{AEAB2683-F521-B2EE-C37F-42C87EF94DF3}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-12T20:51:37.485" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7386AD46-E177-EAF6-158B-6EB952819DA5}">
+  <xltc:threadedComment ref="P11" dT="2026-08-13T06:21:04.919" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{52CB55C7-B411-4BEC-7139-D2CD26A500B9}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-12T20:51:37.485" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{03678F6D-9AE2-D0F2-43D1-F62224D8F251}">
+  <xltc:threadedComment ref="P12" dT="2026-08-13T06:21:04.919" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{BFD9E4FB-2E78-F919-6C44-91F1DEA04EAD}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-12T20:51:37.485" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{3028E4BF-4DB9-7B67-D957-2AD9FF0DB62C}">
+  <xltc:threadedComment ref="P13" dT="2026-08-13T06:21:04.919" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{4B0F141B-CB22-4CDB-7485-A13E53E72F8D}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FD880EAB-91D0-0E6E-801C-B75442FA218C}">
+  <xltc:threadedComment ref="P14" dT="2026-08-13T06:21:04.92" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{BFE9149C-9576-3BEB-27C2-B3903F2C4F9B}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{638261E2-D0D3-145A-FCDE-93F77D04A644}">
+  <xltc:threadedComment ref="P15" dT="2026-08-13T06:21:04.92" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{273D5C2B-4CDD-9FA6-3398-A13DB683C94D}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{881DE873-A154-A8D5-B621-A50E6FD4CEAD}">
+  <xltc:threadedComment ref="P16" dT="2026-08-13T06:21:04.92" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{9784883F-9DF5-7690-A035-85FF5ECED254}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{9CB972C8-2825-D061-D42D-EB50B2E674C2}">
+  <xltc:threadedComment ref="P17" dT="2026-08-13T06:21:04.92" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{E7286862-FFFD-0B76-4375-E1B8A27D14B7}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{DB8F07C9-F7F7-FE73-9AA9-4C295B9B23EB}">
+  <xltc:threadedComment ref="P18" dT="2026-08-13T06:21:04.92" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{04E7811F-A3E7-1812-18AC-7B9233EFED0E}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7B44EA3A-3423-C44B-17E3-6D0080C46F05}">
+  <xltc:threadedComment ref="P19" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{C8B8C70C-0F71-84B5-6B91-75569FA36493}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{4954549F-3C47-FC30-5755-EE5CE0B1AB51}">
+  <xltc:threadedComment ref="P20" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{053A9B83-8DAB-2260-BF5A-31521075D3AF}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{8404FF8A-6FCC-C393-80A0-6D6067BC4469}">
+  <xltc:threadedComment ref="P21" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{38859312-CD6C-159F-43B0-CD57BCD2F9B8}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C87DDDBD-70BD-3F5F-3775-4FB9E051071A}">
+  <xltc:threadedComment ref="P22" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{56612900-921E-DBCB-4BD7-54BBF74ABF52}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{43AC33EC-4AC1-7B72-3678-E9AF3E6C0947}">
+  <xltc:threadedComment ref="P23" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{FDF97378-F548-D44C-9439-682243FFD703}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{D056F8AD-8D62-71DB-77C6-7D348E118036}">
+  <xltc:threadedComment ref="P24" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{526B1780-94D7-5E9B-3D2A-4631AFB48172}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{D9B69C3A-2770-73F9-D4CF-BF9B35B56E67}">
+  <xltc:threadedComment ref="P25" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{3DC5ECEF-306C-2BAE-7FB9-63D1A4F9A7C3}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-12T20:51:37.486" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7266B7B5-E168-4A57-FF19-4DFFCA6F6429}">
+  <xltc:threadedComment ref="P26" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{EDC9DB79-09E3-1A57-8367-29F618EE1C00}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BC835D1B-78AB-F8B6-7665-58CF307B8CBD}">
+  <xltc:threadedComment ref="P27" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{63CC1148-0375-81E0-784E-A6C2A93C801C}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B3C562D9-57EF-1A70-F0B0-C9ED2533183A}">
+  <xltc:threadedComment ref="P28" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{35D67AD4-96E3-A164-85EC-4113D7220D7C}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{15E9E26E-BDFC-A1A7-B42D-11B46DC791D9}">
+  <xltc:threadedComment ref="P29" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{7C5D98EB-F28B-2F48-E724-33FF59A76A1C}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{F41AD288-E4D5-652C-F9ED-09E5CBA414F4}">
+  <xltc:threadedComment ref="P30" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{EDEBAD77-9DD8-C6CC-1DAC-1078DBA43048}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{54ACF17B-CCA7-F56F-1606-F13A0C880FB9}">
+  <xltc:threadedComment ref="P31" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{FAAA3689-5021-D3F6-C1D3-F9E3A3FBD8A4}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{106CDE0D-0847-8774-3A88-7967F6FEFBF5}">
+  <xltc:threadedComment ref="P32" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{F8AD885E-FEB0-BDD4-247B-B4C5B4E0D0D9}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{E4A9B24A-2E53-E635-0FD1-86B1E7B4D4FC}">
+  <xltc:threadedComment ref="P33" dT="2026-08-13T06:21:04.921" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{513488CD-DA7A-0663-2201-2084B17D22C6}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{6744C604-48FA-71F0-0984-3B0C76DF0FCF}">
+  <xltc:threadedComment ref="P34" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{115E7CF2-DF60-273C-0932-CE8171DA8D79}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{5D9FC781-90BA-3859-6F84-328CAEB64272}">
+  <xltc:threadedComment ref="P35" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{64AADA98-73EA-F1F7-55B9-2ABF6E3E0F52}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B7538A62-EED4-E0E2-C67B-592CD2DA0EAC}">
+  <xltc:threadedComment ref="P36" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{C93AE36A-4D69-1794-5687-2D1FD1FDA31B}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{734EE82A-EC02-AC53-6229-5EB357680EF6}">
+  <xltc:threadedComment ref="P37" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{4D7AD839-4DE1-AB06-946D-2F348A3B1DAA}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{2449F982-692F-3693-49FB-AC235D7CF5FF}">
+  <xltc:threadedComment ref="P38" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{1031016E-EC69-58F2-3F88-CE85DA157D24}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{02F9064B-60A6-572B-3507-D60BCDE6CE0D}">
+  <xltc:threadedComment ref="P39" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{5849F2AC-0A3B-9F2E-A1E7-5992A49DE4B0}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BE555562-4937-00C3-67AF-22CB735AE30A}">
+  <xltc:threadedComment ref="P40" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{9127DDB2-4E9F-3B47-D25E-FFE4FAF7F457}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{2D48255E-57E9-A21E-E862-5B16DA725673}">
+  <xltc:threadedComment ref="P41" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{F50EBB24-CA8D-6B51-0A65-774249D47C9E}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BF4A3063-2BA5-12E8-4DE1-94E638E86565}">
+  <xltc:threadedComment ref="P42" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{D0F541E5-408C-CE81-2EB1-3BEEB8A77847}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{339D2B45-F391-AD3F-9928-68F2417BA655}">
+  <xltc:threadedComment ref="P43" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{E37EFC61-5447-9F9C-7B5E-FEA801F1E211}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FE419763-CFB1-9E71-B022-6BFB85067D47}">
+  <xltc:threadedComment ref="P44" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{48FB6D04-A282-3ABC-20AC-10356AD05BBF}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{33C5D95A-DFC4-9AEF-3518-07183671F73B}">
+  <xltc:threadedComment ref="P45" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{E226DFA5-0E1C-B8A4-F90C-EABDC1D94ED0}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-12T20:51:37.487" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{23880101-D8FB-6F6B-00C1-B84E43313AE5}">
+  <xltc:threadedComment ref="P46" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{4B0F2B90-0E46-E722-6CC0-0CE8F6D6CFAF}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BB5FAFEA-EF75-8EFF-94A2-FAB3033B9471}">
+  <xltc:threadedComment ref="P47" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{19919615-1524-1EC2-4674-E7FF34A68A5A}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{0038C068-A2EF-FD32-47D0-82185638F797}">
+  <xltc:threadedComment ref="P48" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{AA2DE2F5-D0A2-1725-8BA6-7B4952AF281E}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A0397957-B818-A5A2-6206-70C445C43FD0}">
+  <xltc:threadedComment ref="P49" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{CA711E05-CDE3-41A6-5A6E-ECAF7A97BAE6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A396B3E0-3A78-1A9C-4BB6-1C7265D008EC}">
+  <xltc:threadedComment ref="P50" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{2963596C-2203-2274-A670-205C6579640E}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{92EB273B-9878-A3EF-23CB-31CA5D97583F}">
+  <xltc:threadedComment ref="P51" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{F40671F1-F455-6791-FE77-304A0C5E1CC7}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{9B29E06A-F146-42D1-9431-2F1B83073011}">
+  <xltc:threadedComment ref="P52" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{6C590A8A-E99D-75EC-05E2-09DBC3A22200}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A6A30EF1-3BD8-AE42-4ADC-3E139B8D75CB}">
+  <xltc:threadedComment ref="P53" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{D73A24F7-B13A-95CD-0C82-0D67008E1A99}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C779C7F9-D99C-2006-AC15-975B5210F958}">
+  <xltc:threadedComment ref="P54" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{10BFFEC8-5BDE-B9DD-5B54-7553FB8B90F9}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A25459FF-4404-A5D9-9C6A-981C855D41B4}">
+  <xltc:threadedComment ref="P55" dT="2026-08-13T06:21:04.922" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{FA73CF8A-A1AF-B949-D042-1BD8564EA5BA}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{CD5CFED8-5444-8040-5FE5-40D1BFCFCDEA}">
+  <xltc:threadedComment ref="P56" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{626C096F-1A95-4AD0-B5B2-531E101A1D26}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{011BE363-BC65-1234-80BD-35C095BA9EA8}">
+  <xltc:threadedComment ref="P57" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{8530A33E-F10F-F115-9A0B-86AE6357F680}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{489756A7-607C-E95E-93FA-958ECFD99B77}">
+  <xltc:threadedComment ref="P58" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{54DDD8BD-37ED-08F8-B317-1FDD96DE29DF}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{3110FEFE-CFCC-6E61-2F84-E3010F2A2E56}">
+  <xltc:threadedComment ref="P59" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{EDDD8B0C-FADF-F92E-9EC5-8BB3373989A5}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{11AEAC18-8255-69B8-C307-F3A8EC597CBB}">
+  <xltc:threadedComment ref="P60" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{DDB422DA-0EE9-489D-AB13-2E7AC64CA5AA}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7E257C73-E64C-C310-0726-0CC995D04D73}">
+  <xltc:threadedComment ref="P61" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{6C730BAF-6D04-ABDC-E564-82DECC058B99}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{A26BBA99-261D-A8C1-1C19-3B6C23781518}">
+  <xltc:threadedComment ref="P62" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{12483A20-F933-9EF7-0180-2190AE789983}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{42C4F2D4-D997-8E25-DBF5-E416D13982E9}">
+  <xltc:threadedComment ref="P63" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{892AC851-0CD4-4741-AFE1-65C9C015CFE1}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{0200DEEE-8DDD-F98D-D75B-354DA4F82D96}">
+  <xltc:threadedComment ref="P64" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{4544D647-7CB2-143E-ABC8-0A8B8DBAEC6B}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C8BD88E9-9304-50E3-8E16-D6C55A85D82F}">
+  <xltc:threadedComment ref="P65" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{97A23423-4C9E-6127-30CE-D02ABD0EEE46}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{6D8D1C81-76D3-7096-11BA-5A5EC67B2A6A}">
+  <xltc:threadedComment ref="P66" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{41BB1A98-21A6-0AB9-4F6B-9666F98FDC13}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{31BD5FE4-E91C-E52C-7DE9-DC8E66E74B66}">
+  <xltc:threadedComment ref="P67" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{2DB3DE93-BA2B-1FF8-7606-5E5888241207}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B8746BCC-7A92-5A75-D95A-97D8AFB392FD}">
+  <xltc:threadedComment ref="P68" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{7DD61FDF-6800-155E-7AD7-F4D8FDF44584}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{AE775D8D-A6BF-AD24-E330-D32376FC9EFF}">
+  <xltc:threadedComment ref="P69" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{B612BDA3-2957-C11B-1864-83B81372AE5E}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{097E4B9D-D491-0EE3-2052-ACEAFB247869}">
+  <xltc:threadedComment ref="P70" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{BD68943E-8A6F-FE6A-C0AF-D6A988CF26C9}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-12T20:51:37.488" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BAB54389-08BB-FCB3-FA4E-D008BD27EF98}">
+  <xltc:threadedComment ref="P71" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{3E8211A8-00BD-BD96-075F-2D7E7B35A5E7}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B6EB26F3-1F85-E7B1-0864-D3DE48E3B21F}">
+  <xltc:threadedComment ref="P72" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{9E8B48B0-45C8-8EB6-3188-B97F2019D711}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{019F2DF5-928D-1D4C-DE17-4E340A98EF86}">
+  <xltc:threadedComment ref="P73" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{91725D02-5D33-3D8A-4BF5-87F90B04DB1C}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{99DC1528-B916-6FB8-3288-9715AE9DD2B9}">
+  <xltc:threadedComment ref="P74" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{43B6808D-EF83-40EA-0766-527F606A7061}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{1DE7D797-4DF6-30EA-56A0-7F11E54456D2}">
+  <xltc:threadedComment ref="P75" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{0F374BE8-0F57-F04A-5392-F3B4F67B103D}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{3111A50E-EAEE-E93F-39D6-3C3749F5171B}">
+  <xltc:threadedComment ref="P76" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{7D90E353-4ACE-7E2F-4231-401D01F4599B}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{BAEBA302-ADD3-AE44-452C-C97146616383}">
+  <xltc:threadedComment ref="P77" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{48AB9CC7-2F02-AC73-AE13-2014F18E0B8D}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{5C0FBD2A-5940-3C5D-2C6B-542E0F6BB157}">
+  <xltc:threadedComment ref="P78" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{4F12B842-9FCD-F1E0-1AF4-EEF2E8D2A478}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{79C20CC6-A9AC-211C-F83E-1635C7DAC3E4}">
+  <xltc:threadedComment ref="P79" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{DE1C148B-43F4-0B5E-6AD1-EA1F5928146F}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{64B0F472-67A6-40C1-30B0-8CE7DFC47D2A}">
+  <xltc:threadedComment ref="P80" dT="2026-08-13T06:21:04.923" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{AE559F99-B4F9-1A12-086C-1D93807DFDD2}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{1D13A87F-E7F0-347E-6024-33FE60195697}">
+  <xltc:threadedComment ref="P81" dT="2026-08-13T06:21:04.924" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{786A0985-07AF-7396-059E-5426D4D26280}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-12T20:51:37.489" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{3147F0B5-2D94-55A9-492D-95CBAA3E40C1}">
+  <xltc:threadedComment ref="P82" dT="2026-08-13T06:21:04.924" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{C71D34D4-97A3-8C9F-CD72-6FAF6F232460}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-12T20:51:37.49" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FF7CAD37-5E80-7B10-8138-128DF1E42913}">
+  <xltc:threadedComment ref="P83" dT="2026-08-13T06:21:04.924" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{1F753C0F-C99C-069A-3154-9F653B82545F}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-12T20:51:37.49" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{E5B395E6-BE93-46DB-6176-E9240DBE5FA7}">
+  <xltc:threadedComment ref="P84" dT="2026-08-13T06:21:04.924" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{73247C21-669F-ED28-2428-0B10BBDEF920}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-12T20:51:37.49" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{7A281728-42ED-41E8-0344-E95F40D4E6E1}">
+  <xltc:threadedComment ref="P85" dT="2026-08-13T06:21:04.924" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{4842873A-57B6-5A39-FB1C-088F4EB5E885}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-12T20:51:37.49" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{E92CF26C-E2E0-4E74-967C-976222B2ED8D}">
+  <xltc:threadedComment ref="P86" dT="2026-08-13T06:21:04.924" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{52D9658A-6AD5-097E-974C-90373148BCE1}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2742,64 +2742,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-12T20:51:38.167" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{8812A0C8-AE12-CDC4-6559-5ED2998582C7}">
+  <xltc:threadedComment ref="J5" dT="2026-08-13T06:21:05.387" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{FDECAD22-EABF-9950-F3B0-568ED895D606}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-12T20:51:38.172" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{FF227541-2EBA-6C23-20BF-5B28E39E9681}">
+  <xltc:threadedComment ref="J6" dT="2026-08-13T06:21:05.392" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{52DEF696-296C-56C3-EBF4-D60CBF9065E1}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-12T20:51:38.176" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{6DE872F6-CA39-0FC9-7DE8-CCF9546B71E5}">
+  <xltc:threadedComment ref="J7" dT="2026-08-13T06:21:05.396" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{06517651-F593-169E-103E-FE9EFCFD8C65}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-12T20:51:38.181" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{CA7CA3B9-387D-9A7E-E5BD-07FB06E11781}">
+  <xltc:threadedComment ref="J8" dT="2026-08-13T06:21:05.401" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{D78C5F5C-6C3A-3C38-2490-7150707B82A5}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-12T20:51:38.185" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{CB8B831A-CE11-2600-48F0-6351067797E4}">
+  <xltc:threadedComment ref="J9" dT="2026-08-13T06:21:05.405" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{69922CBA-FF6F-D1B8-C13E-A808E3819AE4}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-12T20:51:38.189" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C9E6A202-F5C7-C993-DCDC-007DFBA7BEA6}">
+  <xltc:threadedComment ref="J10" dT="2026-08-13T06:21:05.408" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{F186F349-7A2D-81AF-79BC-9B687D906C29}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-12T20:51:38.194" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{CDF35263-C850-DFCD-98B8-586343840BE3}">
+  <xltc:threadedComment ref="J11" dT="2026-08-13T06:21:05.412" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{BFCDE376-E9B0-1F1E-6478-8B5616DBF0B2}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-12T20:51:38.199" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{44D94C18-83CB-3B9B-2D29-05BBC1FBF62B}">
+  <xltc:threadedComment ref="J12" dT="2026-08-13T06:21:05.417" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{A234F373-E1F2-D524-D490-355FF332813B}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-12T20:51:38.204" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{0B3D40B5-E2AC-994F-57E0-3315321ACDDB}">
+  <xltc:threadedComment ref="J13" dT="2026-08-13T06:21:05.421" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{EC8D2654-0413-5627-5C86-20C98A8B96B9}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-12T20:51:38.209" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{B2711685-4E1D-9BB8-5657-87F356D886BB}">
+  <xltc:threadedComment ref="J14" dT="2026-08-13T06:21:05.424" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{FBF17285-3D1D-1A05-3EA3-15EEEDA91D84}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-12T20:51:38.213" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{4E54290C-D4A3-B396-1C0F-2BE4BFF8B4FC}">
+  <xltc:threadedComment ref="J15" dT="2026-08-13T06:21:05.429" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{7755BE64-3FAD-A0C9-8423-BC69B057B0AD}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-12T20:51:38.217" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{DA55FDFC-FFC0-B937-406F-09F9817E6A38}">
+  <xltc:threadedComment ref="J16" dT="2026-08-13T06:21:05.434" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{989F5CBD-3C93-4F19-5827-DA026A80655A}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-12T20:51:38.22" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{583B0DDD-9F98-5FA2-37E3-5C63FE21466A}">
+  <xltc:threadedComment ref="J17" dT="2026-08-13T06:21:05.436" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{1B746040-AD86-C505-EBEF-908BAFE29A8B}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-12T20:51:38.224" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{DCC83C46-E129-758A-352E-069886DF1D30}">
+  <xltc:threadedComment ref="J18" dT="2026-08-13T06:21:05.439" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{9A0D7E97-6B1A-82B0-3D4E-805A4B7275CF}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-12T20:51:38.227" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{E41433D0-30E7-C9AD-5360-E0480823C874}">
+  <xltc:threadedComment ref="J19" dT="2026-08-13T06:21:05.443" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{6D5BEAAC-D760-FF23-0D33-4EDDDA1AF04E}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-12T20:51:38.231" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{74CC3BFD-C520-7302-3AA5-63E435AA8BF1}">
+  <xltc:threadedComment ref="J20" dT="2026-08-13T06:21:05.446" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{E4073DD0-238C-4811-FF2E-C69DD5E485B8}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-12T20:51:38.233" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{22072459-F97F-B746-085E-C1638D4655EB}">
+  <xltc:threadedComment ref="J21" dT="2026-08-13T06:21:05.448" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{CB642E2C-5B8F-F05C-B68F-B944BA6BD445}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-12T20:51:38.238" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{C4E12AE5-C49C-C348-687A-9FF2BF406408}">
+  <xltc:threadedComment ref="J22" dT="2026-08-13T06:21:05.454" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{F2DC5096-2FB2-2BCB-A6D5-D5EE178CD1D9}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-12T20:51:38.242" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{29DD92EC-6D8D-4931-C0AC-C83AA74C94FE}">
+  <xltc:threadedComment ref="J23" dT="2026-08-13T06:21:05.456" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{1676377A-CBA1-47E4-0084-0969CA1E87C0}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-12T20:51:38.246" personId="{02E82BFA-3259-4D8F-88E9-E37EEA3961E4}" id="{37F22D93-CFD6-BE05-6212-E8097B58D230}">
+  <xltc:threadedComment ref="J24" dT="2026-08-13T06:21:05.46" personId="{BF50F089-3CF8-49EE-AFE9-163D5F96598B}" id="{2F20AB08-3138-AE31-6FB1-28B40662FC41}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -7802,7 +7802,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ddb199f43394c37"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc57c013a5f65497a"/>
 </x:worksheet>
 </file>
 
@@ -8862,7 +8862,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16f89965a1d645a4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re00db1f6dc7449de"/>
 </x:worksheet>
 </file>
 
@@ -9941,13 +9941,13 @@
         <x:v>36007930395</x:v>
       </x:c>
       <x:c r="M5" s="60" t="n">
-        <x:v>0.030134294875263184</x:v>
+        <x:v>0.03013429</x:v>
       </x:c>
       <x:c r="N5" s="60" t="n">
-        <x:v>0.07238020756593225</x:v>
+        <x:v>0.07238021</x:v>
       </x:c>
       <x:c r="O5" s="60" t="n">
-        <x:v>0.12612204812470884</x:v>
+        <x:v>0.12612205</x:v>
       </x:c>
       <x:c r="P5" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10003,13 +10003,13 @@
         <x:v>22082831233</x:v>
       </x:c>
       <x:c r="M6" s="60" t="n">
-        <x:v>0.06541508825388861</x:v>
+        <x:v>0.06541509</x:v>
       </x:c>
       <x:c r="N6" s="60" t="n">
-        <x:v>0.16181852087235998</x:v>
+        <x:v>0.16181852</x:v>
       </x:c>
       <x:c r="O6" s="60" t="n">
-        <x:v>0.28037548886802904</x:v>
+        <x:v>0.28037549</x:v>
       </x:c>
       <x:c r="P6" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10065,13 +10065,13 @@
         <x:v>60403577441</x:v>
       </x:c>
       <x:c r="M7" s="60" t="n">
-        <x:v>0.038419949996937</x:v>
+        <x:v>0.03841995</x:v>
       </x:c>
       <x:c r="N7" s="60" t="n">
-        <x:v>0.07981693383189475</x:v>
+        <x:v>0.07981693</x:v>
       </x:c>
       <x:c r="O7" s="60" t="n">
-        <x:v>0.12866368853501123</x:v>
+        <x:v>0.12866369</x:v>
       </x:c>
       <x:c r="P7" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10127,13 +10127,13 @@
         <x:v>47872524086</x:v>
       </x:c>
       <x:c r="M8" s="60" t="n">
-        <x:v>0.04343802090415189</x:v>
+        <x:v>0.04343802</x:v>
       </x:c>
       <x:c r="N8" s="60" t="n">
-        <x:v>0.08703417141853323</x:v>
+        <x:v>0.08703417</x:v>
       </x:c>
       <x:c r="O8" s="60" t="n">
-        <x:v>0.13838916611263669</x:v>
+        <x:v>0.13838917</x:v>
       </x:c>
       <x:c r="P8" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10189,13 +10189,13 @@
         <x:v>64088597983</x:v>
       </x:c>
       <x:c r="M9" s="60" t="n">
-        <x:v>0.03385340235472548</x:v>
+        <x:v>0.0338534</x:v>
       </x:c>
       <x:c r="N9" s="60" t="n">
-        <x:v>0.07618741571166496</x:v>
+        <x:v>0.07618742</x:v>
       </x:c>
       <x:c r="O9" s="60" t="n">
-        <x:v>0.12439649265092252</x:v>
+        <x:v>0.12439649</x:v>
       </x:c>
       <x:c r="P9" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10251,13 +10251,13 @@
         <x:v>31235678739</x:v>
       </x:c>
       <x:c r="M10" s="60" t="n">
-        <x:v>0.06014593280881975</x:v>
+        <x:v>0.06014593</x:v>
       </x:c>
       <x:c r="N10" s="60" t="n">
-        <x:v>0.24354412762620228</x:v>
+        <x:v>0.24354413</x:v>
       </x:c>
       <x:c r="O10" s="60" t="n">
-        <x:v>0.521964619647653</x:v>
+        <x:v>0.52196462</x:v>
       </x:c>
       <x:c r="P10" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10313,13 +10313,13 @@
         <x:v>208847608848</x:v>
       </x:c>
       <x:c r="M11" s="60" t="n">
-        <x:v>0.07977617795324553</x:v>
+        <x:v>0.07977618</x:v>
       </x:c>
       <x:c r="N11" s="60" t="n">
-        <x:v>0.26117009800823665</x:v>
+        <x:v>0.2611701</x:v>
       </x:c>
       <x:c r="O11" s="60" t="n">
-        <x:v>0.545565599026733</x:v>
+        <x:v>0.5455656</x:v>
       </x:c>
       <x:c r="P11" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10375,13 +10375,13 @@
         <x:v>24984685620</x:v>
       </x:c>
       <x:c r="M12" s="60" t="n">
-        <x:v>0.05776215197933541</x:v>
+        <x:v>0.05776215</x:v>
       </x:c>
       <x:c r="N12" s="60" t="n">
-        <x:v>0.23454245186510836</x:v>
+        <x:v>0.23454245</x:v>
       </x:c>
       <x:c r="O12" s="60" t="n">
-        <x:v>0.5397589534307109</x:v>
+        <x:v>0.53975895</x:v>
       </x:c>
       <x:c r="P12" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10437,13 +10437,13 @@
         <x:v>25767187433</x:v>
       </x:c>
       <x:c r="M13" s="60" t="n">
-        <x:v>0.05949732991854441</x:v>
+        <x:v>0.05949733</x:v>
       </x:c>
       <x:c r="N13" s="60" t="n">
-        <x:v>0.24423792550707069</x:v>
+        <x:v>0.24423793</x:v>
       </x:c>
       <x:c r="O13" s="60" t="n">
-        <x:v>0.5416834554041762</x:v>
+        <x:v>0.54168346</x:v>
       </x:c>
       <x:c r="P13" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10499,13 +10499,13 @@
         <x:v>24938791725</x:v>
       </x:c>
       <x:c r="M14" s="60" t="n">
-        <x:v>0.058637885407502484</x:v>
+        <x:v>0.05863789</x:v>
       </x:c>
       <x:c r="N14" s="60" t="n">
-        <x:v>0.24111169077620176</x:v>
+        <x:v>0.24111169</x:v>
       </x:c>
       <x:c r="O14" s="60" t="n">
-        <x:v>0.5318379963652872</x:v>
+        <x:v>0.531838</x:v>
       </x:c>
       <x:c r="P14" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10561,13 +10561,13 @@
         <x:v>154561619771</x:v>
       </x:c>
       <x:c r="M15" s="60" t="n">
-        <x:v>0.05943205340836872</x:v>
+        <x:v>0.05943205</x:v>
       </x:c>
       <x:c r="N15" s="60" t="n">
-        <x:v>0.10071774984639481</x:v>
+        <x:v>0.10071775</x:v>
       </x:c>
       <x:c r="O15" s="60" t="n">
-        <x:v>0.14078205937801608</x:v>
+        <x:v>0.14078206</x:v>
       </x:c>
       <x:c r="P15" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10623,13 +10623,13 @@
         <x:v>73790534040</x:v>
       </x:c>
       <x:c r="M16" s="60" t="n">
-        <x:v>0.11059224180154291</x:v>
+        <x:v>0.11059224</x:v>
       </x:c>
       <x:c r="N16" s="60" t="n">
-        <x:v>0.24147617879804267</x:v>
+        <x:v>0.24147618</x:v>
       </x:c>
       <x:c r="O16" s="60" t="n">
-        <x:v>0.3870340286855654</x:v>
+        <x:v>0.38703403</x:v>
       </x:c>
       <x:c r="P16" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10685,13 +10685,13 @@
         <x:v>124356088867</x:v>
       </x:c>
       <x:c r="M17" s="60" t="n">
-        <x:v>0.07546386226834616</x:v>
+        <x:v>0.07546386</x:v>
       </x:c>
       <x:c r="N17" s="60" t="n">
-        <x:v>0.25988872809161073</x:v>
+        <x:v>0.25988873</x:v>
       </x:c>
       <x:c r="O17" s="60" t="n">
-        <x:v>0.5355914666584228</x:v>
+        <x:v>0.53559147</x:v>
       </x:c>
       <x:c r="P17" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10747,13 +10747,13 @@
         <x:v>112253986260</x:v>
       </x:c>
       <x:c r="M18" s="60" t="n">
-        <x:v>0.021942429535376853</x:v>
+        <x:v>0.02194243</x:v>
       </x:c>
       <x:c r="N18" s="60" t="n">
-        <x:v>0.03723024430613604</x:v>
+        <x:v>0.03723024</x:v>
       </x:c>
       <x:c r="O18" s="60" t="n">
-        <x:v>0.051969500078099216</x:v>
+        <x:v>0.0519695</x:v>
       </x:c>
       <x:c r="P18" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10809,13 +10809,13 @@
         <x:v>13590432589</x:v>
       </x:c>
       <x:c r="M19" s="60" t="n">
-        <x:v>0.11324812098910925</x:v>
+        <x:v>0.11324812</x:v>
       </x:c>
       <x:c r="N19" s="60" t="n">
-        <x:v>0.28674305385473287</x:v>
+        <x:v>0.28674305</x:v>
       </x:c>
       <x:c r="O19" s="60" t="n">
-        <x:v>0.5020732221662244</x:v>
+        <x:v>0.50207322</x:v>
       </x:c>
       <x:c r="P19" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10871,13 +10871,13 @@
         <x:v>68899417238</x:v>
       </x:c>
       <x:c r="M20" s="60" t="n">
-        <x:v>0.0962865404024966</x:v>
+        <x:v>0.09628654</x:v>
       </x:c>
       <x:c r="N20" s="60" t="n">
-        <x:v>0.29000231274421906</x:v>
+        <x:v>0.29000231</x:v>
       </x:c>
       <x:c r="O20" s="60" t="n">
-        <x:v>0.5557109037868515</x:v>
+        <x:v>0.5557109</x:v>
       </x:c>
       <x:c r="P20" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10933,13 +10933,13 @@
         <x:v>62930227771</x:v>
       </x:c>
       <x:c r="M21" s="60" t="n">
-        <x:v>0.09849576320721593</x:v>
+        <x:v>0.09849576</x:v>
       </x:c>
       <x:c r="N21" s="60" t="n">
-        <x:v>0.2899963695316754</x:v>
+        <x:v>0.28999637</x:v>
       </x:c>
       <x:c r="O21" s="60" t="n">
-        <x:v>0.554709480648481</x:v>
+        <x:v>0.55470948</x:v>
       </x:c>
       <x:c r="P21" s="60" t="n">
         <x:v>0.4</x:v>
@@ -10995,13 +10995,13 @@
         <x:v>61919411222</x:v>
       </x:c>
       <x:c r="M22" s="60" t="n">
-        <x:v>0.09928180904833617</x:v>
+        <x:v>0.09928181</x:v>
       </x:c>
       <x:c r="N22" s="60" t="n">
-        <x:v>0.2915493418797914</x:v>
+        <x:v>0.29154934</x:v>
       </x:c>
       <x:c r="O22" s="60" t="n">
-        <x:v>0.5554511809816889</x:v>
+        <x:v>0.55545118</x:v>
       </x:c>
       <x:c r="P22" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11057,13 +11057,13 @@
         <x:v>11617699393</x:v>
       </x:c>
       <x:c r="M23" s="60" t="n">
-        <x:v>0.05985571965676533</x:v>
+        <x:v>0.05985572</x:v>
       </x:c>
       <x:c r="N23" s="60" t="n">
-        <x:v>0.2420929947903187</x:v>
+        <x:v>0.24209299</x:v>
       </x:c>
       <x:c r="O23" s="60" t="n">
-        <x:v>0.5348714544283002</x:v>
+        <x:v>0.53487145</x:v>
       </x:c>
       <x:c r="P23" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11119,13 +11119,13 @@
         <x:v>81350630066</x:v>
       </x:c>
       <x:c r="M24" s="60" t="n">
-        <x:v>0.07732686711121328</x:v>
+        <x:v>0.07732687</x:v>
       </x:c>
       <x:c r="N24" s="60" t="n">
-        <x:v>0.2624638674983691</x:v>
+        <x:v>0.26246387</x:v>
       </x:c>
       <x:c r="O24" s="60" t="n">
-        <x:v>0.5277006362269024</x:v>
+        <x:v>0.52770064</x:v>
       </x:c>
       <x:c r="P24" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11181,13 +11181,13 @@
         <x:v>11223146539</x:v>
       </x:c>
       <x:c r="M25" s="60" t="n">
-        <x:v>0.056313675312609675</x:v>
+        <x:v>0.05631368</x:v>
       </x:c>
       <x:c r="N25" s="60" t="n">
-        <x:v>0.24059547309915366</x:v>
+        <x:v>0.24059547</x:v>
       </x:c>
       <x:c r="O25" s="60" t="n">
-        <x:v>0.5419630766528568</x:v>
+        <x:v>0.54196308</x:v>
       </x:c>
       <x:c r="P25" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11243,13 +11243,13 @@
         <x:v>100955034356</x:v>
       </x:c>
       <x:c r="M26" s="60" t="n">
-        <x:v>0.018583612565157198</x:v>
+        <x:v>0.01858361</x:v>
       </x:c>
       <x:c r="N26" s="60" t="n">
-        <x:v>0.03231816226000572</x:v>
+        <x:v>0.03231816</x:v>
       </x:c>
       <x:c r="O26" s="60" t="n">
-        <x:v>0.046214110002405814</x:v>
+        <x:v>0.04621411</x:v>
       </x:c>
       <x:c r="P26" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11305,13 +11305,13 @@
         <x:v>64068421354</x:v>
       </x:c>
       <x:c r="M27" s="60" t="n">
-        <x:v>0.07937589725048073</x:v>
+        <x:v>0.0793759</x:v>
       </x:c>
       <x:c r="N27" s="60" t="n">
-        <x:v>0.2602087956466014</x:v>
+        <x:v>0.2602088</x:v>
       </x:c>
       <x:c r="O27" s="60" t="n">
-        <x:v>0.5377148369554994</x:v>
+        <x:v>0.53771484</x:v>
       </x:c>
       <x:c r="P27" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11367,13 +11367,13 @@
         <x:v>119532978629</x:v>
       </x:c>
       <x:c r="M28" s="60" t="n">
-        <x:v>0.05969403431878323</x:v>
+        <x:v>0.05969403</x:v>
       </x:c>
       <x:c r="N28" s="60" t="n">
-        <x:v>0.10475196614457755</x:v>
+        <x:v>0.10475197</x:v>
       </x:c>
       <x:c r="O28" s="60" t="n">
-        <x:v>0.1488173286601695</x:v>
+        <x:v>0.14881733</x:v>
       </x:c>
       <x:c r="P28" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11429,13 +11429,13 @@
         <x:v>8828885285</x:v>
       </x:c>
       <x:c r="M29" s="60" t="n">
-        <x:v>0.058409851049309694</x:v>
+        <x:v>0.05840985</x:v>
       </x:c>
       <x:c r="N29" s="60" t="n">
-        <x:v>0.24149939945983706</x:v>
+        <x:v>0.2414994</x:v>
       </x:c>
       <x:c r="O29" s="60" t="n">
-        <x:v>0.5285982315666717</x:v>
+        <x:v>0.52859823</x:v>
       </x:c>
       <x:c r="P29" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11491,13 +11491,13 @@
         <x:v>8939727305</x:v>
       </x:c>
       <x:c r="M30" s="60" t="n">
-        <x:v>0.05955693073196007</x:v>
+        <x:v>0.05955693</x:v>
       </x:c>
       <x:c r="N30" s="60" t="n">
-        <x:v>0.24527883857659377</x:v>
+        <x:v>0.24527884</x:v>
       </x:c>
       <x:c r="O30" s="60" t="n">
-        <x:v>0.5361144682980558</x:v>
+        <x:v>0.53611447</x:v>
       </x:c>
       <x:c r="P30" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11553,13 +11553,13 @@
         <x:v>49499679772</x:v>
       </x:c>
       <x:c r="M31" s="60" t="n">
-        <x:v>0.07443905302382356</x:v>
+        <x:v>0.07443905</x:v>
       </x:c>
       <x:c r="N31" s="60" t="n">
-        <x:v>0.25456097259688826</x:v>
+        <x:v>0.25456097</x:v>
       </x:c>
       <x:c r="O31" s="60" t="n">
-        <x:v>0.534597764512135</x:v>
+        <x:v>0.53459776</x:v>
       </x:c>
       <x:c r="P31" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11615,13 +11615,13 @@
         <x:v>29619077437</x:v>
       </x:c>
       <x:c r="M32" s="60" t="n">
-        <x:v>0.09788479216134033</x:v>
+        <x:v>0.09788479</x:v>
       </x:c>
       <x:c r="N32" s="60" t="n">
-        <x:v>0.2876394254770833</x:v>
+        <x:v>0.28763943</x:v>
       </x:c>
       <x:c r="O32" s="60" t="n">
-        <x:v>0.5509663784985583</x:v>
+        <x:v>0.55096638</x:v>
       </x:c>
       <x:c r="P32" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11677,13 +11677,13 @@
         <x:v>28407204976</x:v>
       </x:c>
       <x:c r="M33" s="60" t="n">
-        <x:v>0.09358920236601843</x:v>
+        <x:v>0.0935892</x:v>
       </x:c>
       <x:c r="N33" s="60" t="n">
-        <x:v>0.28581012236559156</x:v>
+        <x:v>0.28581012</x:v>
       </x:c>
       <x:c r="O33" s="60" t="n">
-        <x:v>0.5519850300258929</x:v>
+        <x:v>0.55198503</x:v>
       </x:c>
       <x:c r="P33" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11739,13 +11739,13 @@
         <x:v>85097319344</x:v>
       </x:c>
       <x:c r="M34" s="60" t="n">
-        <x:v>0.08999013570952864</x:v>
+        <x:v>0.08999014</x:v>
       </x:c>
       <x:c r="N34" s="60" t="n">
-        <x:v>0.15765592780605325</x:v>
+        <x:v>0.15765593</x:v>
       </x:c>
       <x:c r="O34" s="60" t="n">
-        <x:v>0.2247568909146233</x:v>
+        <x:v>0.22475689</x:v>
       </x:c>
       <x:c r="P34" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11801,13 +11801,13 @@
         <x:v>44181193145</x:v>
       </x:c>
       <x:c r="M35" s="60" t="n">
-        <x:v>0.06051206514669652</x:v>
+        <x:v>0.06051207</x:v>
       </x:c>
       <x:c r="N35" s="60" t="n">
-        <x:v>0.10234613516033039</x:v>
+        <x:v>0.10234614</x:v>
       </x:c>
       <x:c r="O35" s="60" t="n">
-        <x:v>0.14473928734345573</x:v>
+        <x:v>0.14473929</x:v>
       </x:c>
       <x:c r="P35" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11863,13 +11863,13 @@
         <x:v>21392587725</x:v>
       </x:c>
       <x:c r="M36" s="60" t="n">
-        <x:v>0.09588890212185046</x:v>
+        <x:v>0.0958889</x:v>
       </x:c>
       <x:c r="N36" s="60" t="n">
-        <x:v>0.28617687127903557</x:v>
+        <x:v>0.28617687</x:v>
       </x:c>
       <x:c r="O36" s="60" t="n">
-        <x:v>0.5497858324665961</x:v>
+        <x:v>0.54978583</x:v>
       </x:c>
       <x:c r="P36" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11925,13 +11925,13 @@
         <x:v>27319764777</x:v>
       </x:c>
       <x:c r="M37" s="60" t="n">
-        <x:v>0.08464713777906621</x:v>
+        <x:v>0.08464714</x:v>
       </x:c>
       <x:c r="N37" s="60" t="n">
-        <x:v>0.26470646953583726</x:v>
+        <x:v>0.26470647</x:v>
       </x:c>
       <x:c r="O37" s="60" t="n">
-        <x:v>0.5494413066996752</x:v>
+        <x:v>0.54944131</x:v>
       </x:c>
       <x:c r="P37" s="60" t="n">
         <x:v>0.4</x:v>
@@ -11987,13 +11987,13 @@
         <x:v>20249719379</x:v>
       </x:c>
       <x:c r="M38" s="60" t="n">
-        <x:v>0.0973490046077004</x:v>
+        <x:v>0.097349</x:v>
       </x:c>
       <x:c r="N38" s="60" t="n">
-        <x:v>0.28796164226136867</x:v>
+        <x:v>0.28796164</x:v>
       </x:c>
       <x:c r="O38" s="60" t="n">
-        <x:v>0.5490990866748383</x:v>
+        <x:v>0.54909909</x:v>
       </x:c>
       <x:c r="P38" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12049,13 +12049,13 @@
         <x:v>20831129580</x:v>
       </x:c>
       <x:c r="M39" s="60" t="n">
-        <x:v>0.16069402522965945</x:v>
+        <x:v>0.16069403</x:v>
       </x:c>
       <x:c r="N39" s="60" t="n">
-        <x:v>0.3259255889225109</x:v>
+        <x:v>0.32592559</x:v>
       </x:c>
       <x:c r="O39" s="60" t="n">
-        <x:v>0.5122228847542915</x:v>
+        <x:v>0.51222288</x:v>
       </x:c>
       <x:c r="P39" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12111,13 +12111,13 @@
         <x:v>16776074399</x:v>
       </x:c>
       <x:c r="M40" s="60" t="n">
-        <x:v>0.09609473124024975</x:v>
+        <x:v>0.09609473</x:v>
       </x:c>
       <x:c r="N40" s="60" t="n">
-        <x:v>0.2864980171144463</x:v>
+        <x:v>0.28649802</x:v>
       </x:c>
       <x:c r="O40" s="60" t="n">
-        <x:v>0.5514789297074226</x:v>
+        <x:v>0.55147893</x:v>
       </x:c>
       <x:c r="P40" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12173,13 +12173,13 @@
         <x:v>2918062912</x:v>
       </x:c>
       <x:c r="M41" s="60" t="n">
-        <x:v>0.06193796359710312</x:v>
+        <x:v>0.06193796</x:v>
       </x:c>
       <x:c r="N41" s="60" t="n">
-        <x:v>0.2386824603951777</x:v>
+        <x:v>0.23868246</x:v>
       </x:c>
       <x:c r="O41" s="60" t="n">
-        <x:v>0.5358074509590197</x:v>
+        <x:v>0.53580745</x:v>
       </x:c>
       <x:c r="P41" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12235,13 +12235,13 @@
         <x:v>20781851793</x:v>
       </x:c>
       <x:c r="M42" s="60" t="n">
-        <x:v>0.08308753941778212</x:v>
+        <x:v>0.08308754</x:v>
       </x:c>
       <x:c r="N42" s="60" t="n">
-        <x:v>0.26280062172465923</x:v>
+        <x:v>0.26280062</x:v>
       </x:c>
       <x:c r="O42" s="60" t="n">
-        <x:v>0.534367325286259</x:v>
+        <x:v>0.53436733</x:v>
       </x:c>
       <x:c r="P42" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12297,13 +12297,13 @@
         <x:v>14012127540</x:v>
       </x:c>
       <x:c r="M43" s="60" t="n">
-        <x:v>0.10070981779153078</x:v>
+        <x:v>0.10070982</x:v>
       </x:c>
       <x:c r="N43" s="60" t="n">
-        <x:v>0.28552321102510725</x:v>
+        <x:v>0.28552321</x:v>
       </x:c>
       <x:c r="O43" s="60" t="n">
-        <x:v>0.5513308530335718</x:v>
+        <x:v>0.55133085</x:v>
       </x:c>
       <x:c r="P43" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12359,13 +12359,13 @@
         <x:v>2738548410</x:v>
       </x:c>
       <x:c r="M44" s="60" t="n">
-        <x:v>0.05506137950746095</x:v>
+        <x:v>0.05506138</x:v>
       </x:c>
       <x:c r="N44" s="60" t="n">
-        <x:v>0.23784217760262277</x:v>
+        <x:v>0.23784218</x:v>
       </x:c>
       <x:c r="O44" s="60" t="n">
-        <x:v>0.533056501858706</x:v>
+        <x:v>0.5330565</x:v>
       </x:c>
       <x:c r="P44" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12421,13 +12421,13 @@
         <x:v>172999102460</x:v>
       </x:c>
       <x:c r="M45" s="60" t="n">
-        <x:v>0.13866246874867125</x:v>
+        <x:v>0.13866247</x:v>
       </x:c>
       <x:c r="N45" s="60" t="n">
-        <x:v>0.33307259368392994</x:v>
+        <x:v>0.33307259</x:v>
       </x:c>
       <x:c r="O45" s="60" t="n">
-        <x:v>0.5647985821416962</x:v>
+        <x:v>0.56479858</x:v>
       </x:c>
       <x:c r="P45" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12483,13 +12483,13 @@
         <x:v>11312412585</x:v>
       </x:c>
       <x:c r="M46" s="60" t="n">
-        <x:v>0.10040793964577313</x:v>
+        <x:v>0.10040794</x:v>
       </x:c>
       <x:c r="N46" s="60" t="n">
-        <x:v>0.2923765910104087</x:v>
+        <x:v>0.29237659</x:v>
       </x:c>
       <x:c r="O46" s="60" t="n">
-        <x:v>0.5524678391652019</x:v>
+        <x:v>0.55246784</x:v>
       </x:c>
       <x:c r="P46" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12545,13 +12545,13 @@
         <x:v>10091183456</x:v>
       </x:c>
       <x:c r="M47" s="60" t="n">
-        <x:v>0.099581962112083</x:v>
+        <x:v>0.09958196</x:v>
       </x:c>
       <x:c r="N47" s="60" t="n">
-        <x:v>0.28366209841900714</x:v>
+        <x:v>0.2836621</x:v>
       </x:c>
       <x:c r="O47" s="60" t="n">
-        <x:v>0.5441863244952249</x:v>
+        <x:v>0.54418632</x:v>
       </x:c>
       <x:c r="P47" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12607,13 +12607,13 @@
         <x:v>2113791649</x:v>
       </x:c>
       <x:c r="M48" s="60" t="n">
-        <x:v>0.054583586341939064</x:v>
+        <x:v>0.05458359</x:v>
       </x:c>
       <x:c r="N48" s="60" t="n">
-        <x:v>0.2357478992697174</x:v>
+        <x:v>0.2357479</x:v>
       </x:c>
       <x:c r="O48" s="60" t="n">
-        <x:v>0.5352857454576712</x:v>
+        <x:v>0.53528575</x:v>
       </x:c>
       <x:c r="P48" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12669,13 +12669,13 @@
         <x:v>10429520313</x:v>
       </x:c>
       <x:c r="M49" s="60" t="n">
-        <x:v>0.09511502057993171</x:v>
+        <x:v>0.09511502</x:v>
       </x:c>
       <x:c r="N49" s="60" t="n">
-        <x:v>0.2857789988378556</x:v>
+        <x:v>0.285779</x:v>
       </x:c>
       <x:c r="O49" s="60" t="n">
-        <x:v>0.5457895712121568</x:v>
+        <x:v>0.54578957</x:v>
       </x:c>
       <x:c r="P49" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12731,13 +12731,13 @@
         <x:v>11928787755</x:v>
       </x:c>
       <x:c r="M50" s="60" t="n">
-        <x:v>0.08108214166738825</x:v>
+        <x:v>0.08108214</x:v>
       </x:c>
       <x:c r="N50" s="60" t="n">
-        <x:v>0.25648930068850795</x:v>
+        <x:v>0.2564893</x:v>
       </x:c>
       <x:c r="O50" s="60" t="n">
-        <x:v>0.5498837201019288</x:v>
+        <x:v>0.54988372</x:v>
       </x:c>
       <x:c r="P50" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12793,13 +12793,13 @@
         <x:v>9158314768</x:v>
       </x:c>
       <x:c r="M51" s="60" t="n">
-        <x:v>0.09776475419438205</x:v>
+        <x:v>0.09776475</x:v>
       </x:c>
       <x:c r="N51" s="60" t="n">
-        <x:v>0.28685162365058753</x:v>
+        <x:v>0.28685162</x:v>
       </x:c>
       <x:c r="O51" s="60" t="n">
-        <x:v>0.5454867948521468</x:v>
+        <x:v>0.54548679</x:v>
       </x:c>
       <x:c r="P51" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12855,13 +12855,13 @@
         <x:v>8914172680</x:v>
       </x:c>
       <x:c r="M52" s="60" t="n">
-        <x:v>0.09496885258724332</x:v>
+        <x:v>0.09496885</x:v>
       </x:c>
       <x:c r="N52" s="60" t="n">
-        <x:v>0.285322493614913</x:v>
+        <x:v>0.28532249</x:v>
       </x:c>
       <x:c r="O52" s="60" t="n">
-        <x:v>0.5431960857655815</x:v>
+        <x:v>0.54319609</x:v>
       </x:c>
       <x:c r="P52" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12917,13 +12917,13 @@
         <x:v>11773925269</x:v>
       </x:c>
       <x:c r="M53" s="60" t="n">
-        <x:v>0.08006508379394711</x:v>
+        <x:v>0.08006508</x:v>
       </x:c>
       <x:c r="N53" s="60" t="n">
-        <x:v>0.2649582363131656</x:v>
+        <x:v>0.26495824</x:v>
       </x:c>
       <x:c r="O53" s="60" t="n">
-        <x:v>0.5430307224918198</x:v>
+        <x:v>0.54303072</x:v>
       </x:c>
       <x:c r="P53" s="60" t="n">
         <x:v>0.4</x:v>
@@ -12979,13 +12979,13 @@
         <x:v>10487012703</x:v>
       </x:c>
       <x:c r="M54" s="60" t="n">
-        <x:v>0.08023987743822523</x:v>
+        <x:v>0.08023988</x:v>
       </x:c>
       <x:c r="N54" s="60" t="n">
-        <x:v>0.26388171594627485</x:v>
+        <x:v>0.26388172</x:v>
       </x:c>
       <x:c r="O54" s="60" t="n">
-        <x:v>0.5369831234113577</x:v>
+        <x:v>0.53698312</x:v>
       </x:c>
       <x:c r="P54" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13041,13 +13041,13 @@
         <x:v>1460207145</x:v>
       </x:c>
       <x:c r="M55" s="60" t="n">
-        <x:v>0.05383309475968111</x:v>
+        <x:v>0.05383309</x:v>
       </x:c>
       <x:c r="N55" s="60" t="n">
-        <x:v>0.23750840249088684</x:v>
+        <x:v>0.2375084</x:v>
       </x:c>
       <x:c r="O55" s="60" t="n">
-        <x:v>0.5255678180354886</x:v>
+        <x:v>0.52556782</x:v>
       </x:c>
       <x:c r="P55" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13103,13 +13103,13 @@
         <x:v>96850998232</x:v>
       </x:c>
       <x:c r="M56" s="60" t="n">
-        <x:v>0.13903648695715654</x:v>
+        <x:v>0.13903649</x:v>
       </x:c>
       <x:c r="N56" s="60" t="n">
-        <x:v>0.33030230934152394</x:v>
+        <x:v>0.33030231</x:v>
       </x:c>
       <x:c r="O56" s="60" t="n">
-        <x:v>0.5734305190540189</x:v>
+        <x:v>0.57343052</x:v>
       </x:c>
       <x:c r="P56" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13165,13 +13165,13 @@
         <x:v>9410799984</x:v>
       </x:c>
       <x:c r="M57" s="60" t="n">
-        <x:v>0.07581312531499518</x:v>
+        <x:v>0.07581313</x:v>
       </x:c>
       <x:c r="N57" s="60" t="n">
-        <x:v>0.2634734028334438</x:v>
+        <x:v>0.2634734</x:v>
       </x:c>
       <x:c r="O57" s="60" t="n">
-        <x:v>0.5361753231891423</x:v>
+        <x:v>0.53617532</x:v>
       </x:c>
       <x:c r="P57" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13227,13 +13227,13 @@
         <x:v>1103917081</x:v>
       </x:c>
       <x:c r="M58" s="60" t="n">
-        <x:v>0.057855380491963246</x:v>
+        <x:v>0.05785538</x:v>
       </x:c>
       <x:c r="N58" s="60" t="n">
-        <x:v>0.23593437959771368</x:v>
+        <x:v>0.23593438</x:v>
       </x:c>
       <x:c r="O58" s="60" t="n">
-        <x:v>0.5132550112315675</x:v>
+        <x:v>0.51325501</x:v>
       </x:c>
       <x:c r="P58" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13289,13 +13289,13 @@
         <x:v>61049850573</x:v>
       </x:c>
       <x:c r="M59" s="60" t="n">
-        <x:v>0.1528851295871911</x:v>
+        <x:v>0.15288513</x:v>
       </x:c>
       <x:c r="N59" s="60" t="n">
-        <x:v>0.3508304682231032</x:v>
+        <x:v>0.35083047</x:v>
       </x:c>
       <x:c r="O59" s="60" t="n">
-        <x:v>0.5884701246753423</x:v>
+        <x:v>0.58847012</x:v>
       </x:c>
       <x:c r="P59" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13351,13 +13351,13 @@
         <x:v>65242158433</x:v>
       </x:c>
       <x:c r="M60" s="60" t="n">
-        <x:v>0.1422670100633581</x:v>
+        <x:v>0.14226701</x:v>
       </x:c>
       <x:c r="N60" s="60" t="n">
-        <x:v>0.33239541405034906</x:v>
+        <x:v>0.33239541</x:v>
       </x:c>
       <x:c r="O60" s="60" t="n">
-        <x:v>0.5750923241775993</x:v>
+        <x:v>0.57509232</x:v>
       </x:c>
       <x:c r="P60" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13413,13 +13413,13 @@
         <x:v>765700864</x:v>
       </x:c>
       <x:c r="M61" s="60" t="n">
-        <x:v>0.059276860879407665</x:v>
+        <x:v>0.05927686</x:v>
       </x:c>
       <x:c r="N61" s="60" t="n">
-        <x:v>0.23689455021075811</x:v>
+        <x:v>0.23689455</x:v>
       </x:c>
       <x:c r="O61" s="60" t="n">
-        <x:v>0.5408885511956655</x:v>
+        <x:v>0.54088855</x:v>
       </x:c>
       <x:c r="P61" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13475,13 +13475,13 @@
         <x:v>55401383735</x:v>
       </x:c>
       <x:c r="M62" s="60" t="n">
-        <x:v>0.13635518471395658</x:v>
+        <x:v>0.13635518</x:v>
       </x:c>
       <x:c r="N62" s="60" t="n">
-        <x:v>0.33436877152897193</x:v>
+        <x:v>0.33436877</x:v>
       </x:c>
       <x:c r="O62" s="60" t="n">
-        <x:v>0.5677578177186852</x:v>
+        <x:v>0.56775782</x:v>
       </x:c>
       <x:c r="P62" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13537,13 +13537,13 @@
         <x:v>3198995576</x:v>
       </x:c>
       <x:c r="M63" s="60" t="n">
-        <x:v>0.09480524003647198</x:v>
+        <x:v>0.09480524</x:v>
       </x:c>
       <x:c r="N63" s="60" t="n">
-        <x:v>0.2913873300435798</x:v>
+        <x:v>0.29138733</x:v>
       </x:c>
       <x:c r="O63" s="60" t="n">
-        <x:v>0.5466487965228958</x:v>
+        <x:v>0.5466488</x:v>
       </x:c>
       <x:c r="P63" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13599,13 +13599,13 @@
         <x:v>577410003</x:v>
       </x:c>
       <x:c r="M64" s="60" t="n">
-        <x:v>0.05607169702857174</x:v>
+        <x:v>0.0560717</x:v>
       </x:c>
       <x:c r="N64" s="60" t="n">
-        <x:v>0.23722133099377157</x:v>
+        <x:v>0.23722133</x:v>
       </x:c>
       <x:c r="O64" s="60" t="n">
-        <x:v>0.5244583972908571</x:v>
+        <x:v>0.5244584</x:v>
       </x:c>
       <x:c r="P64" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13661,13 +13661,13 @@
         <x:v>35328834395</x:v>
       </x:c>
       <x:c r="M65" s="60" t="n">
-        <x:v>0.15010291440846113</x:v>
+        <x:v>0.15010291</x:v>
       </x:c>
       <x:c r="N65" s="60" t="n">
-        <x:v>0.3518274421151198</x:v>
+        <x:v>0.35182744</x:v>
       </x:c>
       <x:c r="O65" s="60" t="n">
-        <x:v>0.5925442380352349</x:v>
+        <x:v>0.59254424</x:v>
       </x:c>
       <x:c r="P65" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13723,13 +13723,13 @@
         <x:v>2035738142</x:v>
       </x:c>
       <x:c r="M66" s="60" t="n">
-        <x:v>0.09947819115475738</x:v>
+        <x:v>0.09947819</x:v>
       </x:c>
       <x:c r="N66" s="60" t="n">
-        <x:v>0.28407130733134695</x:v>
+        <x:v>0.28407131</x:v>
       </x:c>
       <x:c r="O66" s="60" t="n">
-        <x:v>0.548082627060927</x:v>
+        <x:v>0.54808263</x:v>
       </x:c>
       <x:c r="P66" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13785,13 +13785,13 @@
         <x:v>27063204610</x:v>
       </x:c>
       <x:c r="M67" s="60" t="n">
-        <x:v>0.15868408076889853</x:v>
+        <x:v>0.15868408</x:v>
       </x:c>
       <x:c r="N67" s="60" t="n">
-        <x:v>0.3536015207940266</x:v>
+        <x:v>0.35360152</x:v>
       </x:c>
       <x:c r="O67" s="60" t="n">
-        <x:v>0.5943624405430227</x:v>
+        <x:v>0.59436244</x:v>
       </x:c>
       <x:c r="P67" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13847,13 +13847,13 @@
         <x:v>24232970803</x:v>
       </x:c>
       <x:c r="M68" s="60" t="n">
-        <x:v>0.13964481980747906</x:v>
+        <x:v>0.13964482</x:v>
       </x:c>
       <x:c r="N68" s="60" t="n">
-        <x:v>0.32768476341691466</x:v>
+        <x:v>0.32768476</x:v>
       </x:c>
       <x:c r="O68" s="60" t="n">
-        <x:v>0.5749196541449603</x:v>
+        <x:v>0.57491965</x:v>
       </x:c>
       <x:c r="P68" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13909,13 +13909,13 @@
         <x:v>20650381274</x:v>
       </x:c>
       <x:c r="M69" s="60" t="n">
-        <x:v>0.15977295102433106</x:v>
+        <x:v>0.15977295</x:v>
       </x:c>
       <x:c r="N69" s="60" t="n">
-        <x:v>0.3528909487517171</x:v>
+        <x:v>0.35289095</x:v>
       </x:c>
       <x:c r="O69" s="60" t="n">
-        <x:v>0.5845138725922333</x:v>
+        <x:v>0.58451387</x:v>
       </x:c>
       <x:c r="P69" s="60" t="n">
         <x:v>0.4</x:v>
@@ -13971,13 +13971,13 @@
         <x:v>2169197069</x:v>
       </x:c>
       <x:c r="M70" s="60" t="n">
-        <x:v>0.0758911344894779</x:v>
+        <x:v>0.07589113</x:v>
       </x:c>
       <x:c r="N70" s="60" t="n">
-        <x:v>0.2678140585177142</x:v>
+        <x:v>0.26781406</x:v>
       </x:c>
       <x:c r="O70" s="60" t="n">
-        <x:v>0.5390381207397343</x:v>
+        <x:v>0.53903812</x:v>
       </x:c>
       <x:c r="P70" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14033,13 +14033,13 @@
         <x:v>22710386116</x:v>
       </x:c>
       <x:c r="M71" s="60" t="n">
-        <x:v>0.13539688009933706</x:v>
+        <x:v>0.13539688</x:v>
       </x:c>
       <x:c r="N71" s="60" t="n">
-        <x:v>0.3361381692367583</x:v>
+        <x:v>0.33613817</x:v>
       </x:c>
       <x:c r="O71" s="60" t="n">
-        <x:v>0.575412871070798</x:v>
+        <x:v>0.57541287</x:v>
       </x:c>
       <x:c r="P71" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14095,13 +14095,13 @@
         <x:v>16991030080</x:v>
       </x:c>
       <x:c r="M72" s="60" t="n">
-        <x:v>0.15400543383979404</x:v>
+        <x:v>0.15400543</x:v>
       </x:c>
       <x:c r="N72" s="60" t="n">
-        <x:v>0.3495689637575733</x:v>
+        <x:v>0.34956896</x:v>
       </x:c>
       <x:c r="O72" s="60" t="n">
-        <x:v>0.5975412038603469</x:v>
+        <x:v>0.5975412</x:v>
       </x:c>
       <x:c r="P72" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14157,13 +14157,13 @@
         <x:v>18545016584</x:v>
       </x:c>
       <x:c r="M73" s="60" t="n">
-        <x:v>0.13949359754902363</x:v>
+        <x:v>0.1394936</x:v>
       </x:c>
       <x:c r="N73" s="60" t="n">
-        <x:v>0.3311807893340863</x:v>
+        <x:v>0.33118079</x:v>
       </x:c>
       <x:c r="O73" s="60" t="n">
-        <x:v>0.5686223146466987</x:v>
+        <x:v>0.56862231</x:v>
       </x:c>
       <x:c r="P73" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14210,7 +14210,7 @@
         <x:v>111379151</x:v>
       </x:c>
       <x:c r="J74" s="79" t="n">
-        <x:v>201859785</x:v>
+        <x:v>201859786</x:v>
       </x:c>
       <x:c r="K74" s="79" t="n">
         <x:v>391426781</x:v>
@@ -14219,13 +14219,13 @@
         <x:v>1162341739</x:v>
       </x:c>
       <x:c r="M74" s="60" t="n">
-        <x:v>0.09582307233986045</x:v>
+        <x:v>0.09582307</x:v>
       </x:c>
       <x:c r="N74" s="60" t="n">
-        <x:v>0.28454657743398826</x:v>
+        <x:v>0.28454658</x:v>
       </x:c>
       <x:c r="O74" s="60" t="n">
-        <x:v>0.5517649542399158</x:v>
+        <x:v>0.55176495</x:v>
       </x:c>
       <x:c r="P74" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14281,13 +14281,13 @@
         <x:v>1586399985</x:v>
       </x:c>
       <x:c r="M75" s="60" t="n">
-        <x:v>0.07459208118935105</x:v>
+        <x:v>0.07459208</x:v>
       </x:c>
       <x:c r="N75" s="60" t="n">
-        <x:v>0.26124930102084964</x:v>
+        <x:v>0.2612493</x:v>
       </x:c>
       <x:c r="O75" s="60" t="n">
-        <x:v>0.5442902846503808</x:v>
+        <x:v>0.54429028</x:v>
       </x:c>
       <x:c r="P75" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14343,13 +14343,13 @@
         <x:v>1273369030</x:v>
       </x:c>
       <x:c r="M76" s="60" t="n">
-        <x:v>0.0758078773931982</x:v>
+        <x:v>0.07580788</x:v>
       </x:c>
       <x:c r="N76" s="60" t="n">
-        <x:v>0.259219937483861</x:v>
+        <x:v>0.25921994</x:v>
       </x:c>
       <x:c r="O76" s="60" t="n">
-        <x:v>0.5307542656842682</x:v>
+        <x:v>0.53075427</x:v>
       </x:c>
       <x:c r="P76" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14405,13 +14405,13 @@
         <x:v>143851677</x:v>
       </x:c>
       <x:c r="M77" s="60" t="n">
-        <x:v>0.057981692450543625</x:v>
+        <x:v>0.05798169</x:v>
       </x:c>
       <x:c r="N77" s="60" t="n">
-        <x:v>0.23953980811909914</x:v>
+        <x:v>0.23953981</x:v>
       </x:c>
       <x:c r="O77" s="60" t="n">
-        <x:v>0.5419023262398911</x:v>
+        <x:v>0.54190233</x:v>
       </x:c>
       <x:c r="P77" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14467,13 +14467,13 @@
         <x:v>10411888773</x:v>
       </x:c>
       <x:c r="M78" s="60" t="n">
-        <x:v>0.13270259783975952</x:v>
+        <x:v>0.1327026</x:v>
       </x:c>
       <x:c r="N78" s="60" t="n">
-        <x:v>0.3333806045201002</x:v>
+        <x:v>0.3333806</x:v>
       </x:c>
       <x:c r="O78" s="60" t="n">
-        <x:v>0.5799923330846631</x:v>
+        <x:v>0.57999233</x:v>
       </x:c>
       <x:c r="P78" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14529,13 +14529,13 @@
         <x:v>7977727305</x:v>
       </x:c>
       <x:c r="M79" s="60" t="n">
-        <x:v>0.15556324640648622</x:v>
+        <x:v>0.15556325</x:v>
       </x:c>
       <x:c r="N79" s="60" t="n">
-        <x:v>0.3546310080642221</x:v>
+        <x:v>0.35463101</x:v>
       </x:c>
       <x:c r="O79" s="60" t="n">
-        <x:v>0.5878429358416998</x:v>
+        <x:v>0.58784294</x:v>
       </x:c>
       <x:c r="P79" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14591,13 +14591,13 @@
         <x:v>6674984854</x:v>
       </x:c>
       <x:c r="M80" s="60" t="n">
-        <x:v>0.15393325220277285</x:v>
+        <x:v>0.15393325</x:v>
       </x:c>
       <x:c r="N80" s="60" t="n">
-        <x:v>0.3486587149289716</x:v>
+        <x:v>0.34865871</x:v>
       </x:c>
       <x:c r="O80" s="60" t="n">
-        <x:v>0.5966962617393033</x:v>
+        <x:v>0.59669626</x:v>
       </x:c>
       <x:c r="P80" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14653,13 +14653,13 @@
         <x:v>7762249301</x:v>
       </x:c>
       <x:c r="M81" s="60" t="n">
-        <x:v>0.13751254067403254</x:v>
+        <x:v>0.13751254</x:v>
       </x:c>
       <x:c r="N81" s="60" t="n">
-        <x:v>0.33336179102249097</x:v>
+        <x:v>0.33336179</x:v>
       </x:c>
       <x:c r="O81" s="60" t="n">
-        <x:v>0.5685074797470399</x:v>
+        <x:v>0.56850748</x:v>
       </x:c>
       <x:c r="P81" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14715,13 +14715,13 @@
         <x:v>6170799043</x:v>
       </x:c>
       <x:c r="M82" s="60" t="n">
-        <x:v>0.14672407527033082</x:v>
+        <x:v>0.14672408</x:v>
       </x:c>
       <x:c r="N82" s="60" t="n">
-        <x:v>0.34772613115651124</x:v>
+        <x:v>0.34772613</x:v>
       </x:c>
       <x:c r="O82" s="60" t="n">
-        <x:v>0.5983416907086512</x:v>
+        <x:v>0.59834169</x:v>
       </x:c>
       <x:c r="P82" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14777,13 +14777,13 @@
         <x:v>6423284733</x:v>
       </x:c>
       <x:c r="M83" s="60" t="n">
-        <x:v>0.1411928776265905</x:v>
+        <x:v>0.14119288</x:v>
       </x:c>
       <x:c r="N83" s="60" t="n">
-        <x:v>0.3293801844583917</x:v>
+        <x:v>0.32938018</x:v>
       </x:c>
       <x:c r="O83" s="60" t="n">
-        <x:v>0.5743605686196296</x:v>
+        <x:v>0.57436057</x:v>
       </x:c>
       <x:c r="P83" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14839,13 +14839,13 @@
         <x:v>5655962813</x:v>
       </x:c>
       <x:c r="M84" s="60" t="n">
-        <x:v>0.15320379798500974</x:v>
+        <x:v>0.1532038</x:v>
       </x:c>
       <x:c r="N84" s="60" t="n">
-        <x:v>0.34940616631005283</x:v>
+        <x:v>0.34940617</x:v>
       </x:c>
       <x:c r="O84" s="60" t="n">
-        <x:v>0.5977513327300051</x:v>
+        <x:v>0.59775133</x:v>
       </x:c>
       <x:c r="P84" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14901,13 +14901,13 @@
         <x:v>5512796902</x:v>
       </x:c>
       <x:c r="M85" s="60" t="n">
-        <x:v>0.14104366202694632</x:v>
+        <x:v>0.14104366</x:v>
       </x:c>
       <x:c r="N85" s="60" t="n">
-        <x:v>0.330745528028918</x:v>
+        <x:v>0.33074553</x:v>
       </x:c>
       <x:c r="O85" s="60" t="n">
-        <x:v>0.5695062387425024</x:v>
+        <x:v>0.56950624</x:v>
       </x:c>
       <x:c r="P85" s="60" t="n">
         <x:v>0.4</x:v>
@@ -14963,13 +14963,13 @@
         <x:v>66032029</x:v>
       </x:c>
       <x:c r="M86" s="60" t="n">
-        <x:v>0.059128385322414476</x:v>
+        <x:v>0.05912839</x:v>
       </x:c>
       <x:c r="N86" s="60" t="n">
-        <x:v>0.23902877668283895</x:v>
+        <x:v>0.23902878</x:v>
       </x:c>
       <x:c r="O86" s="60" t="n">
-        <x:v>0.537775662562963</x:v>
+        <x:v>0.53777566</x:v>
       </x:c>
       <x:c r="P86" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15025,13 +15025,13 @@
         <x:v>311914535</x:v>
       </x:c>
       <x:c r="M87" s="60" t="n">
-        <x:v>0.08000069548019041</x:v>
+        <x:v>0.0800007</x:v>
       </x:c>
       <x:c r="N87" s="60" t="n">
-        <x:v>0.25614808040107107</x:v>
+        <x:v>0.25614808</x:v>
       </x:c>
       <x:c r="O87" s="60" t="n">
-        <x:v>0.5417957305930154</x:v>
+        <x:v>0.54179573</x:v>
       </x:c>
       <x:c r="P87" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15087,13 +15087,13 @@
         <x:v>3150427075</x:v>
       </x:c>
       <x:c r="M88" s="60" t="n">
-        <x:v>0.15987532111669478</x:v>
+        <x:v>0.15987532</x:v>
       </x:c>
       <x:c r="N88" s="60" t="n">
-        <x:v>0.3557561618348383</x:v>
+        <x:v>0.35575616</x:v>
       </x:c>
       <x:c r="O88" s="60" t="n">
-        <x:v>0.5965248523800092</x:v>
+        <x:v>0.59652485</x:v>
       </x:c>
       <x:c r="P88" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15149,13 +15149,13 @@
         <x:v>299309437</x:v>
       </x:c>
       <x:c r="M89" s="60" t="n">
-        <x:v>0.07928030460676123</x:v>
+        <x:v>0.0792803</x:v>
       </x:c>
       <x:c r="N89" s="60" t="n">
-        <x:v>0.26349395372180207</x:v>
+        <x:v>0.26349395</x:v>
       </x:c>
       <x:c r="O89" s="60" t="n">
-        <x:v>0.5400034131292338</x:v>
+        <x:v>0.54000341</x:v>
       </x:c>
       <x:c r="P89" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15211,13 +15211,13 @@
         <x:v>2407226467</x:v>
       </x:c>
       <x:c r="M90" s="60" t="n">
-        <x:v>0.14935064333062287</x:v>
+        <x:v>0.14935064</x:v>
       </x:c>
       <x:c r="N90" s="60" t="n">
-        <x:v>0.3510842962723428</x:v>
+        <x:v>0.3510843</x:v>
       </x:c>
       <x:c r="O90" s="60" t="n">
-        <x:v>0.5907813454050208</x:v>
+        <x:v>0.59078135</x:v>
       </x:c>
       <x:c r="P90" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15273,13 +15273,13 @@
         <x:v>1553389871</x:v>
       </x:c>
       <x:c r="M91" s="60" t="n">
-        <x:v>0.1415115981139059</x:v>
+        <x:v>0.1415116</x:v>
       </x:c>
       <x:c r="N91" s="60" t="n">
-        <x:v>0.33577666002654183</x:v>
+        <x:v>0.33577666</x:v>
       </x:c>
       <x:c r="O91" s="60" t="n">
-        <x:v>0.5824523943009257</x:v>
+        <x:v>0.58245239</x:v>
       </x:c>
       <x:c r="P91" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15335,13 +15335,13 @@
         <x:v>1098982180</x:v>
       </x:c>
       <x:c r="M92" s="60" t="n">
-        <x:v>0.13796929915349582</x:v>
+        <x:v>0.1379693</x:v>
       </x:c>
       <x:c r="N92" s="60" t="n">
-        <x:v>0.33280748286176065</x:v>
+        <x:v>0.33280748</x:v>
       </x:c>
       <x:c r="O92" s="60" t="n">
-        <x:v>0.5675865332348029</x:v>
+        <x:v>0.56758653</x:v>
       </x:c>
       <x:c r="P92" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15397,13 +15397,13 @@
         <x:v>906823837</x:v>
       </x:c>
       <x:c r="M93" s="60" t="n">
-        <x:v>0.13717063569266863</x:v>
+        <x:v>0.13717064</x:v>
       </x:c>
       <x:c r="N93" s="60" t="n">
-        <x:v>0.3279829120033917</x:v>
+        <x:v>0.32798291</x:v>
       </x:c>
       <x:c r="O93" s="60" t="n">
-        <x:v>0.5767720949553141</x:v>
+        <x:v>0.57677209</x:v>
       </x:c>
       <x:c r="P93" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15459,13 +15459,13 @@
         <x:v>706545811</x:v>
       </x:c>
       <x:c r="M94" s="60" t="n">
-        <x:v>0.15487032511431684</x:v>
+        <x:v>0.15487033</x:v>
       </x:c>
       <x:c r="N94" s="60" t="n">
-        <x:v>0.347528944289013</x:v>
+        <x:v>0.34752894</x:v>
       </x:c>
       <x:c r="O94" s="60" t="n">
-        <x:v>0.5949762827278698</x:v>
+        <x:v>0.59497628</x:v>
       </x:c>
       <x:c r="P94" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15521,13 +15521,13 @@
         <x:v>74388380</x:v>
       </x:c>
       <x:c r="M95" s="60" t="n">
-        <x:v>0.07996194308491547</x:v>
+        <x:v>0.07996194</x:v>
       </x:c>
       <x:c r="N95" s="60" t="n">
-        <x:v>0.263774993882805</x:v>
+        <x:v>0.26377499</x:v>
       </x:c>
       <x:c r="O95" s="60" t="n">
-        <x:v>0.5344293384884676</x:v>
+        <x:v>0.53442934</x:v>
       </x:c>
       <x:c r="P95" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15583,13 +15583,13 @@
         <x:v>558168176</x:v>
       </x:c>
       <x:c r="M96" s="60" t="n">
-        <x:v>0.15235544623152342</x:v>
+        <x:v>0.15235545</x:v>
       </x:c>
       <x:c r="N96" s="60" t="n">
-        <x:v>0.3534211018551118</x:v>
+        <x:v>0.3534211</x:v>
       </x:c>
       <x:c r="O96" s="60" t="n">
-        <x:v>0.5897810177625622</x:v>
+        <x:v>0.58978102</x:v>
       </x:c>
       <x:c r="P96" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15645,13 +15645,13 @@
         <x:v>438434317</x:v>
       </x:c>
       <x:c r="M97" s="60" t="n">
-        <x:v>0.15663281003275367</x:v>
+        <x:v>0.15663281</x:v>
       </x:c>
       <x:c r="N97" s="60" t="n">
-        <x:v>0.3543115635719129</x:v>
+        <x:v>0.35431156</x:v>
       </x:c>
       <x:c r="O97" s="60" t="n">
-        <x:v>0.5811272460952601</x:v>
+        <x:v>0.58112725</x:v>
       </x:c>
       <x:c r="P97" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15707,13 +15707,13 @@
         <x:v>225720257</x:v>
       </x:c>
       <x:c r="M98" s="60" t="n">
-        <x:v>0.1393503096930404</x:v>
+        <x:v>0.13935031</x:v>
       </x:c>
       <x:c r="N98" s="60" t="n">
-        <x:v>0.3302703623788037</x:v>
+        <x:v>0.33027036</x:v>
       </x:c>
       <x:c r="O98" s="60" t="n">
-        <x:v>0.5745711134656708</x:v>
+        <x:v>0.57457111</x:v>
       </x:c>
       <x:c r="P98" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15769,13 +15769,13 @@
         <x:v>217598804</x:v>
       </x:c>
       <x:c r="M99" s="60" t="n">
-        <x:v>0.14994254709537672</x:v>
+        <x:v>0.14994255</x:v>
       </x:c>
       <x:c r="N99" s="60" t="n">
-        <x:v>0.35261697118400404</x:v>
+        <x:v>0.35261697</x:v>
       </x:c>
       <x:c r="O99" s="60" t="n">
-        <x:v>0.5923329411202023</x:v>
+        <x:v>0.59233294</x:v>
       </x:c>
       <x:c r="P99" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15831,13 +15831,13 @@
         <x:v>124012840</x:v>
       </x:c>
       <x:c r="M100" s="60" t="n">
-        <x:v>0.13933594923454623</x:v>
+        <x:v>0.13933595</x:v>
       </x:c>
       <x:c r="N100" s="60" t="n">
-        <x:v>0.3299720569879731</x:v>
+        <x:v>0.32997206</x:v>
       </x:c>
       <x:c r="O100" s="60" t="n">
-        <x:v>0.5757070444258258</x:v>
+        <x:v>0.57570704</x:v>
       </x:c>
       <x:c r="P100" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15893,13 +15893,13 @@
         <x:v>103426921</x:v>
       </x:c>
       <x:c r="M101" s="60" t="n">
-        <x:v>0.15474167617378115</x:v>
+        <x:v>0.15474168</x:v>
       </x:c>
       <x:c r="N101" s="60" t="n">
-        <x:v>0.348396856167403</x:v>
+        <x:v>0.34839686</x:v>
       </x:c>
       <x:c r="O101" s="60" t="n">
-        <x:v>0.5904320867837234</x:v>
+        <x:v>0.59043209</x:v>
       </x:c>
       <x:c r="P101" s="60" t="n">
         <x:v>0.4</x:v>
@@ -15955,13 +15955,13 @@
         <x:v>42948708</x:v>
       </x:c>
       <x:c r="M102" s="60" t="n">
-        <x:v>0.14405400741204757</x:v>
+        <x:v>0.14405401</x:v>
       </x:c>
       <x:c r="N102" s="60" t="n">
-        <x:v>0.33066759833201087</x:v>
+        <x:v>0.3306676</x:v>
       </x:c>
       <x:c r="O102" s="60" t="n">
-        <x:v>0.5703376141555456</x:v>
+        <x:v>0.57033761</x:v>
       </x:c>
       <x:c r="P102" s="60" t="n">
         <x:v>0.4</x:v>
@@ -16017,13 +16017,13 @@
         <x:v>37191791</x:v>
       </x:c>
       <x:c r="M103" s="60" t="n">
-        <x:v>0.15351623452791013</x:v>
+        <x:v>0.15351623</x:v>
       </x:c>
       <x:c r="N103" s="60" t="n">
-        <x:v>0.35249474702465106</x:v>
+        <x:v>0.35249475</x:v>
       </x:c>
       <x:c r="O103" s="60" t="n">
-        <x:v>0.5939919106085141</x:v>
+        <x:v>0.59399191</x:v>
       </x:c>
       <x:c r="P103" s="60" t="n">
         <x:v>0.4</x:v>
@@ -16079,13 +16079,13 @@
         <x:v>26690474809</x:v>
       </x:c>
       <x:c r="M104" s="60" t="n">
-        <x:v>0.19354122269601623</x:v>
+        <x:v>0.19354122</x:v>
       </x:c>
       <x:c r="N104" s="60" t="n">
-        <x:v>0.41874351247493935</x:v>
+        <x:v>0.41874351</x:v>
       </x:c>
       <x:c r="O104" s="60" t="n">
-        <x:v>0.6754622367322481</x:v>
+        <x:v>0.67546224</x:v>
       </x:c>
       <x:c r="P104" s="60" t="n">
         <x:v>0.4</x:v>
@@ -20015,6 +20015,6 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9209b29ba07c40d5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R388a1b7bc9e241f0"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Regenerate V3.1.1 deliverables from the clean commit
First build in which clean_worktree is both true and meaningful: source
and all 74 reproducibility-gated artifacts match commit f5015d8, and the
eight deliverables that stamp their own creation time are reported
separately rather than counted as drift. 16/16 checks PASS.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R85785b356f604014"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R8a59b25cf4ba4d34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R428e369d5fc74a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rc21066791fc3423a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R08a0351e8b7f49df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Rf3be4fca1920409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R532baf8aa92c4d49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R2490ddd02c224d85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R1ccf9b16f9e34daa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R29110f6a13834a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="Rc9391111351d4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rcb793d76a4e64027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R688466755ead4e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="R7c0e3ed2dd874566"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Rc395202b6ae74a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R065b38c51d0c4a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R2be49a70bfb14ff2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Ra6a26162be964a03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,88 +18,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={CC4CFB03-5DD1-548A-5EDA-EB3C658E7D6C}</x:author>
-    <x:author>tc={94F31227-EC85-0309-4C38-757F1F13F021}</x:author>
-    <x:author>tc={763EC0B8-9A34-4E63-9EA1-C25C152E644F}</x:author>
-    <x:author>tc={EDEE2F21-8C7C-0A16-CBFA-D89BB89D783F}</x:author>
-    <x:author>tc={1BC5137B-9CBE-025D-0115-C6AF58FE56FA}</x:author>
-    <x:author>tc={6D455CF3-D224-A096-1CC1-3B7EDE3770B2}</x:author>
-    <x:author>tc={B1C7A9E5-FA9A-B290-FDBA-391E687567BD}</x:author>
-    <x:author>tc={AD9B86A0-704C-ED83-C8CE-E993A3680AD8}</x:author>
-    <x:author>tc={E9567DB2-E4A4-BD54-A15C-EE318F149E7C}</x:author>
-    <x:author>tc={5AA32AF5-2460-2652-9FC0-C13F568267B1}</x:author>
-    <x:author>tc={2B2B76AD-E182-2825-38F8-085934593D20}</x:author>
-    <x:author>tc={126B858B-8478-B315-3D31-D4D11C92D932}</x:author>
-    <x:author>tc={71DC2737-8C1A-B73A-5054-AD0CA99CF86C}</x:author>
-    <x:author>tc={80D8D3DE-5FD5-8417-918D-4C29661E06FD}</x:author>
-    <x:author>tc={C19392AF-2D87-00A6-E5B3-22AA8F556527}</x:author>
-    <x:author>tc={BA3BAFCA-A3F0-4C55-80B2-BC6C7CDC175B}</x:author>
-    <x:author>tc={BA3701F5-9133-64C4-3EF8-C46F8A6D9DF4}</x:author>
-    <x:author>tc={3FE20876-E7F2-A33E-B4B1-E7B542981658}</x:author>
-    <x:author>tc={1383E8B0-7989-3E0C-8C9A-1C95F27BA662}</x:author>
-    <x:author>tc={C4ECAD9A-F597-8C29-71D2-481AA9D3B40E}</x:author>
-    <x:author>tc={F03FCD14-B86A-BA51-9178-951D87FF8A02}</x:author>
-    <x:author>tc={F4FB6FC8-09E8-6941-1FA1-6CDFBA05F4A7}</x:author>
-    <x:author>tc={FAB077CB-EA3D-958B-D86C-B8D3BD7F5510}</x:author>
-    <x:author>tc={E7ADB5CF-1674-548B-3ACB-ADC0B3BFBAE0}</x:author>
-    <x:author>tc={D68CF1B3-641D-0EE8-372D-2D3C29CB1DB6}</x:author>
-    <x:author>tc={B819BD9E-5E80-8B82-66D1-ECDEE4F969FA}</x:author>
-    <x:author>tc={4147D225-4A98-E329-11A3-2F02353C1A12}</x:author>
-    <x:author>tc={195F3174-74E2-1053-8D0B-6D8AE23510EB}</x:author>
-    <x:author>tc={27287E2C-E40A-0D1F-3068-F52137CC03B0}</x:author>
-    <x:author>tc={6EE192F8-0655-37A3-06F3-63D6C4B2FF11}</x:author>
-    <x:author>tc={4CFAF0D5-8D0E-6D10-3574-D46B8676B45E}</x:author>
-    <x:author>tc={8CB6B34D-0A27-90BC-1CFF-D345DD04A236}</x:author>
-    <x:author>tc={71114867-E631-33C4-99C2-ADA5EE424963}</x:author>
-    <x:author>tc={DC166D12-F31C-C6A0-2444-ADAF7FC3D935}</x:author>
-    <x:author>tc={1060D2B0-3760-6F37-6C2B-C2E6CD6E1221}</x:author>
-    <x:author>tc={7EF1990A-D058-6276-71FF-CB4B5DE49E9E}</x:author>
-    <x:author>tc={DCE19479-B373-5123-C96E-98834DE5B3E2}</x:author>
-    <x:author>tc={529F85BE-5AA5-4B84-06AE-DB3091B2DC47}</x:author>
-    <x:author>tc={9461FC7D-60BC-6B02-A5DC-C437E1C9E62D}</x:author>
-    <x:author>tc={8AACD3EC-0BCC-2EFE-31E8-9600DC24BBEC}</x:author>
-    <x:author>tc={571BA2D7-E32A-C324-3C52-45F1BB266C89}</x:author>
-    <x:author>tc={B840A8D3-6A69-85CC-2268-FE011C545A2C}</x:author>
-    <x:author>tc={C769EF04-53D1-32E0-69BA-B9E5412A9C60}</x:author>
-    <x:author>tc={DECCF804-05D7-F488-65F2-006C3E094CEF}</x:author>
-    <x:author>tc={BA1B0BEF-D8B2-D5C1-9243-79B30C9F0AE0}</x:author>
-    <x:author>tc={760F8E4F-17A8-D4B8-DF85-136C6CBD0142}</x:author>
-    <x:author>tc={8769AF10-4E15-C591-FC5D-0B5B3B8E77BB}</x:author>
-    <x:author>tc={896696FF-A1E2-6B3B-5CE9-65E61791D307}</x:author>
-    <x:author>tc={7F3932EB-A497-6998-088A-577F9096D13D}</x:author>
-    <x:author>tc={7C307DC0-C1E2-FEF7-4EA1-272629EB2CCC}</x:author>
-    <x:author>tc={1C4A9BA9-E112-B8C4-FA82-DE13EB58DE6E}</x:author>
-    <x:author>tc={0F98FC95-29E9-7A82-2F54-AF82B109DEFD}</x:author>
-    <x:author>tc={60251A10-F844-0F0D-A9C6-23588ABF13B4}</x:author>
-    <x:author>tc={2717F9A6-EBA1-591C-938B-06BDDECA023B}</x:author>
-    <x:author>tc={75F764D3-C568-1DE7-FA96-1D806A269D59}</x:author>
-    <x:author>tc={FCE1FD4F-A5AD-0721-AEAA-C1080A47653B}</x:author>
-    <x:author>tc={A7A8E0FE-F76C-4679-9866-41669B23C7F4}</x:author>
-    <x:author>tc={6E234A2D-D06E-8418-93B5-E9B65C3F10DD}</x:author>
-    <x:author>tc={6AA6ED60-C597-5F1A-F385-9DCE93519AE5}</x:author>
-    <x:author>tc={B50FCEFF-7169-A425-5CA1-4D700944EF7D}</x:author>
-    <x:author>tc={6FA16210-C3E9-90C3-99FC-2BA5183DD9C9}</x:author>
-    <x:author>tc={BF1E1B04-A11F-D879-B226-1454584AC2F2}</x:author>
-    <x:author>tc={F048CD8F-C06C-8041-85B7-869713C1FAAE}</x:author>
-    <x:author>tc={7BB204AD-5904-4F72-D602-7FB91C7308A6}</x:author>
-    <x:author>tc={3FA395CE-7014-AEA1-DA13-D6F8B7A622E7}</x:author>
-    <x:author>tc={D42904B0-75A5-0AF0-D8DE-268FC0D0D1C3}</x:author>
-    <x:author>tc={625F82DA-B230-1EBC-8083-68F812A66A65}</x:author>
-    <x:author>tc={501B5F46-0BD1-45D3-4F51-7520B2A36B43}</x:author>
-    <x:author>tc={436A0272-2ACB-C643-A25B-C057F780A24C}</x:author>
-    <x:author>tc={03B7105B-F1A3-B144-DA34-2308027D68DD}</x:author>
-    <x:author>tc={5DDDB1F3-2ED2-9986-E999-2A89DF276981}</x:author>
-    <x:author>tc={A4DB01C2-6866-2E86-76BD-BA6131F161E0}</x:author>
-    <x:author>tc={3DDF3995-E808-6B13-F671-8C604F555C43}</x:author>
-    <x:author>tc={F5425FE7-40D1-F91B-9C30-3A169A05019D}</x:author>
-    <x:author>tc={DDF45385-3192-9B14-BB74-41F9729DE279}</x:author>
-    <x:author>tc={AD99753A-5CC9-08C2-ED82-6AAB789196B1}</x:author>
-    <x:author>tc={E8ED60AE-FB15-E19C-724B-6F52657EFB83}</x:author>
-    <x:author>tc={E387118F-BB76-BCCB-8B34-D9403C627B90}</x:author>
-    <x:author>tc={699298B9-8C7E-8D53-D7A2-D391CAA65C08}</x:author>
-    <x:author>tc={7E94DC4F-9F5F-2C31-0E56-B25549C4114D}</x:author>
-    <x:author>tc={63924084-A4B4-A2C8-9AE0-901C6DEE975C}</x:author>
-    <x:author>tc={FF5AF36B-9034-0A1E-0659-33A2B79D0A61}</x:author>
+    <x:author>tc={B1F1D5AE-8EBF-0084-68B9-588044F855FA}</x:author>
+    <x:author>tc={7231126E-BFE8-3149-9559-5C1A6E685DFA}</x:author>
+    <x:author>tc={5DB9FB1D-6005-55BB-E387-9C72FF3CBF9F}</x:author>
+    <x:author>tc={910E8916-EC32-3A8E-D222-263C7EF0BD91}</x:author>
+    <x:author>tc={30CAB49F-185C-2455-CED0-A1B8D048806F}</x:author>
+    <x:author>tc={1A4CA30F-85AB-8658-20D9-CB00B1BEB9CA}</x:author>
+    <x:author>tc={4F3231EC-6AE1-2072-C2AC-E683E85BBC79}</x:author>
+    <x:author>tc={89DEC437-E16F-56DE-3A10-68F4F9F5AFE6}</x:author>
+    <x:author>tc={3EC4B70D-03D2-5B2D-B490-EECBE8661DF3}</x:author>
+    <x:author>tc={BE220695-912F-4438-2E7A-F6117F708332}</x:author>
+    <x:author>tc={B487C9BC-2365-D46A-2D3C-F4F7AD8B7B17}</x:author>
+    <x:author>tc={EB67CA8A-8543-97B8-6D43-E331884F3C27}</x:author>
+    <x:author>tc={2408450E-AD95-0CE5-1B57-694349598BFB}</x:author>
+    <x:author>tc={9D6F731B-543C-9A8E-F3E0-F7F7D7EF7EF9}</x:author>
+    <x:author>tc={8A96D604-FB14-A681-46EF-CDAF047B04C8}</x:author>
+    <x:author>tc={0EA1C43B-38E0-EB4F-5424-F88282DF615B}</x:author>
+    <x:author>tc={BCF230C7-EAC4-09E3-3774-1FB4243FE18A}</x:author>
+    <x:author>tc={72182531-88E8-7A81-CA18-6BD8BDF28F1F}</x:author>
+    <x:author>tc={4E3A9C64-512C-C023-AC10-90D732DA7E36}</x:author>
+    <x:author>tc={2D46A642-6ACA-63D2-95AF-B860815B81E3}</x:author>
+    <x:author>tc={C87A2A95-2138-AD87-DD51-5B955612640D}</x:author>
+    <x:author>tc={BE7FCA45-36B2-63AC-CECB-D8116A094326}</x:author>
+    <x:author>tc={ADAE87A1-2761-2924-3B0E-4B303487CBB4}</x:author>
+    <x:author>tc={4BDE2C53-A72E-3F0B-4154-ED839E66DC45}</x:author>
+    <x:author>tc={4054DC46-FF06-1700-D2B7-DF2670B2C656}</x:author>
+    <x:author>tc={E80A436B-C17C-AACA-80D6-A25DC12812E1}</x:author>
+    <x:author>tc={86FEFEC8-0B01-6E20-F14D-2FC16DD96231}</x:author>
+    <x:author>tc={AAEFD3B3-8790-8D7F-320D-2CDA2FF8A342}</x:author>
+    <x:author>tc={22C2CD20-E295-821C-1EE1-909A06C7A55A}</x:author>
+    <x:author>tc={45657CAB-FA0B-4401-4903-20DA87258319}</x:author>
+    <x:author>tc={9577CE79-E215-56E2-1E17-924923780664}</x:author>
+    <x:author>tc={622FAE1C-1B4B-5926-B5B7-D9CE82932DCA}</x:author>
+    <x:author>tc={847434EA-754E-5944-2608-A5B78BA89C4E}</x:author>
+    <x:author>tc={9E1DB528-14BE-9B10-D946-8A26CD50C4B5}</x:author>
+    <x:author>tc={29D45C1A-9323-306E-EBBE-BD13A640DF3F}</x:author>
+    <x:author>tc={81B11D3C-8402-604C-197C-D3AC438D4894}</x:author>
+    <x:author>tc={9D8FABD7-EF03-A37C-FE21-C59947595333}</x:author>
+    <x:author>tc={4F270035-584E-92CD-91EC-BEBEB84E6B21}</x:author>
+    <x:author>tc={4268C114-4691-A5F5-E92E-DBA812B6D837}</x:author>
+    <x:author>tc={7335AA0A-4A79-55E2-569C-BC721767ECD8}</x:author>
+    <x:author>tc={16768DF3-5223-24F3-7E1E-E2D89517ECAF}</x:author>
+    <x:author>tc={F41DF9E7-3000-9978-F972-589AD85B3148}</x:author>
+    <x:author>tc={BCD5127B-E29F-3A59-C866-DFB43DA4D90C}</x:author>
+    <x:author>tc={9F4F3142-4641-3DD9-17B0-1EEDCFA44831}</x:author>
+    <x:author>tc={DAF0C64C-88C6-9D6A-2889-2B84162C1EE6}</x:author>
+    <x:author>tc={C591FD97-9A19-731C-BD65-7C7B49F6E820}</x:author>
+    <x:author>tc={B65B88BE-B1C0-67A9-27E5-52CB7284ED0F}</x:author>
+    <x:author>tc={7561914A-6C35-08F8-65B5-9D3C0E93CE57}</x:author>
+    <x:author>tc={09EFD1F1-C5AE-97CA-E019-AAACA66DEB49}</x:author>
+    <x:author>tc={0A545C43-FDD9-7CA6-29B4-C00AE3437969}</x:author>
+    <x:author>tc={DEC38D3B-C28F-AB7A-866B-00BEEFAAC695}</x:author>
+    <x:author>tc={F269F1AD-014D-88F3-DE81-86A62A5F6960}</x:author>
+    <x:author>tc={46B546BE-D1D5-5159-CF60-298E6676403A}</x:author>
+    <x:author>tc={B74533AB-09F4-9D57-353B-68A04A6DA2C6}</x:author>
+    <x:author>tc={AD27CC21-B213-CEE9-D47B-5FF9B97B4C9D}</x:author>
+    <x:author>tc={56F33B31-B447-3C03-BC07-8DF6DAD3E8BE}</x:author>
+    <x:author>tc={39FCA924-ABA8-C06F-F2C9-9FD6E3CB341D}</x:author>
+    <x:author>tc={12F0FF2C-91E0-1F17-FAB2-C654D27B41CA}</x:author>
+    <x:author>tc={6C9879EE-F2A8-9F5B-DC96-993988AB2E83}</x:author>
+    <x:author>tc={6EE345CC-A49F-239F-3409-DBA94CB65DE8}</x:author>
+    <x:author>tc={3D356D90-79C3-0C83-B8B9-DFD48BB73F29}</x:author>
+    <x:author>tc={C6556742-5E2C-5399-5286-D424B1C03177}</x:author>
+    <x:author>tc={1D86F6A4-162F-790C-BCED-72F639ECFB28}</x:author>
+    <x:author>tc={AD7EE60B-9B00-11D1-2945-E6266D3D318B}</x:author>
+    <x:author>tc={B7FA6F6B-1DCD-8C2A-7827-BBEDF2BC839F}</x:author>
+    <x:author>tc={9F00003B-A343-FDC5-8CF6-F233621EE92F}</x:author>
+    <x:author>tc={E0591950-7C86-12B6-CF26-BBF0BD5A424D}</x:author>
+    <x:author>tc={D190965A-7312-1E68-DD1B-5CAE0AC647E1}</x:author>
+    <x:author>tc={4C2131E1-089A-795C-1F39-834625B25BF6}</x:author>
+    <x:author>tc={0C0F2D4B-F426-0F38-91CA-9DDDEEC2B4AD}</x:author>
+    <x:author>tc={4CCEE3EC-CFC9-867B-17AE-BE1C867313DC}</x:author>
+    <x:author>tc={F8A39C87-E75F-9602-49DA-AEC00879B93E}</x:author>
+    <x:author>tc={18EE0677-6AC0-8F98-112A-42EFA485E797}</x:author>
+    <x:author>tc={E5F5DC43-70B6-B936-EAFE-D04E9B151BEE}</x:author>
+    <x:author>tc={423999F5-1FB9-4434-85E1-C51D1FE81372}</x:author>
+    <x:author>tc={839B6BF3-EF91-4FAA-39CA-1EF58A0BD9F4}</x:author>
+    <x:author>tc={C5BD0A00-04D8-68F0-AB32-A4E5296CAEA9}</x:author>
+    <x:author>tc={D8A463D4-B481-45D2-7E42-A93303517D14}</x:author>
+    <x:author>tc={61738CD4-C155-1B7F-ED09-A467CEA156C0}</x:author>
+    <x:author>tc={EB912D5D-EEB9-CFAF-0DA8-76FF7D648441}</x:author>
+    <x:author>tc={74619266-E08E-B097-1BAD-70C1CF56DAAC}</x:author>
+    <x:author>tc={BFFF1BAD-54D6-A74D-44E8-F922D6F58F15}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1175,26 +1175,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={E6544F10-0C97-C8AA-9837-D285C37E7F77}</x:author>
-    <x:author>tc={54A31122-763A-CA4B-6E06-E8A95C9E4EEC}</x:author>
-    <x:author>tc={037D2A01-81EB-6661-6220-72E149A6C8F0}</x:author>
-    <x:author>tc={B256CE58-E3F9-81CA-7249-8A38E34C866D}</x:author>
-    <x:author>tc={1B5B8133-2782-4688-A320-630F230CCD48}</x:author>
-    <x:author>tc={BBE04B97-7DFB-394C-E57A-8DBBE52BF457}</x:author>
-    <x:author>tc={20614F84-2248-ADF7-3E4E-7FFD9E6E4FCF}</x:author>
-    <x:author>tc={36DB5222-E723-2AB9-43BB-8978D85D7452}</x:author>
-    <x:author>tc={56C587BD-2992-C7CD-29E7-8069D0C30920}</x:author>
-    <x:author>tc={74390662-9EE3-DA1E-E831-671A02938D4D}</x:author>
-    <x:author>tc={B4789910-C767-1AFF-8121-B7CBD3C1683F}</x:author>
-    <x:author>tc={2A92B604-161F-A2A1-68F2-00380FB6D95F}</x:author>
-    <x:author>tc={38BAB3DC-3E42-1E38-A345-D773920F1A18}</x:author>
-    <x:author>tc={1526E168-58CB-B77A-FB7A-8926D79B25A3}</x:author>
-    <x:author>tc={1C88D8F1-594B-9DFD-7731-D5F0D5F87704}</x:author>
-    <x:author>tc={D91F79E7-6F53-7369-6A9C-3ABF2C8B885E}</x:author>
-    <x:author>tc={22EA1B97-97F4-0702-6B91-6997A8A60541}</x:author>
-    <x:author>tc={91E43DF2-86A6-66CA-3584-7C3DFE2606FF}</x:author>
-    <x:author>tc={F3741990-9FF5-CD11-7731-E40F9C494305}</x:author>
-    <x:author>tc={E33182D8-C6FF-D9E9-5B55-36905FD6B5C7}</x:author>
+    <x:author>tc={19EB02AB-B83A-8CE4-4EAB-38B680BC7C11}</x:author>
+    <x:author>tc={5E8B4292-D60A-4F18-B196-478BC9B0DB86}</x:author>
+    <x:author>tc={9893D5B2-25CE-34F9-3E46-3929CB53FE0A}</x:author>
+    <x:author>tc={4D92B10D-A494-0DAA-C2EB-5354306BE40F}</x:author>
+    <x:author>tc={D81A038F-D375-8269-1EE7-03F00A787DFE}</x:author>
+    <x:author>tc={22B62C71-3741-13AA-BFAE-1FC875AFD0F6}</x:author>
+    <x:author>tc={4E45B394-F82E-8C1D-F696-FFE7A6F883F8}</x:author>
+    <x:author>tc={A7D145CC-DC9D-9040-56C8-54C83A96E458}</x:author>
+    <x:author>tc={402F9E84-53D3-5F1A-5678-036937599159}</x:author>
+    <x:author>tc={2251A2FE-1BAA-338C-85A7-83AF318DC367}</x:author>
+    <x:author>tc={A67DA749-29E6-F1A3-094F-6791B0B741A1}</x:author>
+    <x:author>tc={1D25686C-8B9C-76F0-3A81-CA36379FBFA2}</x:author>
+    <x:author>tc={D3714FDA-5B97-3AED-F460-AF87D4C7FE58}</x:author>
+    <x:author>tc={0D0070A3-19EA-A803-9FF1-86DF63427505}</x:author>
+    <x:author>tc={66EC6765-ACDD-E01B-6A8E-D687E9B53A17}</x:author>
+    <x:author>tc={BE063722-D0B2-1C17-7A27-F8EBB067EDF8}</x:author>
+    <x:author>tc={129AC679-C322-7EDF-2D05-F930C01785C1}</x:author>
+    <x:author>tc={5B59801D-8187-A143-4078-DC34F3DCA574}</x:author>
+    <x:author>tc={5767ABB8-D080-C7E0-276B-CAEA4EBA3D8C}</x:author>
+    <x:author>tc={B0B1EB2E-B4BB-9060-6D43-CE609EE006EA}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2037,7 +2037,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6aa555770ddd4dac"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca9693ce0e474968"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2048,7 +2048,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}"/>
 </xltc:personList>
 </file>
 
@@ -2245,493 +2245,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-13T10:01:59.948" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{CC4CFB03-5DD1-548A-5EDA-EB3C658E7D6C}">
+  <xltc:threadedComment ref="P5" dT="2026-08-13T10:48:46.183" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{B1F1D5AE-8EBF-0084-68B9-588044F855FA}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-13T10:01:59.957" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{94F31227-EC85-0309-4C38-757F1F13F021}">
+  <xltc:threadedComment ref="P6" dT="2026-08-13T10:48:46.186" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{7231126E-BFE8-3149-9559-5C1A6E685DFA}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-13T10:01:59.957" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{763EC0B8-9A34-4E63-9EA1-C25C152E644F}">
+  <xltc:threadedComment ref="P7" dT="2026-08-13T10:48:46.186" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{5DB9FB1D-6005-55BB-E387-9C72FF3CBF9F}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-13T10:01:59.958" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{EDEE2F21-8C7C-0A16-CBFA-D89BB89D783F}">
+  <xltc:threadedComment ref="P8" dT="2026-08-13T10:48:46.187" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{910E8916-EC32-3A8E-D222-263C7EF0BD91}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-13T10:01:59.958" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{1BC5137B-9CBE-025D-0115-C6AF58FE56FA}">
+  <xltc:threadedComment ref="P9" dT="2026-08-13T10:48:46.187" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{30CAB49F-185C-2455-CED0-A1B8D048806F}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-13T10:01:59.958" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{6D455CF3-D224-A096-1CC1-3B7EDE3770B2}">
+  <xltc:threadedComment ref="P10" dT="2026-08-13T10:48:46.187" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{1A4CA30F-85AB-8658-20D9-CB00B1BEB9CA}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-13T10:01:59.958" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{B1C7A9E5-FA9A-B290-FDBA-391E687567BD}">
+  <xltc:threadedComment ref="P11" dT="2026-08-13T10:48:46.187" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4F3231EC-6AE1-2072-C2AC-E683E85BBC79}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-13T10:01:59.958" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{AD9B86A0-704C-ED83-C8CE-E993A3680AD8}">
+  <xltc:threadedComment ref="P12" dT="2026-08-13T10:48:46.187" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{89DEC437-E16F-56DE-3A10-68F4F9F5AFE6}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-13T10:01:59.958" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{E9567DB2-E4A4-BD54-A15C-EE318F149E7C}">
+  <xltc:threadedComment ref="P13" dT="2026-08-13T10:48:46.187" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{3EC4B70D-03D2-5B2D-B490-EECBE8661DF3}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{5AA32AF5-2460-2652-9FC0-C13F568267B1}">
+  <xltc:threadedComment ref="P14" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{BE220695-912F-4438-2E7A-F6117F708332}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{2B2B76AD-E182-2825-38F8-085934593D20}">
+  <xltc:threadedComment ref="P15" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{B487C9BC-2365-D46A-2D3C-F4F7AD8B7B17}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{126B858B-8478-B315-3D31-D4D11C92D932}">
+  <xltc:threadedComment ref="P16" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{EB67CA8A-8543-97B8-6D43-E331884F3C27}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{71DC2737-8C1A-B73A-5054-AD0CA99CF86C}">
+  <xltc:threadedComment ref="P17" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{2408450E-AD95-0CE5-1B57-694349598BFB}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{80D8D3DE-5FD5-8417-918D-4C29661E06FD}">
+  <xltc:threadedComment ref="P18" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{9D6F731B-543C-9A8E-F3E0-F7F7D7EF7EF9}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{C19392AF-2D87-00A6-E5B3-22AA8F556527}">
+  <xltc:threadedComment ref="P19" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{8A96D604-FB14-A681-46EF-CDAF047B04C8}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{BA3BAFCA-A3F0-4C55-80B2-BC6C7CDC175B}">
+  <xltc:threadedComment ref="P20" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{0EA1C43B-38E0-EB4F-5424-F88282DF615B}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{BA3701F5-9133-64C4-3EF8-C46F8A6D9DF4}">
+  <xltc:threadedComment ref="P21" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{BCF230C7-EAC4-09E3-3774-1FB4243FE18A}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{3FE20876-E7F2-A33E-B4B1-E7B542981658}">
+  <xltc:threadedComment ref="P22" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{72182531-88E8-7A81-CA18-6BD8BDF28F1F}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-13T10:01:59.959" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{1383E8B0-7989-3E0C-8C9A-1C95F27BA662}">
+  <xltc:threadedComment ref="P23" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4E3A9C64-512C-C023-AC10-90D732DA7E36}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{C4ECAD9A-F597-8C29-71D2-481AA9D3B40E}">
+  <xltc:threadedComment ref="P24" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{2D46A642-6ACA-63D2-95AF-B860815B81E3}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{F03FCD14-B86A-BA51-9178-951D87FF8A02}">
+  <xltc:threadedComment ref="P25" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{C87A2A95-2138-AD87-DD51-5B955612640D}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{F4FB6FC8-09E8-6941-1FA1-6CDFBA05F4A7}">
+  <xltc:threadedComment ref="P26" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{BE7FCA45-36B2-63AC-CECB-D8116A094326}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{FAB077CB-EA3D-958B-D86C-B8D3BD7F5510}">
+  <xltc:threadedComment ref="P27" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{ADAE87A1-2761-2924-3B0E-4B303487CBB4}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{E7ADB5CF-1674-548B-3ACB-ADC0B3BFBAE0}">
+  <xltc:threadedComment ref="P28" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4BDE2C53-A72E-3F0B-4154-ED839E66DC45}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{D68CF1B3-641D-0EE8-372D-2D3C29CB1DB6}">
+  <xltc:threadedComment ref="P29" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4054DC46-FF06-1700-D2B7-DF2670B2C656}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{B819BD9E-5E80-8B82-66D1-ECDEE4F969FA}">
+  <xltc:threadedComment ref="P30" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{E80A436B-C17C-AACA-80D6-A25DC12812E1}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{4147D225-4A98-E329-11A3-2F02353C1A12}">
+  <xltc:threadedComment ref="P31" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{86FEFEC8-0B01-6E20-F14D-2FC16DD96231}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{195F3174-74E2-1053-8D0B-6D8AE23510EB}">
+  <xltc:threadedComment ref="P32" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{AAEFD3B3-8790-8D7F-320D-2CDA2FF8A342}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{27287E2C-E40A-0D1F-3068-F52137CC03B0}">
+  <xltc:threadedComment ref="P33" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{22C2CD20-E295-821C-1EE1-909A06C7A55A}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{6EE192F8-0655-37A3-06F3-63D6C4B2FF11}">
+  <xltc:threadedComment ref="P34" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{45657CAB-FA0B-4401-4903-20DA87258319}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{4CFAF0D5-8D0E-6D10-3574-D46B8676B45E}">
+  <xltc:threadedComment ref="P35" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{9577CE79-E215-56E2-1E17-924923780664}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{8CB6B34D-0A27-90BC-1CFF-D345DD04A236}">
+  <xltc:threadedComment ref="P36" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{622FAE1C-1B4B-5926-B5B7-D9CE82932DCA}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{71114867-E631-33C4-99C2-ADA5EE424963}">
+  <xltc:threadedComment ref="P37" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{847434EA-754E-5944-2608-A5B78BA89C4E}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{DC166D12-F31C-C6A0-2444-ADAF7FC3D935}">
+  <xltc:threadedComment ref="P38" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{9E1DB528-14BE-9B10-D946-8A26CD50C4B5}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{1060D2B0-3760-6F37-6C2B-C2E6CD6E1221}">
+  <xltc:threadedComment ref="P39" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{29D45C1A-9323-306E-EBBE-BD13A640DF3F}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-13T10:01:59.96" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{7EF1990A-D058-6276-71FF-CB4B5DE49E9E}">
+  <xltc:threadedComment ref="P40" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{81B11D3C-8402-604C-197C-D3AC438D4894}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{DCE19479-B373-5123-C96E-98834DE5B3E2}">
+  <xltc:threadedComment ref="P41" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{9D8FABD7-EF03-A37C-FE21-C59947595333}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{529F85BE-5AA5-4B84-06AE-DB3091B2DC47}">
+  <xltc:threadedComment ref="P42" dT="2026-08-13T10:48:46.188" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4F270035-584E-92CD-91EC-BEBEB84E6B21}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{9461FC7D-60BC-6B02-A5DC-C437E1C9E62D}">
+  <xltc:threadedComment ref="P43" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4268C114-4691-A5F5-E92E-DBA812B6D837}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{8AACD3EC-0BCC-2EFE-31E8-9600DC24BBEC}">
+  <xltc:threadedComment ref="P44" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{7335AA0A-4A79-55E2-569C-BC721767ECD8}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{571BA2D7-E32A-C324-3C52-45F1BB266C89}">
+  <xltc:threadedComment ref="P45" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{16768DF3-5223-24F3-7E1E-E2D89517ECAF}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{B840A8D3-6A69-85CC-2268-FE011C545A2C}">
+  <xltc:threadedComment ref="P46" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{F41DF9E7-3000-9978-F972-589AD85B3148}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{C769EF04-53D1-32E0-69BA-B9E5412A9C60}">
+  <xltc:threadedComment ref="P47" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{BCD5127B-E29F-3A59-C866-DFB43DA4D90C}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{DECCF804-05D7-F488-65F2-006C3E094CEF}">
+  <xltc:threadedComment ref="P48" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{9F4F3142-4641-3DD9-17B0-1EEDCFA44831}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{BA1B0BEF-D8B2-D5C1-9243-79B30C9F0AE0}">
+  <xltc:threadedComment ref="P49" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{DAF0C64C-88C6-9D6A-2889-2B84162C1EE6}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{760F8E4F-17A8-D4B8-DF85-136C6CBD0142}">
+  <xltc:threadedComment ref="P50" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{C591FD97-9A19-731C-BD65-7C7B49F6E820}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{8769AF10-4E15-C591-FC5D-0B5B3B8E77BB}">
+  <xltc:threadedComment ref="P51" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{B65B88BE-B1C0-67A9-27E5-52CB7284ED0F}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{896696FF-A1E2-6B3B-5CE9-65E61791D307}">
+  <xltc:threadedComment ref="P52" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{7561914A-6C35-08F8-65B5-9D3C0E93CE57}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{7F3932EB-A497-6998-088A-577F9096D13D}">
+  <xltc:threadedComment ref="P53" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{09EFD1F1-C5AE-97CA-E019-AAACA66DEB49}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{7C307DC0-C1E2-FEF7-4EA1-272629EB2CCC}">
+  <xltc:threadedComment ref="P54" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{0A545C43-FDD9-7CA6-29B4-C00AE3437969}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{1C4A9BA9-E112-B8C4-FA82-DE13EB58DE6E}">
+  <xltc:threadedComment ref="P55" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{DEC38D3B-C28F-AB7A-866B-00BEEFAAC695}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{0F98FC95-29E9-7A82-2F54-AF82B109DEFD}">
+  <xltc:threadedComment ref="P56" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{F269F1AD-014D-88F3-DE81-86A62A5F6960}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{60251A10-F844-0F0D-A9C6-23588ABF13B4}">
+  <xltc:threadedComment ref="P57" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{46B546BE-D1D5-5159-CF60-298E6676403A}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-13T10:01:59.961" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{2717F9A6-EBA1-591C-938B-06BDDECA023B}">
+  <xltc:threadedComment ref="P58" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{B74533AB-09F4-9D57-353B-68A04A6DA2C6}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{75F764D3-C568-1DE7-FA96-1D806A269D59}">
+  <xltc:threadedComment ref="P59" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{AD27CC21-B213-CEE9-D47B-5FF9B97B4C9D}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{FCE1FD4F-A5AD-0721-AEAA-C1080A47653B}">
+  <xltc:threadedComment ref="P60" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{56F33B31-B447-3C03-BC07-8DF6DAD3E8BE}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{A7A8E0FE-F76C-4679-9866-41669B23C7F4}">
+  <xltc:threadedComment ref="P61" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{39FCA924-ABA8-C06F-F2C9-9FD6E3CB341D}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{6E234A2D-D06E-8418-93B5-E9B65C3F10DD}">
+  <xltc:threadedComment ref="P62" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{12F0FF2C-91E0-1F17-FAB2-C654D27B41CA}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{6AA6ED60-C597-5F1A-F385-9DCE93519AE5}">
+  <xltc:threadedComment ref="P63" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{6C9879EE-F2A8-9F5B-DC96-993988AB2E83}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{B50FCEFF-7169-A425-5CA1-4D700944EF7D}">
+  <xltc:threadedComment ref="P64" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{6EE345CC-A49F-239F-3409-DBA94CB65DE8}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{6FA16210-C3E9-90C3-99FC-2BA5183DD9C9}">
+  <xltc:threadedComment ref="P65" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{3D356D90-79C3-0C83-B8B9-DFD48BB73F29}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{BF1E1B04-A11F-D879-B226-1454584AC2F2}">
+  <xltc:threadedComment ref="P66" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{C6556742-5E2C-5399-5286-D424B1C03177}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{F048CD8F-C06C-8041-85B7-869713C1FAAE}">
+  <xltc:threadedComment ref="P67" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{1D86F6A4-162F-790C-BCED-72F639ECFB28}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{7BB204AD-5904-4F72-D602-7FB91C7308A6}">
+  <xltc:threadedComment ref="P68" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{AD7EE60B-9B00-11D1-2945-E6266D3D318B}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{3FA395CE-7014-AEA1-DA13-D6F8B7A622E7}">
+  <xltc:threadedComment ref="P69" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{B7FA6F6B-1DCD-8C2A-7827-BBEDF2BC839F}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{D42904B0-75A5-0AF0-D8DE-268FC0D0D1C3}">
+  <xltc:threadedComment ref="P70" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{9F00003B-A343-FDC5-8CF6-F233621EE92F}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{625F82DA-B230-1EBC-8083-68F812A66A65}">
+  <xltc:threadedComment ref="P71" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{E0591950-7C86-12B6-CF26-BBF0BD5A424D}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{501B5F46-0BD1-45D3-4F51-7520B2A36B43}">
+  <xltc:threadedComment ref="P72" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{D190965A-7312-1E68-DD1B-5CAE0AC647E1}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{436A0272-2ACB-C643-A25B-C057F780A24C}">
+  <xltc:threadedComment ref="P73" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4C2131E1-089A-795C-1F39-834625B25BF6}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{03B7105B-F1A3-B144-DA34-2308027D68DD}">
+  <xltc:threadedComment ref="P74" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{0C0F2D4B-F426-0F38-91CA-9DDDEEC2B4AD}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{5DDDB1F3-2ED2-9986-E999-2A89DF276981}">
+  <xltc:threadedComment ref="P75" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4CCEE3EC-CFC9-867B-17AE-BE1C867313DC}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{A4DB01C2-6866-2E86-76BD-BA6131F161E0}">
+  <xltc:threadedComment ref="P76" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{F8A39C87-E75F-9602-49DA-AEC00879B93E}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{3DDF3995-E808-6B13-F671-8C604F555C43}">
+  <xltc:threadedComment ref="P77" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{18EE0677-6AC0-8F98-112A-42EFA485E797}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{F5425FE7-40D1-F91B-9C30-3A169A05019D}">
+  <xltc:threadedComment ref="P78" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{E5F5DC43-70B6-B936-EAFE-D04E9B151BEE}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{DDF45385-3192-9B14-BB74-41F9729DE279}">
+  <xltc:threadedComment ref="P79" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{423999F5-1FB9-4434-85E1-C51D1FE81372}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{AD99753A-5CC9-08C2-ED82-6AAB789196B1}">
+  <xltc:threadedComment ref="P80" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{839B6BF3-EF91-4FAA-39CA-1EF58A0BD9F4}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-13T10:01:59.962" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{E8ED60AE-FB15-E19C-724B-6F52657EFB83}">
+  <xltc:threadedComment ref="P81" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{C5BD0A00-04D8-68F0-AB32-A4E5296CAEA9}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-13T10:01:59.963" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{E387118F-BB76-BCCB-8B34-D9403C627B90}">
+  <xltc:threadedComment ref="P82" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{D8A463D4-B481-45D2-7E42-A93303517D14}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-13T10:01:59.963" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{699298B9-8C7E-8D53-D7A2-D391CAA65C08}">
+  <xltc:threadedComment ref="P83" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{61738CD4-C155-1B7F-ED09-A467CEA156C0}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-13T10:01:59.963" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{7E94DC4F-9F5F-2C31-0E56-B25549C4114D}">
+  <xltc:threadedComment ref="P84" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{EB912D5D-EEB9-CFAF-0DA8-76FF7D648441}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-13T10:01:59.963" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{63924084-A4B4-A2C8-9AE0-901C6DEE975C}">
+  <xltc:threadedComment ref="P85" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{74619266-E08E-B097-1BAD-70C1CF56DAAC}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-13T10:01:59.963" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{FF5AF36B-9034-0A1E-0659-33A2B79D0A61}">
+  <xltc:threadedComment ref="P86" dT="2026-08-13T10:48:46.189" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{BFFF1BAD-54D6-A74D-44E8-F922D6F58F15}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2742,64 +2742,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-13T10:02:00.52" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{E6544F10-0C97-C8AA-9837-D285C37E7F77}">
+  <xltc:threadedComment ref="J5" dT="2026-08-13T10:48:46.529" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{19EB02AB-B83A-8CE4-4EAB-38B680BC7C11}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-13T10:02:00.524" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{54A31122-763A-CA4B-6E06-E8A95C9E4EEC}">
+  <xltc:threadedComment ref="J6" dT="2026-08-13T10:48:46.531" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{5E8B4292-D60A-4F18-B196-478BC9B0DB86}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-13T10:02:00.528" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{037D2A01-81EB-6661-6220-72E149A6C8F0}">
+  <xltc:threadedComment ref="J7" dT="2026-08-13T10:48:46.534" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{9893D5B2-25CE-34F9-3E46-3929CB53FE0A}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-13T10:02:00.534" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{B256CE58-E3F9-81CA-7249-8A38E34C866D}">
+  <xltc:threadedComment ref="J8" dT="2026-08-13T10:48:46.537" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4D92B10D-A494-0DAA-C2EB-5354306BE40F}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-13T10:02:00.538" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{1B5B8133-2782-4688-A320-630F230CCD48}">
+  <xltc:threadedComment ref="J9" dT="2026-08-13T10:48:46.539" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{D81A038F-D375-8269-1EE7-03F00A787DFE}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-13T10:02:00.54" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{BBE04B97-7DFB-394C-E57A-8DBBE52BF457}">
+  <xltc:threadedComment ref="J10" dT="2026-08-13T10:48:46.542" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{22B62C71-3741-13AA-BFAE-1FC875AFD0F6}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-13T10:02:00.546" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{20614F84-2248-ADF7-3E4E-7FFD9E6E4FCF}">
+  <xltc:threadedComment ref="J11" dT="2026-08-13T10:48:46.544" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{4E45B394-F82E-8C1D-F696-FFE7A6F883F8}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-13T10:02:00.55" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{36DB5222-E723-2AB9-43BB-8978D85D7452}">
+  <xltc:threadedComment ref="J12" dT="2026-08-13T10:48:46.548" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{A7D145CC-DC9D-9040-56C8-54C83A96E458}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-13T10:02:00.554" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{56C587BD-2992-C7CD-29E7-8069D0C30920}">
+  <xltc:threadedComment ref="J13" dT="2026-08-13T10:48:46.551" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{402F9E84-53D3-5F1A-5678-036937599159}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-13T10:02:00.558" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{74390662-9EE3-DA1E-E831-671A02938D4D}">
+  <xltc:threadedComment ref="J14" dT="2026-08-13T10:48:46.553" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{2251A2FE-1BAA-338C-85A7-83AF318DC367}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-13T10:02:00.562" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{B4789910-C767-1AFF-8121-B7CBD3C1683F}">
+  <xltc:threadedComment ref="J15" dT="2026-08-13T10:48:46.556" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{A67DA749-29E6-F1A3-094F-6791B0B741A1}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-13T10:02:00.568" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{2A92B604-161F-A2A1-68F2-00380FB6D95F}">
+  <xltc:threadedComment ref="J16" dT="2026-08-13T10:48:46.558" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{1D25686C-8B9C-76F0-3A81-CA36379FBFA2}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-13T10:02:00.571" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{38BAB3DC-3E42-1E38-A345-D773920F1A18}">
+  <xltc:threadedComment ref="J17" dT="2026-08-13T10:48:46.561" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{D3714FDA-5B97-3AED-F460-AF87D4C7FE58}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-13T10:02:00.574" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{1526E168-58CB-B77A-FB7A-8926D79B25A3}">
+  <xltc:threadedComment ref="J18" dT="2026-08-13T10:48:46.563" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{0D0070A3-19EA-A803-9FF1-86DF63427505}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-13T10:02:00.577" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{1C88D8F1-594B-9DFD-7731-D5F0D5F87704}">
+  <xltc:threadedComment ref="J19" dT="2026-08-13T10:48:46.564" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{66EC6765-ACDD-E01B-6A8E-D687E9B53A17}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-13T10:02:00.581" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{D91F79E7-6F53-7369-6A9C-3ABF2C8B885E}">
+  <xltc:threadedComment ref="J20" dT="2026-08-13T10:48:46.566" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{BE063722-D0B2-1C17-7A27-F8EBB067EDF8}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-13T10:02:00.586" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{22EA1B97-97F4-0702-6B91-6997A8A60541}">
+  <xltc:threadedComment ref="J21" dT="2026-08-13T10:48:46.569" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{129AC679-C322-7EDF-2D05-F930C01785C1}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-13T10:02:00.591" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{91E43DF2-86A6-66CA-3584-7C3DFE2606FF}">
+  <xltc:threadedComment ref="J22" dT="2026-08-13T10:48:46.571" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{5B59801D-8187-A143-4078-DC34F3DCA574}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-13T10:02:00.594" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{F3741990-9FF5-CD11-7731-E40F9C494305}">
+  <xltc:threadedComment ref="J23" dT="2026-08-13T10:48:46.574" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{5767ABB8-D080-C7E0-276B-CAEA4EBA3D8C}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-13T10:02:00.599" personId="{FAB92DDB-880D-4221-A6A8-E30F82860DC6}" id="{E33182D8-C6FF-D9E9-5B55-36905FD6B5C7}">
+  <xltc:threadedComment ref="J24" dT="2026-08-13T10:48:46.577" personId="{46DDD0B6-2CC7-4EA2-92EA-A0FBB82DA6A8}" id="{B0B1EB2E-B4BB-9060-6D43-CE609EE006EA}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -7802,7 +7802,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ee979a9a747414a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc97ec5767a54952"/>
 </x:worksheet>
 </file>
 
@@ -8862,7 +8862,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f8df8f8f9484c8f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R955eede67e084976"/>
 </x:worksheet>
 </file>
 
@@ -20015,6 +20015,6 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb64f2301ab1848e8"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1b912fd1b004ea9"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Regenerate V3.2 deliverables from the clean commit
Second consecutive build produced an identical gated artifact set:
clean_worktree true, dirty_paths empty, and only the seven self-timestamping
deliverables plus the self-referential manifest rewritten. 18/18 checks.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
+++ b/outputs/audit/Public-Facts-Anchor-Register-V3.1.1.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R0fd3da53c6474eb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="Rae05839ab057421d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="Rb1c4d596084647c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="Rc8317bd219ed4179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="Rc317cd6f360540c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="Rdc21dd7409b249e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R9b5dc4f8bd2a4bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R85bf14222c8345e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rd4ba0bcbaed34017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Red7147dc254a47f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Facts" sheetId="2" r:id="R538457d61b55440f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Coverage" sheetId="3" r:id="R8570bb181e464318"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Anchors" sheetId="4" r:id="R8fba07ff55a944d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Decision Impact" sheetId="5" r:id="Ra2d74081ce854e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Queue" sheetId="6" r:id="R5385c86cbbe54f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rc2e677fc5c724239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R1de2b458adaf4ba7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rb6709aa19e9547d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,88 +18,88 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={A40E139C-450C-2E5A-11A2-84CC2E6500E7}</x:author>
-    <x:author>tc={C7120340-DFAC-0758-37AD-017692481328}</x:author>
-    <x:author>tc={19FB0F36-B006-39A3-CA23-340C32C626E1}</x:author>
-    <x:author>tc={7DF876DF-B50B-B062-508C-140073E397EE}</x:author>
-    <x:author>tc={CE317F38-E135-CAA6-2F8D-581B467DBD51}</x:author>
-    <x:author>tc={8B2FAE9F-DB78-168D-D737-A25F46B49B31}</x:author>
-    <x:author>tc={C53CE978-BB6D-F679-DFFD-1C66BB6961AA}</x:author>
-    <x:author>tc={800C2571-7A93-7D42-D62D-108C1BD9B011}</x:author>
-    <x:author>tc={AA6A20B5-89B8-F7EC-956A-F65B11E30FEA}</x:author>
-    <x:author>tc={AC84A0BF-C857-AD62-C31D-B2496EC05624}</x:author>
-    <x:author>tc={525E74AB-B7B0-3B0C-F386-1D12441BC8AD}</x:author>
-    <x:author>tc={0EB83D38-B901-763B-9E3C-80489E2F258F}</x:author>
-    <x:author>tc={9D22D550-7056-F555-36E4-E270081901C3}</x:author>
-    <x:author>tc={6FC39242-4A03-4B55-A266-E28DAA041BCF}</x:author>
-    <x:author>tc={ACF2B236-B5B7-9588-800C-B3CBA0356402}</x:author>
-    <x:author>tc={B6B85072-9530-6796-5ADE-7BEFF1C441C8}</x:author>
-    <x:author>tc={911F8CD8-A6B4-2B2F-5245-6A4F33BA800F}</x:author>
-    <x:author>tc={DBCD60BF-BDE6-1D40-7765-6DE5112A74C0}</x:author>
-    <x:author>tc={85863BA4-EE75-063E-8400-19F2A2E622C8}</x:author>
-    <x:author>tc={5FB4578F-5F43-A12A-0B75-3B0A7ACEBF27}</x:author>
-    <x:author>tc={C02DEB98-E710-0CAA-9713-A179950CACBC}</x:author>
-    <x:author>tc={767EDA63-D307-79FB-0A54-FC077F25DB0D}</x:author>
-    <x:author>tc={D92ADAB0-3AF5-12EB-3FC5-F40EB3271526}</x:author>
-    <x:author>tc={53553C3E-97F2-9ABC-CC37-494AB6BCF02D}</x:author>
-    <x:author>tc={6E38FFBD-0E69-6F58-C6FB-E525FD293DF7}</x:author>
-    <x:author>tc={655F3035-CEC8-5A77-CC92-C2F5E9B52252}</x:author>
-    <x:author>tc={30B66BD0-10DB-7378-49F9-D6C98554C042}</x:author>
-    <x:author>tc={B96417D9-2317-2961-AC77-42B5707004FE}</x:author>
-    <x:author>tc={ADCB7DD4-3F5D-D119-F707-76ACBFF2193B}</x:author>
-    <x:author>tc={0325D8E4-95B0-0D83-6D59-1D9D067D75B0}</x:author>
-    <x:author>tc={A4F4BEF0-90E9-3AEB-EBFB-C11160520E96}</x:author>
-    <x:author>tc={C482A02C-8CFA-6034-9C21-DAB786CDA651}</x:author>
-    <x:author>tc={F3F412F1-0B3C-5A2F-D1E8-4685104B0B45}</x:author>
-    <x:author>tc={EEE74F05-B71A-BE53-1CFF-3932D68FACC4}</x:author>
-    <x:author>tc={46105A14-3CDC-4A8F-B1BF-06CB9FB80081}</x:author>
-    <x:author>tc={7334A953-B784-7069-115C-43FBCC52D86F}</x:author>
-    <x:author>tc={28CAEF51-DFBA-B4DF-D2E0-F72213D92EA6}</x:author>
-    <x:author>tc={0F11B26E-2953-49FC-F3BC-1945E211EF79}</x:author>
-    <x:author>tc={631A80DD-A75D-A0CB-9AE3-12FEE87B6C2B}</x:author>
-    <x:author>tc={BFAEBF46-5285-4C0F-563E-0D6F87CC58E7}</x:author>
-    <x:author>tc={6B6AB023-6B38-679B-1FEE-43FF97795296}</x:author>
-    <x:author>tc={B1A57EBE-1BE2-4102-B718-572EBD18D0A4}</x:author>
-    <x:author>tc={A45A8206-B2AC-29BF-D77C-CA5A906B4F7C}</x:author>
-    <x:author>tc={6E37C73B-A8C4-C43C-A2A6-FFA8463C73D2}</x:author>
-    <x:author>tc={19A2F6BD-7CB4-2C59-A575-252DFE6CBDA1}</x:author>
-    <x:author>tc={C3B91BCB-60CC-DB85-5D4A-2C23E9A2D283}</x:author>
-    <x:author>tc={31F47784-7570-C70A-A35E-9BF8BD2BA136}</x:author>
-    <x:author>tc={DB619A28-DDF9-7479-C215-B93C16646AE8}</x:author>
-    <x:author>tc={E5B0B5DF-32CA-1D43-F4D9-19AAA5B3C3D9}</x:author>
-    <x:author>tc={4FEAD983-C9AF-020C-0FD9-0C992540078A}</x:author>
-    <x:author>tc={2B524F18-D1CE-AF7B-C358-C78C59B36DB4}</x:author>
-    <x:author>tc={8686BF4A-E392-0E4F-A3D5-3ED5E4DD158C}</x:author>
-    <x:author>tc={1E74F05A-28D7-D9BC-C7ED-7346333DEA2B}</x:author>
-    <x:author>tc={926DFEF5-00A6-A680-41A8-C644471622DF}</x:author>
-    <x:author>tc={BE769349-C898-8EA5-79AC-F549F4509D0E}</x:author>
-    <x:author>tc={80F4D301-AEA1-8FD2-B7C9-DB216A35861D}</x:author>
-    <x:author>tc={82D9D992-0103-7597-FFDF-242192E93C3C}</x:author>
-    <x:author>tc={7E74EB64-38FB-DDD6-B3B4-382303B94AA5}</x:author>
-    <x:author>tc={9051500E-1BA8-EBD8-ED1C-50B06B90E871}</x:author>
-    <x:author>tc={285852A2-EB14-2F7D-D258-78E3A0414F47}</x:author>
-    <x:author>tc={EAD34261-3B5A-4AEE-6805-DCAF229D62C7}</x:author>
-    <x:author>tc={D94799C8-2A43-8D0D-6424-92B7F7D022AD}</x:author>
-    <x:author>tc={DB823940-58F7-72CA-E976-C2BA9A93ECB5}</x:author>
-    <x:author>tc={42ECDCF3-F215-2900-0E9F-99C2F29365D8}</x:author>
-    <x:author>tc={AE221677-12CC-2217-0A5A-5778CC9E1300}</x:author>
-    <x:author>tc={E22D7C22-4DCF-DE41-3F3A-DC295E520744}</x:author>
-    <x:author>tc={E7E49E75-DA38-4B2B-BE4D-F50AAC24860B}</x:author>
-    <x:author>tc={FE69C779-91C2-0E7E-858C-EA96B0EBCE08}</x:author>
-    <x:author>tc={4A416B06-99B7-E437-F3E2-8405A0D98BD3}</x:author>
-    <x:author>tc={9E6F027E-2267-CDE0-0603-674413B70DB3}</x:author>
-    <x:author>tc={02028335-A1F8-F064-D740-6BE027A923FB}</x:author>
-    <x:author>tc={3A89FC5C-0D61-FA33-BA8F-339ABE0912A2}</x:author>
-    <x:author>tc={8FCBCB03-0DFC-1AFE-EB17-F427276BA20F}</x:author>
-    <x:author>tc={77A6E231-21AE-F66D-D211-164FBB2E8DED}</x:author>
-    <x:author>tc={7D22A3F2-D4C9-7EBE-4C36-A5E564D099FA}</x:author>
-    <x:author>tc={6F104F1D-84C3-0FB9-8885-5F4D48531871}</x:author>
-    <x:author>tc={FCCBBFA1-24E0-2ECE-EB37-806DB36AC90C}</x:author>
-    <x:author>tc={AB7C2528-F367-AFFE-4205-1F9DD2C6F441}</x:author>
-    <x:author>tc={1C4365EB-7A12-19EB-6F23-09BF7854F864}</x:author>
-    <x:author>tc={3F03CB66-095C-3404-E5AE-B8B563887750}</x:author>
-    <x:author>tc={E6D42EC5-8BE4-DB23-356E-E8975A92AF6F}</x:author>
-    <x:author>tc={77C690BB-D307-3F3C-26FD-4F2712DC5136}</x:author>
+    <x:author>tc={690181E6-AE14-9913-C612-A6DA423575B9}</x:author>
+    <x:author>tc={6C1DEEEA-0004-47FE-65ED-DE6EC665703B}</x:author>
+    <x:author>tc={A4AF04D7-281F-AC4F-E4BE-74D75B6842E3}</x:author>
+    <x:author>tc={60781879-7FBA-69D0-78C8-BF9ECF9DE9D3}</x:author>
+    <x:author>tc={999156F6-43BB-F8B0-6282-33286AD78759}</x:author>
+    <x:author>tc={2328DED2-E989-51F3-5788-F80996AAC5B0}</x:author>
+    <x:author>tc={F233D94C-49F3-2C60-8C84-24D6505AF417}</x:author>
+    <x:author>tc={79613A44-8164-42BA-18B7-0C6F477443AA}</x:author>
+    <x:author>tc={E93EE893-01B7-3B84-F6C2-4A8773453090}</x:author>
+    <x:author>tc={9253FC64-C2F3-3B4B-CA95-1050937028F2}</x:author>
+    <x:author>tc={D7331CEC-91E2-F308-9D23-0149AE0923BB}</x:author>
+    <x:author>tc={1ED6BE11-E32C-BFB2-3618-FF16C03C01DF}</x:author>
+    <x:author>tc={C32EB202-30C1-74D3-CA0D-00FBB3887851}</x:author>
+    <x:author>tc={CCD66828-D507-3941-8FDE-C1C024610DB6}</x:author>
+    <x:author>tc={53579FA4-A2BF-0514-DE57-9920FF3684B9}</x:author>
+    <x:author>tc={336AC136-CE80-E3AC-DD9E-B490B8FB1529}</x:author>
+    <x:author>tc={F89E09ED-3F3D-DDF3-BF8E-54F72E11F5AE}</x:author>
+    <x:author>tc={62873C05-7078-14AC-4870-A0B36C074EC0}</x:author>
+    <x:author>tc={911754FB-7BA4-1326-8162-A70E5294E261}</x:author>
+    <x:author>tc={CC1AA7DD-89F7-220C-FA7F-4B303EADEA0D}</x:author>
+    <x:author>tc={2BB3CFB4-F980-4B4B-FD1F-93BAB256EEA2}</x:author>
+    <x:author>tc={CF849447-A81D-2BF2-DC5A-0E92B85A8E7A}</x:author>
+    <x:author>tc={40975AC3-4F1D-12DA-F17C-EE19FAD8F8E8}</x:author>
+    <x:author>tc={C49F8C3E-9C99-D905-0CDD-2BDDDA31328A}</x:author>
+    <x:author>tc={25E36FF7-90DA-2C15-3B67-2EC9F9911E77}</x:author>
+    <x:author>tc={0DF2E3D6-1151-0820-D1BF-E7D42DD2F512}</x:author>
+    <x:author>tc={90433ED7-F595-F28F-0081-7E8582CD5033}</x:author>
+    <x:author>tc={3438016A-878B-B90B-DF8E-578C29AB409A}</x:author>
+    <x:author>tc={6F07FD29-1751-108A-C18E-01A5B7A885F7}</x:author>
+    <x:author>tc={55908B64-4BF6-359B-C8F1-A81148F8B75C}</x:author>
+    <x:author>tc={6390E830-1DA7-C1BC-353F-AF7EDBAAC1D0}</x:author>
+    <x:author>tc={85B11369-F366-15E6-3B72-C90B27E2AE15}</x:author>
+    <x:author>tc={E6E0E485-9324-74B9-24C6-521E999E7F4B}</x:author>
+    <x:author>tc={E3501298-7B65-6B2F-51C7-0C60132CBB22}</x:author>
+    <x:author>tc={F515B0A9-323F-D63A-965B-9DED8BC0CEEC}</x:author>
+    <x:author>tc={D99CE189-1A18-515C-8C8B-3EDFC451755F}</x:author>
+    <x:author>tc={CF14C768-414F-3033-3897-89CCCC5323DA}</x:author>
+    <x:author>tc={1DD90BE6-4CF0-4F5A-BB70-09CF2695C172}</x:author>
+    <x:author>tc={7CEFD05C-8A95-0B2C-4D6E-B1ED289FE9B9}</x:author>
+    <x:author>tc={513E7AB3-89CC-8103-AADE-F8099C233B47}</x:author>
+    <x:author>tc={7ED69721-931A-3600-458A-4FEF9C54A5F4}</x:author>
+    <x:author>tc={5694288F-399C-DB8E-5CFF-15D27083DC07}</x:author>
+    <x:author>tc={1474DEB2-992A-CD29-870F-EC301F80779D}</x:author>
+    <x:author>tc={0629F531-4F0E-174E-08FA-0F0CE4B88C37}</x:author>
+    <x:author>tc={CCC7088B-0D89-F0E7-5758-AFCC02615445}</x:author>
+    <x:author>tc={440B5151-885B-CA76-5F1D-55E01036679B}</x:author>
+    <x:author>tc={A8AF2223-9342-CC44-020C-A66C4A7CA94C}</x:author>
+    <x:author>tc={4030A7C1-CD2F-276F-FE5D-FB5D27013441}</x:author>
+    <x:author>tc={002AF734-66B0-79A2-66DD-F286A908C60C}</x:author>
+    <x:author>tc={C82E0938-7D4D-C994-5FFA-B4F0329EDA14}</x:author>
+    <x:author>tc={99E9F44C-9786-33CE-BC34-AD4A3E755777}</x:author>
+    <x:author>tc={0CC656E7-50D8-AA8E-233E-47A999C5DF67}</x:author>
+    <x:author>tc={73A442B9-33BE-1B29-CBBB-A1B73A345A2B}</x:author>
+    <x:author>tc={EB65E9B3-6640-FC5B-FA53-0A5C06426B54}</x:author>
+    <x:author>tc={787BBB27-B36A-60EF-DA64-F9BAE245CE7A}</x:author>
+    <x:author>tc={EF7F3B93-3B57-D877-7BE2-DFBD9FE6BFB5}</x:author>
+    <x:author>tc={05AE0EA1-0F0B-73C8-62E6-370FE555D9DC}</x:author>
+    <x:author>tc={FC4B743F-C0B9-183B-7162-518AFC4AE12F}</x:author>
+    <x:author>tc={2F1BC2C6-A97F-5195-1FCC-3BB39DCFE62D}</x:author>
+    <x:author>tc={0347AF34-0611-3519-8170-746B07699079}</x:author>
+    <x:author>tc={42058C14-2FDF-66C6-354C-6A599D4AD350}</x:author>
+    <x:author>tc={387BF00F-88FD-86D6-94F0-60907880BF19}</x:author>
+    <x:author>tc={41A1CB82-8A76-F07F-CB16-8F6A76A6AFEA}</x:author>
+    <x:author>tc={4520C69F-2A35-2A51-EEA0-5DDB09087C14}</x:author>
+    <x:author>tc={B4E2105E-2831-0460-E431-6C9D805D6DC7}</x:author>
+    <x:author>tc={B39B1996-0E18-2F2E-4F40-62B03F693537}</x:author>
+    <x:author>tc={3BC87D96-B05B-8958-635E-C66826D394C6}</x:author>
+    <x:author>tc={932C1101-2A3F-64AF-ED02-2D8ED89CB61A}</x:author>
+    <x:author>tc={B6F2A0CA-BCC7-966B-7269-57969A66E25D}</x:author>
+    <x:author>tc={841D9532-9692-B359-CF19-2ACA98571B14}</x:author>
+    <x:author>tc={F75A9377-1A94-2807-65F9-DFE2D0B0C564}</x:author>
+    <x:author>tc={D651B341-8017-6F43-7D13-1F6A2E0CE639}</x:author>
+    <x:author>tc={019574C1-C2D6-9D01-1B09-92C44D8919B4}</x:author>
+    <x:author>tc={B82CD612-1083-092D-25AF-7DDFE2C12C63}</x:author>
+    <x:author>tc={43827401-9729-C2F4-B538-74E267729C46}</x:author>
+    <x:author>tc={5E336747-0123-6D4A-458B-9EC79815C379}</x:author>
+    <x:author>tc={E8A42772-0744-BB49-C6CD-22184FA6F8F7}</x:author>
+    <x:author>tc={F8BABEF1-219F-5AA2-A49A-3A48153CD84C}</x:author>
+    <x:author>tc={4C4BADA7-DC39-C76C-6638-783DFC1781C8}</x:author>
+    <x:author>tc={DF837794-31DD-20EF-599F-45523E2B054D}</x:author>
+    <x:author>tc={FCA8385D-924A-F8F3-4270-0FB7532DF3F7}</x:author>
+    <x:author>tc={6D538EC1-799B-2E21-B797-837119C99EEA}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="P5" authorId="0">
@@ -1175,26 +1175,26 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={056BFFBA-1801-631C-3654-01E2B2FEFFA1}</x:author>
-    <x:author>tc={AEB35E22-B146-E986-D70B-680EB7EBA741}</x:author>
-    <x:author>tc={1A66EC80-39A8-BBFD-3F0B-A8FB8A71076C}</x:author>
-    <x:author>tc={283BC70E-764F-9D7D-76D2-C1E754232E7C}</x:author>
-    <x:author>tc={2B4D5C58-7CC8-8965-AE53-FAF3E77DF125}</x:author>
-    <x:author>tc={CE85C480-8E26-EFF5-D7AE-A1C07D9B98B6}</x:author>
-    <x:author>tc={41BEFA26-1CA3-717B-C25E-6FAF19367372}</x:author>
-    <x:author>tc={253A4618-3510-1622-74B0-CB88D82A95CF}</x:author>
-    <x:author>tc={FD8FC314-3FE9-7295-B95C-749D9AF03F40}</x:author>
-    <x:author>tc={A542688D-10E7-AC16-BF62-7C9420A0CB6A}</x:author>
-    <x:author>tc={DDCCE20C-D9C3-F33C-99F1-3542159C292B}</x:author>
-    <x:author>tc={7A8C311B-1177-37FC-55E5-7BA1626253B4}</x:author>
-    <x:author>tc={3A2B0191-F99E-961A-C5FA-AB373DECB115}</x:author>
-    <x:author>tc={94B90196-28B0-BBF4-EDB3-1D42F95D11F5}</x:author>
-    <x:author>tc={2C5D4759-15DC-9CF4-A10A-E4DD2B0C28D8}</x:author>
-    <x:author>tc={D5163183-B337-0253-F177-61E462FF999F}</x:author>
-    <x:author>tc={8DD6D4F6-BF6F-3D9B-E666-BF8235FA60E3}</x:author>
-    <x:author>tc={560957A6-2914-F33B-FDC5-B3985B6BD162}</x:author>
-    <x:author>tc={7CE10764-0905-1DAA-5C75-9DF0DAAB717E}</x:author>
-    <x:author>tc={6F155B2F-3B59-BFE4-A5D9-BA0F24D73EBE}</x:author>
+    <x:author>tc={03358198-A18A-0637-AE13-2EBB49B74CCB}</x:author>
+    <x:author>tc={16E09466-770F-DC6D-B8AE-5F56C968BC0B}</x:author>
+    <x:author>tc={5A87A16A-54A6-6A4A-A716-713CF075763C}</x:author>
+    <x:author>tc={51A5BCFB-330F-5404-5AB5-4D111557355C}</x:author>
+    <x:author>tc={31BFA9BA-FEBF-C930-7B72-05A92515189D}</x:author>
+    <x:author>tc={6FFA8427-BE49-9BF8-DACD-0E54AF69D979}</x:author>
+    <x:author>tc={4D05509C-70F1-DB4D-9D32-2F454F56A4A8}</x:author>
+    <x:author>tc={1BCE242B-A16F-D35F-0139-0CACF590FBE4}</x:author>
+    <x:author>tc={788A8C39-4C7F-5DDF-B66C-0C91073C4346}</x:author>
+    <x:author>tc={8FF0089B-7903-3B52-0C52-781D7BBE47A3}</x:author>
+    <x:author>tc={ABFFBA4E-13E6-F46E-1003-C8FC3BFC4E41}</x:author>
+    <x:author>tc={DE42D7FF-E748-9CEF-9DA2-741C9C7F4306}</x:author>
+    <x:author>tc={11EEA32B-D415-FB31-AE8E-2F237C5305B9}</x:author>
+    <x:author>tc={F3491057-0054-94D5-4F22-2DB6E419570E}</x:author>
+    <x:author>tc={9CF4DCE5-1115-069E-5C9B-6BE71474B259}</x:author>
+    <x:author>tc={D4B87D3D-C97C-5223-C7A2-F8BBDAD3F1A4}</x:author>
+    <x:author>tc={F5AF6B59-C1F3-82DA-AEBC-95BE9980CBFA}</x:author>
+    <x:author>tc={5CAEF3D3-B404-BE2E-09F3-6E792A945106}</x:author>
+    <x:author>tc={4A9BBAB3-4446-5BA9-62A0-A9F3F0ADDC81}</x:author>
+    <x:author>tc={E5CBD345-6B49-A62D-9E0C-20D78646AABD}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="J5" authorId="0">
@@ -2037,7 +2037,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R136e50952cde4c52"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R418f6472e70b4eb9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2048,7 +2048,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}"/>
+  <xltc:person displayName="Corporate Wallet Digital Twin V3.1.1" id="{9DFC5A97-C476-4693-ACBE-129047B28BFB}"/>
 </xltc:personList>
 </file>
 
@@ -2245,493 +2245,493 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="P5" dT="2026-08-14T10:54:56.935" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{A40E139C-450C-2E5A-11A2-84CC2E6500E7}">
+  <xltc:threadedComment ref="P5" dT="2026-08-14T11:00:52.348" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{690181E6-AE14-9913-C612-A6DA423575B9}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P6" dT="2026-08-14T10:54:56.941" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{C7120340-DFAC-0758-37AD-017692481328}">
+  <xltc:threadedComment ref="P6" dT="2026-08-14T11:00:52.35" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{6C1DEEEA-0004-47FE-65ED-DE6EC665703B}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P7" dT="2026-08-14T10:54:56.941" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{19FB0F36-B006-39A3-CA23-340C32C626E1}">
+  <xltc:threadedComment ref="P7" dT="2026-08-14T11:00:52.35" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{A4AF04D7-281F-AC4F-E4BE-74D75B6842E3}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P8" dT="2026-08-14T10:54:56.941" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{7DF876DF-B50B-B062-508C-140073E397EE}">
+  <xltc:threadedComment ref="P8" dT="2026-08-14T11:00:52.35" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{60781879-7FBA-69D0-78C8-BF9ECF9DE9D3}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P9" dT="2026-08-14T10:54:56.941" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{CE317F38-E135-CAA6-2F8D-581B467DBD51}">
+  <xltc:threadedComment ref="P9" dT="2026-08-14T11:00:52.35" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{999156F6-43BB-F8B0-6282-33286AD78759}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P10" dT="2026-08-14T10:54:56.942" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{8B2FAE9F-DB78-168D-D737-A25F46B49B31}">
+  <xltc:threadedComment ref="P10" dT="2026-08-14T11:00:52.35" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{2328DED2-E989-51F3-5788-F80996AAC5B0}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 119
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P11" dT="2026-08-14T10:54:56.942" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{C53CE978-BB6D-F679-DFFD-1C66BB6961AA}">
+  <xltc:threadedComment ref="P11" dT="2026-08-14T11:00:52.35" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{F233D94C-49F3-2C60-8C84-24D6505AF417}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 160
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P12" dT="2026-08-14T10:54:56.942" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{800C2571-7A93-7D42-D62D-108C1BD9B011}">
+  <xltc:threadedComment ref="P12" dT="2026-08-14T11:00:52.35" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{79613A44-8164-42BA-18B7-0C6F477443AA}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P13" dT="2026-08-14T10:54:56.942" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{AA6A20B5-89B8-F7EC-956A-F65B11E30FEA}">
+  <xltc:threadedComment ref="P13" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{E93EE893-01B7-3B84-F6C2-4A8773453090}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 139
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P14" dT="2026-08-14T10:54:56.942" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{AC84A0BF-C857-AD62-C31D-B2496EC05624}">
+  <xltc:threadedComment ref="P14" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{9253FC64-C2F3-3B4B-CA95-1050937028F2}">
     <xltc:text>Source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf
 Page: 118
 Available: 2025-08-19
 SHA-256: seed-register-hash:BHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P15" dT="2026-08-14T10:54:56.942" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{525E74AB-B7B0-3B0C-F386-1D12441BC8AD}">
+  <xltc:threadedComment ref="P15" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{D7331CEC-91E2-F308-9D23-0149AE0923BB}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P16" dT="2026-08-14T10:54:56.942" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{0EB83D38-B901-763B-9E3C-80489E2F258F}">
+  <xltc:threadedComment ref="P16" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{1ED6BE11-E32C-BFB2-3618-FF16C03C01DF}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 205
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P17" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{9D22D550-7056-F555-36E4-E270081901C3}">
+  <xltc:threadedComment ref="P17" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{C32EB202-30C1-74D3-CA0D-00FBB3887851}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P18" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{6FC39242-4A03-4B55-A266-E28DAA041BCF}">
+  <xltc:threadedComment ref="P18" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{CCD66828-D507-3941-8FDE-C1C024610DB6}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 186
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P19" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{ACF2B236-B5B7-9588-800C-B3CBA0356402}">
+  <xltc:threadedComment ref="P19" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{53579FA4-A2BF-0514-DE57-9920FF3684B9}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P20" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{B6B85072-9530-6796-5ADE-7BEFF1C441C8}">
+  <xltc:threadedComment ref="P20" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{336AC136-CE80-E3AC-DD9E-B490B8FB1529}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 138
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P21" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{911F8CD8-A6B4-2B2F-5245-6A4F33BA800F}">
+  <xltc:threadedComment ref="P21" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{F89E09ED-3F3D-DDF3-BF8E-54F72E11F5AE}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 212
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P22" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{DBCD60BF-BDE6-1D40-7765-6DE5112A74C0}">
+  <xltc:threadedComment ref="P22" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{62873C05-7078-14AC-4870-A0B36C074EC0}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P23" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{85863BA4-EE75-063E-8400-19F2A2E622C8}">
+  <xltc:threadedComment ref="P23" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{911754FB-7BA4-1326-8162-A70E5294E261}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 185
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P24" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{5FB4578F-5F43-A12A-0B75-3B0A7ACEBF27}">
+  <xltc:threadedComment ref="P24" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{CC1AA7DD-89F7-220C-FA7F-4B303EADEA0D}">
     <xltc:text>Source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf
 Page: 136
 Available: 2026-03-10
 SHA-256: seed-register-hash:GLEN-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P25" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{C02DEB98-E710-0CAA-9713-A179950CACBC}">
+  <xltc:threadedComment ref="P25" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{2BB3CFB4-F980-4B4B-FD1F-93BAB256EEA2}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P26" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{767EDA63-D307-79FB-0A54-FC077F25DB0D}">
+  <xltc:threadedComment ref="P26" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{CF849447-A81D-2BF2-DC5A-0E92B85A8E7A}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 274
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P27" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{D92ADAB0-3AF5-12EB-3FC5-F40EB3271526}">
+  <xltc:threadedComment ref="P27" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{40975AC3-4F1D-12DA-F17C-EE19FAD8F8E8}">
     <xltc:text>Source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf
 Page: 272
 Available: 2026-03-02
 SHA-256: 362b9ebb43ca8ce3cf0a87f5ba174047ab499c4cd8f5a48eeb1bf83530a176fb</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P28" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{53553C3E-97F2-9ABC-CC37-494AB6BCF02D}">
+  <xltc:threadedComment ref="P28" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{C49F8C3E-9C99-D905-0CDD-2BDDDA31328A}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P29" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{6E38FFBD-0E69-6F58-C6FB-E525FD293DF7}">
+  <xltc:threadedComment ref="P29" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{25E36FF7-90DA-2C15-3B67-2EC9F9911E77}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 160
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P30" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{655F3035-CEC8-5A77-CC92-C2F5E9B52252}">
+  <xltc:threadedComment ref="P30" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{0DF2E3D6-1151-0820-D1BF-E7D42DD2F512}">
     <xltc:text>Source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf
 Page: 158
 Available: 2026-03-26
 SHA-256: 958d89150d1125af3eb9032ac7f3c9da2c22c8bfd67e8447c688c8ad0c21dd35</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P31" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{30B66BD0-10DB-7378-49F9-D6C98554C042}">
+  <xltc:threadedComment ref="P31" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{90433ED7-F595-F28F-0081-7E8582CD5033}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P32" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{B96417D9-2317-2961-AC77-42B5707004FE}">
+  <xltc:threadedComment ref="P32" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{3438016A-878B-B90B-DF8E-578C29AB409A}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 74
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P33" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{ADCB7DD4-3F5D-D119-F707-76ACBFF2193B}">
+  <xltc:threadedComment ref="P33" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{6F07FD29-1751-108A-C18E-01A5B7A885F7}">
     <xltc:text>Source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf
 Page: 72
 Available: 2026-03-27
 SHA-256: 0819d8e37085aaa5adb8305c3bcdd5b5a9631cf40f594950beaeb6c77077fc0a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P34" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{0325D8E4-95B0-0D83-6D59-1D9D067D75B0}">
+  <xltc:threadedComment ref="P34" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{55908B64-4BF6-359B-C8F1-A81148F8B75C}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P35" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{A4F4BEF0-90E9-3AEB-EBFB-C11160520E96}">
+  <xltc:threadedComment ref="P35" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{6390E830-1DA7-C1BC-353F-AF7EDBAAC1D0}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 25
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P36" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{C482A02C-8CFA-6034-9C21-DAB786CDA651}">
+  <xltc:threadedComment ref="P36" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{85B11369-F366-15E6-3B72-C90B27E2AE15}">
     <xltc:text>Source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf
 Page: 24
 Available: 2026-03-27
 SHA-256: 84ab45295a07c93d3fa39a24962c05ac600f45ed2c9683b16b4dc2cc7ba170f8</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P37" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{F3F412F1-0B3C-5A2F-D1E8-4685104B0B45}">
+  <xltc:threadedComment ref="P37" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{E6E0E485-9324-74B9-24C6-521E999E7F4B}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P38" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{EEE74F05-B71A-BE53-1CFF-3932D68FACC4}">
+  <xltc:threadedComment ref="P38" dT="2026-08-14T11:00:52.351" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{E3501298-7B65-6B2F-51C7-0C60132CBB22}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P39" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{46105A14-3CDC-4A8F-B1BF-06CB9FB80081}">
+  <xltc:threadedComment ref="P39" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{F515B0A9-323F-D63A-965B-9DED8BC0CEEC}">
     <xltc:text>Source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf
 Page: 19
 Available: 2025-09-15
 SHA-256: 3f03545e101a357d73e3f26863473adc341b4b0382ab2b8248b322900ef38b3c</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P40" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{7334A953-B784-7069-115C-43FBCC52D86F}">
+  <xltc:threadedComment ref="P40" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{D99CE189-1A18-515C-8C8B-3EDFC451755F}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P41" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{28CAEF51-DFBA-B4DF-D2E0-F72213D92EA6}">
+  <xltc:threadedComment ref="P41" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{CF14C768-414F-3033-3897-89CCCC5323DA}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P42" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{0F11B26E-2953-49FC-F3BC-1945E211EF79}">
+  <xltc:threadedComment ref="P42" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{1DD90BE6-4CF0-4F5A-BB70-09CF2695C172}">
     <xltc:text>Source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf
 Page: 42
 Available: 2025-03-07
 SHA-256: fc2487f72420917e9c52f78bc4a7800a1e4270781aa2117632f69680b4ca14da</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P43" dT="2026-08-14T10:54:56.943" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{631A80DD-A75D-A0CB-9AE3-12FEE87B6C2B}">
+  <xltc:threadedComment ref="P43" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{7CEFD05C-8A95-0B2C-4D6E-B1ED289FE9B9}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P44" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{BFAEBF46-5285-4C0F-563E-0D6F87CC58E7}">
+  <xltc:threadedComment ref="P44" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{513E7AB3-89CC-8103-AADE-F8099C233B47}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AP-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P45" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{6B6AB023-6B38-679B-1FEE-43FF97795296}">
+  <xltc:threadedComment ref="P45" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{7ED69721-931A-3600-458A-4FEF9C54A5F4}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P46" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{B1A57EBE-1BE2-4102-B718-572EBD18D0A4}">
+  <xltc:threadedComment ref="P46" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{5694288F-399C-DB8E-5CFF-15D27083DC07}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-AR-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P47" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{A45A8206-B2AC-29BF-D77C-CA5A906B4F7C}">
+  <xltc:threadedComment ref="P47" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{1474DEB2-992A-CD29-870F-EC301F80779D}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-COST</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P48" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{6E37C73B-A8C4-C43C-A2A6-FFA8463C73D2}">
+  <xltc:threadedComment ref="P48" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{0629F531-4F0E-174E-08FA-0F0CE4B88C37}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-DEBT</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P49" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{19A2F6BD-7CB4-2C59-A575-252DFE6CBDA1}">
+  <xltc:threadedComment ref="P49" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{CCC7088B-0D89-F0E7-5758-AFCC02615445}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 118
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-FX</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P50" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{C3B91BCB-60CC-DB85-5D4A-2C23E9A2D283}">
+  <xltc:threadedComment ref="P50" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{440B5151-885B-CA76-5F1D-55E01036679B}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-CLOSE</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P51" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{31F47784-7570-C70A-A35E-9BF8BD2BA136}">
+  <xltc:threadedComment ref="P51" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{A8AF2223-9342-CC44-020C-A66C4A7CA94C}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-INV-OPEN</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P52" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{DB619A28-DDF9-7479-C215-B93C16646AE8}">
+  <xltc:threadedComment ref="P52" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{4030A7C1-CD2F-276F-FE5D-FB5D27013441}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 19
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-REV</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P53" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{E5B0B5DF-32CA-1D43-F4D9-19AAA5B3C3D9}">
+  <xltc:threadedComment ref="P53" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{002AF734-66B0-79A2-66DD-F286A908C60C}">
     <xltc:text>Source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf
 Page: 18
 Available: 2025-10-13
 SHA-256: seed-register-hash:SHP-2025-STF</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P54" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{4FEAD983-C9AF-020C-0FD9-0C992540078A}">
+  <xltc:threadedComment ref="P54" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{C82E0938-7D4D-C994-5FFA-B4F0329EDA14}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P55" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{2B524F18-D1CE-AF7B-C358-C78C59B36DB4}">
+  <xltc:threadedComment ref="P55" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{99E9F44C-9786-33CE-BC34-AD4A3E755777}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 19
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P56" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{8686BF4A-E392-0E4F-A3D5-3ED5E4DD158C}">
+  <xltc:threadedComment ref="P56" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{0CC656E7-50D8-AA8E-233E-47A999C5DF67}">
     <xltc:text>Source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf
 Page: 18
 Available: 2025-10-30
 SHA-256: f2516d780aff52d4a5de8be9a2f02e753e948e13450e77f2b1603784b5215c9f</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P57" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{1E74F05A-28D7-D9BC-C7ED-7346333DEA2B}">
+  <xltc:threadedComment ref="P57" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{73A442B9-33BE-1B29-CBBB-A1B73A345A2B}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P58" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{926DFEF5-00A6-A680-41A8-C644471622DF}">
+  <xltc:threadedComment ref="P58" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{EB65E9B3-6640-FC5B-FA53-0A5C06426B54}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 23
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P59" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{BE769349-C898-8EA5-79AC-F549F4509D0E}">
+  <xltc:threadedComment ref="P59" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{787BBB27-B36A-60EF-DA64-F9BAE245CE7A}">
     <xltc:text>Source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf
 Page: 21
 Available: 2025-12-15
 SHA-256: 7715894a86e0e6b06b26b90b6e5bad3ffb85b8cd6166701bf52ddf8e053193d3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P60" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{80F4D301-AEA1-8FD2-B7C9-DB216A35861D}">
+  <xltc:threadedComment ref="P60" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{EF7F3B93-3B57-D877-7BE2-DFBD9FE6BFB5}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P61" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{82D9D992-0103-7597-FFDF-242192E93C3C}">
+  <xltc:threadedComment ref="P61" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{05AE0EA1-0F0B-73C8-62E6-370FE555D9DC}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P62" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{7E74EB64-38FB-DDD6-B3B4-382303B94AA5}">
+  <xltc:threadedComment ref="P62" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{FC4B743F-C0B9-183B-7162-518AFC4AE12F}">
     <xltc:text>Source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf
 Page: 10
 Available: 2025-11-06
 SHA-256: 664c3ce033c0d36157277ae5ef9f28a933edd4acebc8cec649069cd20d9c576d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P63" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{9051500E-1BA8-EBD8-ED1C-50B06B90E871}">
+  <xltc:threadedComment ref="P63" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{2F1BC2C6-A97F-5195-1FCC-3BB39DCFE62D}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P64" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{285852A2-EB14-2F7D-D258-78E3A0414F47}">
+  <xltc:threadedComment ref="P64" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{0347AF34-0611-3519-8170-746B07699079}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 310
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P65" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{EAD34261-3B5A-4AEE-6805-DCAF229D62C7}">
+  <xltc:threadedComment ref="P65" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{42058C14-2FDF-66C6-354C-6A599D4AD350}">
     <xltc:text>Source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf
 Page: 311
 Available: 2026-03-18
 SHA-256: 4124bee2bfb55a181cda56963bd733605a2cc53a7882b1d6108358b33da479f3</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P66" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{D94799C8-2A43-8D0D-6424-92B7F7D022AD}">
+  <xltc:threadedComment ref="P66" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{387BF00F-88FD-86D6-94F0-60907880BF19}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P67" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{DB823940-58F7-72CA-E976-C2BA9A93ECB5}">
+  <xltc:threadedComment ref="P67" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{41A1CB82-8A76-F07F-CB16-8F6A76A6AFEA}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 140
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P68" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{42ECDCF3-F215-2900-0E9F-99C2F29365D8}">
+  <xltc:threadedComment ref="P68" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{4520C69F-2A35-2A51-EEA0-5DDB09087C14}">
     <xltc:text>Source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf
 Page: 141
 Available: 2026-06-29
 SHA-256: 3ea6278d374118f72fe41ac635d4b622bc1b59be44f5db9c0a7bc321ceabf077</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P69" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{AE221677-12CC-2217-0A5A-5778CC9E1300}">
+  <xltc:threadedComment ref="P69" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{B4E2105E-2831-0460-E431-6C9D805D6DC7}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P70" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{E22D7C22-4DCF-DE41-3F3A-DC295E520744}">
+  <xltc:threadedComment ref="P70" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{B39B1996-0E18-2F2E-4F40-62B03F693537}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 32
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P71" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{E7E49E75-DA38-4B2B-BE4D-F50AAC24860B}">
+  <xltc:threadedComment ref="P71" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{3BC87D96-B05B-8958-635E-C66826D394C6}">
     <xltc:text>Source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf
 Page: 33
 Available: 2026-06-29
 SHA-256: e0d23733f611c2b81f2b8c7362c492178fe52b3109472db1e08efe824298f17b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P72" dT="2026-08-14T10:54:56.944" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{FE69C779-91C2-0E7E-858C-EA96B0EBCE08}">
+  <xltc:threadedComment ref="P72" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{932C1101-2A3F-64AF-ED02-2D8ED89CB61A}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P73" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{4A416B06-99B7-E437-F3E2-8405A0D98BD3}">
+  <xltc:threadedComment ref="P73" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{B6F2A0CA-BCC7-966B-7269-57969A66E25D}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 23
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P74" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{9E6F027E-2267-CDE0-0603-674413B70DB3}">
+  <xltc:threadedComment ref="P74" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{841D9532-9692-B359-CF19-2ACA98571B14}">
     <xltc:text>Source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf
 Page: 21
 Available: 2026-03-16
 SHA-256: bea72f5adefd24ecb4dd8ed36e523730e19a3efb2fa9f79b63567bc4fac2e59b</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P75" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{02028335-A1F8-F064-D740-6BE027A923FB}">
+  <xltc:threadedComment ref="P75" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{F75A9377-1A94-2807-65F9-DFE2D0B0C564}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P76" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{3A89FC5C-0D61-FA33-BA8F-339ABE0912A2}">
+  <xltc:threadedComment ref="P76" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{D651B341-8017-6F43-7D13-1F6A2E0CE639}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 21
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P77" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{8FCBCB03-0DFC-1AFE-EB17-F427276BA20F}">
+  <xltc:threadedComment ref="P77" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{019574C1-C2D6-9D01-1B09-92C44D8919B4}">
     <xltc:text>Source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf
 Page: 19
 Available: 2026-06-12
 SHA-256: d6f149d15a1e7a0edc82acd536f2d59644e2c9acce621a65878aa322390fd896</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P78" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{77A6E231-21AE-F66D-D211-164FBB2E8DED}">
+  <xltc:threadedComment ref="P78" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{B82CD612-1083-092D-25AF-7DDFE2C12C63}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 43
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P79" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{7D22A3F2-D4C9-7EBE-4C36-A5E564D099FA}">
+  <xltc:threadedComment ref="P79" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{43827401-9729-C2F4-B538-74E267729C46}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 44
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P80" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{6F104F1D-84C3-0FB9-8885-5F4D48531871}">
+  <xltc:threadedComment ref="P80" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{5E336747-0123-6D4A-458B-9EC79815C379}">
     <xltc:text>Source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf
 Page: 40
 Available: 2025-10-24
 SHA-256: 2a44e26a70a3c05c45814de4aba756ef39bfa15e05137f49edd3ec22b722260a</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P81" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{FCCBBFA1-24E0-2ECE-EB37-806DB36AC90C}">
+  <xltc:threadedComment ref="P81" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{E8A42772-0744-BB49-C6CD-22184FA6F8F7}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P82" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{AB7C2528-F367-AFFE-4205-1F9DD2C6F441}">
+  <xltc:threadedComment ref="P82" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{F8BABEF1-219F-5AA2-A49A-3A48153CD84C}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 15
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P83" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{1C4365EB-7A12-19EB-6F23-09BF7854F864}">
+  <xltc:threadedComment ref="P83" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{4C4BADA7-DC39-C76C-6638-783DFC1781C8}">
     <xltc:text>Source: https://www.aspenpharma.com/download/annual-financial-statements-2/
 Page: 16
 Available: 2025-10-02
 SHA-256: a091fee4d4b575781836440b929291617c128f8f857b2dd0a7e0dfb4c1bcc53d</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P84" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{3F03CB66-095C-3404-E5AE-B8B563887750}">
+  <xltc:threadedComment ref="P84" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{DF837794-31DD-20EF-599F-45523E2B054D}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P85" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{E6D42EC5-8BE4-DB23-356E-E8975A92AF6F}">
+  <xltc:threadedComment ref="P85" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{FCA8385D-924A-F8F3-4270-0FB7532DF3F7}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 22
 Available: 2026-02-25
 SHA-256: 71bcff13a20668eea8842f5ef28273ba787b0042b2fe7e1ea9faeb03b581ed53</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="P86" dT="2026-08-14T10:54:56.945" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{77C690BB-D307-3F3C-26FD-4F2712DC5136}">
+  <xltc:threadedComment ref="P86" dT="2026-08-14T11:00:52.352" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{6D538EC1-799B-2E21-B797-837119C99EEA}">
     <xltc:text>Source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf
 Page: 21
 Available: 2026-02-25
@@ -2742,64 +2742,64 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="J5" dT="2026-08-14T10:54:57.273" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{056BFFBA-1801-631C-3654-01E2B2FEFFA1}">
+  <xltc:threadedComment ref="J5" dT="2026-08-14T11:00:52.633" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{03358198-A18A-0637-AE13-2EBB49B74CCB}">
     <xltc:text>Official source: https://www.bhp.com/-/media/documents/investors/annual-reports/2025/250819_bhpannualreport2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J6" dT="2026-08-14T10:54:57.275" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{AEB35E22-B146-E986-D70B-680EB7EBA741}">
+  <xltc:threadedComment ref="J6" dT="2026-08-14T11:00:52.635" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{16E09466-770F-DC6D-B8AE-5F56C968BC0B}">
     <xltc:text>Official source: https://www.glencore.com/.rest/api/v1/documents/static/9b103e11-72e7-40bf-ae7c-eabe57361522/GLEN-2025-Annual-Report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J7" dT="2026-08-14T10:54:57.278" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{1A66EC80-39A8-BBFD-3F0B-A8FB8A71076C}">
+  <xltc:threadedComment ref="J7" dT="2026-08-14T11:00:52.637" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{5A87A16A-54A6-6A4A-A716-713CF075763C}">
     <xltc:text>Official source: https://www.angloamerican.com/~/media/Files/A/Anglo-American-Group-v9/PLC/investors/annual-reporting/2025/aa-annual-report-full-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J8" dT="2026-08-14T10:54:57.281" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{283BC70E-764F-9D7D-76D2-C1E754232E7C}">
+  <xltc:threadedComment ref="J8" dT="2026-08-14T11:00:52.64" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{51A5BCFB-330F-5404-5AB5-4D111557355C}">
     <xltc:text>Official source: https://reports.anglogoldashanti.com/25/download/AGA-AR25.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J9" dT="2026-08-14T10:54:57.284" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{2B4D5C58-7CC8-8965-AE53-FAF3E77DF125}">
+  <xltc:threadedComment ref="J9" dT="2026-08-14T11:00:52.642" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{31BFA9BA-FEBF-C930-7B72-05A92515189D}">
     <xltc:text>Official source: https://www.goldfields.com/pdf/investors/integrated-annual-reports/2025/afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J10" dT="2026-08-14T10:54:57.288" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{CE85C480-8E26-EFF5-D7AE-A1C07D9B98B6}">
+  <xltc:threadedComment ref="J10" dT="2026-08-14T11:00:52.643" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{6FFA8427-BE49-9BF8-DACD-0E54AF69D979}">
     <xltc:text>Official source: https://www.valterraplatinum.com/wp-content/uploads/2026/05/annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J11" dT="2026-08-14T10:54:57.291" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{41BEFA26-1CA3-717B-C25E-6FAF19367372}">
+  <xltc:threadedComment ref="J11" dT="2026-08-14T11:00:52.645" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{4D05509C-70F1-DB4D-9D32-2F454F56A4A8}">
     <xltc:text>Official source: https://group.outsurance.co.za/globalassets/documents/investor-relations/reports-and-results/2025/ogl-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J12" dT="2026-08-14T10:54:57.296" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{253A4618-3510-1622-74B0-CB88D82A95CF}">
+  <xltc:threadedComment ref="J12" dT="2026-08-14T11:00:52.647" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{1BCE242B-A16F-D35F-0139-0CACF590FBE4}">
     <xltc:text>Official source: https://www.sanlam.com/downloads/integrated-report-and-annual-financial-statements/2024/Sanlam-AFS-2024-spreads.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J13" dT="2026-08-14T10:54:57.298" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{FD8FC314-3FE9-7295-B95C-749D9AF03F40}">
+  <xltc:threadedComment ref="J13" dT="2026-08-14T11:00:52.649" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{788A8C39-4C7F-5DDF-B66C-0C91073C4346}">
     <xltc:text>Official source: https://www.shopriteholdings.co.za/docs/shp-afs-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J14" dT="2026-08-14T10:54:57.301" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{A542688D-10E7-AC16-BF62-7C9420A0CB6A}">
+  <xltc:threadedComment ref="J14" dT="2026-08-14T11:00:52.651" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{8FF0089B-7903-3B52-0C52-781D7BBE47A3}">
     <xltc:text>Official source: https://www.bidcorpgroup.com/pdf/reports/2025/Bidcorp-2025-AIR.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J15" dT="2026-08-14T10:54:57.305" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{DDCCE20C-D9C3-F33C-99F1-3542159C292B}">
+  <xltc:threadedComment ref="J15" dT="2026-08-14T11:00:52.654" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{ABFFBA4E-13E6-F46E-1003-C8FC3BFC4E41}">
     <xltc:text>Official source: https://pepkor.co.za/wp-content/uploads/Pepkor-annual-financial-statements-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J16" dT="2026-08-14T10:54:57.308" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{7A8C311B-1177-37FC-55E5-7BA1626253B4}">
+  <xltc:threadedComment ref="J16" dT="2026-08-14T11:00:52.656" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{DE42D7FF-E748-9CEF-9DA2-741C9C7F4306}">
     <xltc:text>Official source: https://clicksgroup.co.za/iar2025/wp-content/uploads/CGL-YE25-Annual-financial-statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J17" dT="2026-08-14T10:54:57.311" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{3A2B0191-F99E-961A-C5FA-AB373DECB115}">
+  <xltc:threadedComment ref="J17" dT="2026-08-14T11:00:52.659" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{11EEA32B-D415-FB31-AE8E-2F237C5305B9}">
     <xltc:text>Official source: https://nepirockcastle.com/wp-content/uploads/2026/03/NEPI_Rockcastle_Annual_Report_2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J18" dT="2026-08-14T10:54:57.314" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{94B90196-28B0-BBF4-EDB3-1D42F95D11F5}">
+  <xltc:threadedComment ref="J18" dT="2026-08-14T11:00:52.661" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{F3491057-0054-94D5-4F22-2DB6E419570E}">
     <xltc:text>Official source: https://www.prosus.com/~/media/Files/P/prosus-corp-v2/results-reports-and-events-archive/annual-report/2026/fy2026-annual-report.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J19" dT="2026-08-14T10:54:57.317" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{2C5D4759-15DC-9CF4-A10A-E4DD2B0C28D8}">
+  <xltc:threadedComment ref="J19" dT="2026-08-14T11:00:52.664" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{9CF4DCE5-1115-069E-5C9B-6BE71474B259}">
     <xltc:text>Official source: https://www.naspers.com/~/media/Files/N/Naspers-Corp-V2/results-reports-and-events-archive/latest-results/fy-2026/naspers-annual-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J20" dT="2026-08-14T10:54:57.319" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{D5163183-B337-0253-F177-61E462FF999F}">
+  <xltc:threadedComment ref="J20" dT="2026-08-14T11:00:52.666" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{D4B87D3D-C97C-5223-C7A2-F8BBDAD3F1A4}">
     <xltc:text>Official source: https://www.mtn.com/wp-content/uploads/2026/03/MTN-Group-FY-25-Annual-Financial-Statements.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J21" dT="2026-08-14T10:54:57.321" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{8DD6D4F6-BF6F-3D9B-E666-BF8235FA60E3}">
+  <xltc:threadedComment ref="J21" dT="2026-08-14T11:00:52.668" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{F5AF6B59-C1F3-82DA-AEBC-95BE9980CBFA}">
     <xltc:text>Official source: https://vodacom-reports.co.za/integrated-reports/ir-2026/documents/vodacom-consolidated-and-separate-financial-statements-2026.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J22" dT="2026-08-14T10:54:57.325" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{560957A6-2914-F33B-FDC5-B3985B6BD162}">
+  <xltc:threadedComment ref="J22" dT="2026-08-14T11:00:52.67" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{5CAEF3D3-B404-BE2E-09F3-6E792A945106}">
     <xltc:text>Official source: https://bidvest.co.za/pdf/annual-reports/2025/bidvest-iar-2025.pdf</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J23" dT="2026-08-14T10:54:57.328" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{7CE10764-0905-1DAA-5C75-9DF0DAAB717E}">
+  <xltc:threadedComment ref="J23" dT="2026-08-14T11:00:52.671" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{4A9BBAB3-4446-5BA9-62A0-A9F3F0ADDC81}">
     <xltc:text>Official source: https://www.aspenpharma.com/download/annual-financial-statements-2/</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J24" dT="2026-08-14T10:54:57.331" personId="{65ABB4F9-023C-4AE2-A790-71CAEBD0C99A}" id="{6F155B2F-3B59-BFE4-A5D9-BA0F24D73EBE}">
+  <xltc:threadedComment ref="J24" dT="2026-08-14T11:00:52.674" personId="{9DFC5A97-C476-4693-ACBE-129047B28BFB}" id="{E5CBD345-6B49-A62D-9E0C-20D78646AABD}">
     <xltc:text>Official source: https://senspdf.jse.co.za/documents/2026/JSE/isse/SHCE/FY25Result.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -7802,7 +7802,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb553a9dcf194a19"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf22efd13e553485a"/>
 </x:worksheet>
 </file>
 
@@ -8862,7 +8862,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="PENDING"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd16b3b571aec41fa"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5018c898539d4913"/>
 </x:worksheet>
 </file>
 
@@ -20015,6 +20015,6 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R899828e8cb314418"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc217fd8a488e46d4"/>
 </x:worksheet>
 </file>
</xml_diff>